<commit_message>
🤖 Daily run: 2026-09-24 16:42
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$56</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 22/09/2026 às 16:21</t>
+          <t>Gerado em 24/09/2026 às 16:34</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6">
@@ -638,27 +638,27 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>161372.4137931034</v>
+        <v>161778.5714285714</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1073,11 +1073,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146360</v>
+        <v>146374</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 04/2026 – Contrat. de consult. - Engenharia de Dados</t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1095,27 +1095,27 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46287</v>
+        <v>46295</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>130000</v>
+        <v>120000</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>estatisticastrabalho@trabalho.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1140,11 +1140,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146361</v>
+        <v>146375</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Consultoria Especializada - Qualidade de Dados I</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1162,27 +1162,27 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46287</v>
+        <v>46295</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>130000</v>
+        <v>120000</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>estatisticastrabalho@trabalho.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1207,11 +1207,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146362</v>
+        <v>146384</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 06/2026 - Consultoria Especializada - Qualidade de Dados II</t>
+          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1234,22 +1234,22 @@
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46287</v>
+        <v>46296</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>130000</v>
+        <v>120000</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>estatisticastrabalho@trabalho.gov.br</t>
+          <t>dirp@mdh.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1274,11 +1274,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146374</v>
+        <v>146385</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1301,22 +1301,22 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46280</v>
+        <v>46289</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46295</v>
+        <v>46311</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1341,11 +1341,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146375</v>
+        <v>146386</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1363,27 +1363,27 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46280</v>
+        <v>46282</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46295</v>
+        <v>46292</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>120000</v>
+        <v>92520</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>processoseletivo.sat@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
@@ -1408,11 +1408,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146384</v>
+        <v>146380</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
+          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1426,31 +1426,31 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46283</v>
+        <v>46287</v>
       </c>
       <c r="K10" s="14" t="n">
         <v>46296</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>120000</v>
+        <v>126500</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>dirp@mdh.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr">
@@ -1475,11 +1475,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146386</v>
+        <v>146381</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
+          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1493,31 +1493,31 @@
         </is>
       </c>
       <c r="F11" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
-          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46282</v>
+        <v>46287</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46292</v>
+        <v>46296</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>92520</v>
+        <v>126500</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>processoseletivo.sat@trabalho.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
@@ -1542,11 +1542,11 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146380</v>
+        <v>146383</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
+          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -1584,7 +1584,7 @@
         <v>46296</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>126500</v>
+        <v>86800</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1609,16 +1609,16 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146381</v>
+        <v>146357</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1676,16 +1676,16 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146383</v>
+        <v>146358</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
+          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1718,7 +1718,7 @@
         <v>46296</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>86800</v>
+        <v>126500</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
@@ -1743,11 +1743,11 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>146357</v>
+        <v>146390</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
+          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1761,31 +1761,31 @@
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="J15" s="22" t="n">
-        <v>46287</v>
+        <v>46282</v>
       </c>
       <c r="K15" s="22" t="n">
         <v>46296</v>
       </c>
       <c r="L15" s="23" t="n">
-        <v>126500</v>
+        <v>49580</v>
       </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="N15" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>selecaopnud0326@pge.ba.gov.br</t>
         </is>
       </c>
       <c r="O15" s="24" t="inlineStr">
@@ -1806,87 +1806,79 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="n">
-        <v>146358</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr"/>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L16" s="15" t="n">
-        <v>126500</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr"/>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>146390</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
@@ -1904,36 +1896,26 @@
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>Salvador/BA</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L17" s="23" t="n">
-        <v>49580</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr">
-        <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr"/>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -1945,12 +1927,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1966,7 +1948,7 @@
       <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1990,7 +1972,7 @@
       <c r="N18" s="12" t="inlineStr"/>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2002,12 +1984,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2017,15 +1999,13 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2049,7 +2029,7 @@
       <c r="N19" s="20" t="inlineStr"/>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2061,12 +2041,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2082,7 +2062,7 @@
       <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2106,7 +2086,7 @@
       <c r="N20" s="12" t="inlineStr"/>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2118,12 +2098,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2163,7 +2143,7 @@
       <c r="N21" s="20" t="inlineStr"/>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2175,12 +2155,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:6277cc83-3d55-4575-091b-08df172a76c5</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>14BRZ1163 - Publicação -  Edital 69/2026 - 01 Vaga consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2190,13 +2170,15 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2206,10 +2188,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46316</v>
+        <v>46294</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2220,7 +2202,7 @@
       <c r="N22" s="12" t="inlineStr"/>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2232,12 +2214,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:6c8e0acd-2d12-4dc7-e28e-08df14acbbca</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ1102- Edital nº 36/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2263,10 +2245,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46316</v>
+        <v>46293</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2277,7 +2259,7 @@
       <c r="N23" s="20" t="inlineStr"/>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2271,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:3622350f-775c-4cc9-9b64-08df0ff5ff21</t>
+          <t>unesco:5f5ec6eb-c0e8-4e67-e28f-08df14acbbca</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 914BRZ1166 - Edital nº 01.2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1102- Edital nº 37/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2320,10 +2302,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46283</v>
+        <v>46289</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46288</v>
+        <v>46293</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2334,7 +2316,7 @@
       <c r="N24" s="12" t="inlineStr"/>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2346,12 +2328,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
+          <t>unesco:dceb9c82-2a2c-4ba9-e290-08df14acbbca</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
+          <t>914BRZ1102- Edital nº 38/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2361,15 +2343,13 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2379,10 +2359,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2393,7 +2373,7 @@
       <c r="N25" s="20" t="inlineStr"/>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2405,28 +2385,30 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
+          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2436,10 +2418,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46292</v>
+        <v>46295</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2450,7 +2432,7 @@
       <c r="N26" s="12" t="inlineStr"/>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2462,17 +2444,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
+          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
+          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2485,7 +2467,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2495,10 +2477,10 @@
       </c>
       <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46287</v>
+        <v>46282</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46292</v>
+        <v>46289</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2509,7 +2491,7 @@
       <c r="N27" s="20" t="inlineStr"/>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2521,30 +2503,28 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
+          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2568,29 +2548,29 @@
       <c r="N28" s="12" t="inlineStr"/>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2599,67 +2579,57 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Saúde</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr">
-        <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46224</v>
+        <v>46287</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46233</v>
-      </c>
-      <c r="L29" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr"/>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2668,45 +2638,35 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr">
-        <is>
-          <t>Brasília DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46227</v>
+        <v>46285</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46231</v>
-      </c>
-      <c r="L30" s="15" t="n">
-        <v>150000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr"/>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2718,12 +2678,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2733,13 +2693,15 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2749,17 +2711,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46238</v>
+        <v>46233</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>30000</v>
+        <v>288000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2773,7 +2735,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2854,12 +2816,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2877,27 +2839,27 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>204000</v>
+        <v>288000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2911,7 +2873,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2923,12 +2885,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2946,27 +2908,27 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46237</v>
+        <v>46245</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>288000</v>
+        <v>80000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2980,7 +2942,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2992,12 +2954,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3015,7 +2977,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3049,7 +3011,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3061,12 +3023,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3084,7 +3046,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3104,7 +3066,7 @@
         <v>46245</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3118,7 +3080,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3130,12 +3092,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3145,15 +3107,13 @@
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F37" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F37" s="21" t="inlineStr"/>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3163,17 +3123,17 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>80000</v>
+        <v>30000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3187,7 +3147,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3199,12 +3159,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3222,7 +3182,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3232,7 +3192,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
@@ -3242,7 +3202,7 @@
         <v>46245</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3256,7 +3216,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3268,12 +3228,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3287,7 +3247,7 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
@@ -3301,19 +3261,21 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L39" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L39" s="23" t="n">
+        <v>100000</v>
+      </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3323,7 +3285,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3335,12 +3297,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3350,13 +3312,15 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3366,17 +3330,17 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46252</v>
+        <v>46257</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>286000</v>
+        <v>54000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3390,7 +3354,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3402,12 +3366,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3421,35 +3385,33 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
         <v>46246</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L41" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3459,7 +3421,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3540,30 +3502,28 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F43" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F43" s="21" t="inlineStr"/>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3573,17 +3533,17 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46251</v>
+        <v>46227</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46256</v>
+        <v>46252</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>50000</v>
+        <v>286000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3597,7 +3557,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3678,17 +3638,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3701,7 +3661,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3711,21 +3671,21 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46272</v>
+        <v>46256</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3735,7 +3695,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3816,22 +3776,22 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
@@ -3839,31 +3799,31 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46270</v>
+        <v>46272</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>30000</v>
+        <v>54000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3873,7 +3833,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3885,22 +3845,22 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
@@ -3908,27 +3868,27 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46288</v>
+        <v>46270</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3942,7 +3902,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3954,12 +3914,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3977,27 +3937,27 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46280</v>
+        <v>46288</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>50000</v>
+        <v>70000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4011,7 +3971,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -4023,12 +3983,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4042,11 +4002,11 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -4056,16 +4016,18 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
         <v>46275</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L50" s="15" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4078,7 +4040,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4090,17 +4052,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4113,41 +4075,41 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46244</v>
+        <v>46281</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46296</v>
+        <v>46286</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>935000</v>
+        <v>110000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -4159,17 +4121,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4178,45 +4140,43 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46244</v>
+        <v>46275</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L52" s="15" t="n">
-        <v>350000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L52" s="15" t="inlineStr"/>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4228,22 +4188,22 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
@@ -4251,27 +4211,27 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="K53" s="22" t="n">
         <v>46286</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>110000</v>
+        <v>30000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4285,7 +4245,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -4297,12 +4257,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4312,15 +4272,15 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4330,31 +4290,29 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46282</v>
+        <v>46278</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L54" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46289</v>
+      </c>
+      <c r="L54" s="15" t="inlineStr"/>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -4366,17 +4324,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4385,48 +4343,119 @@
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46278</v>
+        <v>46244</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46289</v>
-      </c>
-      <c r="L55" s="23" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L55" s="23" t="n">
+        <v>350000</v>
+      </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F56" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J56" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K56" s="14" t="n">
+        <v>46296</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>935000</v>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N56" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O56" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O55"/>
+  <autoFilter ref="A1:O56"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4482,6 +4511,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4520,27 +4550,27 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -4582,7 +4612,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -4592,7 +4622,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -4644,7 +4674,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -4654,7 +4684,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -4716,7 +4746,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -4726,7 +4756,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -4736,7 +4766,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -4746,7 +4776,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -4824,21 +4854,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -4848,7 +4878,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -4874,11 +4904,11 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -4894,11 +4924,11 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4946,7 +4976,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4961,7 +4991,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4976,7 +5006,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4991,7 +5021,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-25 16:43
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$59</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 24/09/2026 às 16:34</t>
+          <t>Gerado em 25/09/2026 às 16:37</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
@@ -644,21 +644,21 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1806,17 +1806,15 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>146394</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1826,54 +1824,64 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr"/>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J16" s="14" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L16" s="15" t="inlineStr"/>
+        <v>46304</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>90000</v>
+      </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>146396</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1891,31 +1899,41 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr"/>
+          <t>MTE</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Brasília, com disponibilidade para viagens</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="n">
-        <v>46286</v>
+        <v>46290</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L17" s="23" t="inlineStr"/>
+        <v>46303</v>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>208966.53</v>
+      </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>selecao.spt@trabalho.gov.br</t>
+        </is>
+      </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1927,12 +1945,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1948,7 +1966,7 @@
       <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1984,12 +2002,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1999,13 +2017,15 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2041,12 +2061,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2062,7 +2082,7 @@
       <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2098,12 +2118,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2155,12 +2175,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:6277cc83-3d55-4575-091b-08df172a76c5</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>14BRZ1163 - Publicação -  Edital 69/2026 - 01 Vaga consultor Individual</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2170,15 +2190,13 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2188,10 +2206,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46294</v>
+        <v>46316</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2214,12 +2232,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:6c8e0acd-2d12-4dc7-e28e-08df14acbbca</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 36/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2245,10 +2263,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46293</v>
+        <v>46316</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2271,12 +2289,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:5f5ec6eb-c0e8-4e67-e28f-08df14acbbca</t>
+          <t>unesco:5028b251-6c79-4f6d-f98d-08df189e5e5f</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 37/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1102- Edital nº 39/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2286,13 +2304,15 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2302,10 +2322,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2328,12 +2348,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:dceb9c82-2a2c-4ba9-e290-08df14acbbca</t>
+          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 38/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2343,13 +2363,15 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2359,10 +2381,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2385,12 +2407,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
+          <t>unesco:6277cc83-3d55-4575-091b-08df172a76c5</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
+          <t>14BRZ1163 - Publicação -  Edital 69/2026 - 01 Vaga consultor Individual</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2408,7 +2430,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2421,7 +2443,7 @@
         <v>46289</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46295</v>
+        <v>46294</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2444,12 +2466,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:34a61630-55f8-4262-9489-08df0f3a2d32</t>
+          <t>unesco:6c8e0acd-2d12-4dc7-e28e-08df14acbbca</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1156 - edital 08/2026 - Consultor Individual</t>
+          <t>914BRZ1102- Edital nº 36/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2459,15 +2481,13 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="inlineStr"/>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2477,10 +2497,10 @@
       </c>
       <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2503,17 +2523,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
+          <t>unesco:5f5ec6eb-c0e8-4e67-e28f-08df14acbbca</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1102- Edital nº 37/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2534,10 +2554,10 @@
       </c>
       <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
@@ -2560,30 +2580,28 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
+          <t>unesco:dceb9c82-2a2c-4ba9-e290-08df14acbbca</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
+          <t>914BRZ1102- Edital nº 38/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="inlineStr"/>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2593,10 +2611,10 @@
       </c>
       <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
@@ -2619,17 +2637,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
+          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2642,7 +2660,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2652,10 +2670,10 @@
       </c>
       <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46292</v>
+        <v>46295</v>
       </c>
       <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
@@ -2673,17 +2691,17 @@
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2693,71 +2711,59 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr"/>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr">
-        <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr"/>
       <c r="J31" s="22" t="n">
-        <v>46224</v>
+        <v>46285</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46233</v>
-      </c>
-      <c r="L31" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr"/>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2766,67 +2772,57 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.343</v>
+        <v>0.3</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Saúde</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr">
-        <is>
-          <t>Remoto, Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46232</v>
+        <v>46287</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L32" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr"/>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2835,45 +2831,35 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I33" s="19" t="inlineStr">
-        <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="22" t="n">
-        <v>46232</v>
+        <v>46285</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46237</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N33" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr"/>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2885,12 +2871,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2908,7 +2894,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2918,17 +2904,17 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46240</v>
+        <v>46224</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46245</v>
+        <v>46233</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2942,7 +2928,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2954,12 +2940,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -2969,15 +2955,13 @@
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="inlineStr"/>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -2987,17 +2971,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3011,7 +2995,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3023,17 +3007,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3042,11 +3026,11 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3056,17 +3040,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3080,7 +3064,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3092,12 +3076,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3107,13 +3091,15 @@
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F37" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F37" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3123,17 +3109,17 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3147,7 +3133,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3145,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3182,27 +3168,27 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3216,7 +3202,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3228,12 +3214,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3251,7 +3237,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3271,7 +3257,7 @@
         <v>46245</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>100000</v>
+        <v>204000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3285,7 +3271,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3297,12 +3283,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3320,27 +3306,27 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>54000</v>
+        <v>80000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3354,7 +3340,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3366,12 +3352,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3385,7 +3371,7 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
@@ -3399,19 +3385,21 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L41" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L41" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3421,7 +3409,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3433,12 +3421,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3456,27 +3444,27 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>54000</v>
+        <v>100000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3490,7 +3478,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3502,12 +3490,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3517,37 +3505,37 @@
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F43" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F43" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46252</v>
-      </c>
-      <c r="L43" s="23" t="n">
-        <v>286000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L43" s="23" t="inlineStr"/>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3557,7 +3545,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3569,12 +3557,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3584,15 +3572,13 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="inlineStr"/>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3602,17 +3588,17 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
+        <v>46227</v>
+      </c>
+      <c r="K44" s="14" t="n">
         <v>46252</v>
       </c>
-      <c r="K44" s="14" t="n">
-        <v>46259</v>
-      </c>
       <c r="L44" s="15" t="n">
-        <v>60000</v>
+        <v>286000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3626,7 +3612,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3638,17 +3624,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3661,7 +3647,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3671,17 +3657,17 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3695,7 +3681,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3707,17 +3693,17 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -3730,41 +3716,41 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46208</v>
+        <v>46246</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>500000</v>
+        <v>54000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3776,17 +3762,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3799,7 +3785,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3809,21 +3795,21 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46272</v>
+        <v>46256</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3833,7 +3819,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3845,22 +3831,22 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
@@ -3868,27 +3854,27 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46265</v>
+        <v>46252</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3902,7 +3888,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3900,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3937,7 +3923,7 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -3947,21 +3933,21 @@
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46266</v>
+        <v>46246</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46288</v>
+        <v>46272</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>70000</v>
+        <v>54000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
@@ -3971,7 +3957,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3983,17 +3969,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4006,41 +3992,41 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46275</v>
+        <v>46208</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46280</v>
+        <v>46259</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>50000</v>
+        <v>500000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4052,12 +4038,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4067,7 +4053,7 @@
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
@@ -4075,7 +4061,7 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -4085,17 +4071,17 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46281</v>
+        <v>46265</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46286</v>
+        <v>46270</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>110000</v>
+        <v>30000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4109,7 +4095,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -4121,12 +4107,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4140,30 +4126,32 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L52" s="15" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L52" s="15" t="n">
+        <v>70000</v>
+      </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4176,7 +4164,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -4188,12 +4176,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4203,7 +4191,7 @@
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
@@ -4211,27 +4199,27 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46282</v>
+        <v>46275</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4245,7 +4233,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4257,12 +4245,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4280,39 +4268,39 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46278</v>
+        <v>46275</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46289</v>
+        <v>46281</v>
       </c>
       <c r="L54" s="15" t="inlineStr"/>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4324,17 +4312,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4347,41 +4335,41 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46244</v>
+        <v>46281</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46300</v>
+        <v>46286</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>350000</v>
+        <v>110000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -4393,22 +4381,22 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
@@ -4416,46 +4404,251 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J56" s="14" t="n">
+        <v>46282</v>
+      </c>
+      <c r="K56" s="14" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N56" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O56" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F57" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G57" s="19" t="inlineStr">
+        <is>
           <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
-      <c r="H56" s="11" t="inlineStr">
+      <c r="H57" s="19" t="inlineStr">
         <is>
           <t>OEI/MDHC</t>
         </is>
       </c>
-      <c r="I56" s="11" t="inlineStr">
+      <c r="I57" s="19" t="inlineStr">
         <is>
           <t>Nacional</t>
         </is>
       </c>
-      <c r="J56" s="14" t="n">
+      <c r="J57" s="22" t="n">
         <v>46244</v>
       </c>
-      <c r="K56" s="14" t="n">
+      <c r="K57" s="22" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L57" s="23" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M57" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N57" s="20" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O57" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H58" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="J58" s="14" t="n">
+        <v>46278</v>
+      </c>
+      <c r="K58" s="14" t="n">
+        <v>46289</v>
+      </c>
+      <c r="L58" s="15" t="inlineStr"/>
+      <c r="M58" s="9" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N58" s="12" t="inlineStr">
+        <is>
+          <t>ugp@educacao.sp.gov.br</t>
+        </is>
+      </c>
+      <c r="O58" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F59" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J59" s="22" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K59" s="22" t="n">
         <v>46296</v>
       </c>
-      <c r="L56" s="15" t="n">
+      <c r="L59" s="23" t="n">
         <v>935000</v>
       </c>
-      <c r="M56" s="9" t="inlineStr">
+      <c r="M59" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
         </is>
       </c>
-      <c r="N56" s="12" t="inlineStr">
+      <c r="N59" s="20" t="inlineStr">
         <is>
           <t>compras.bra@oei.int</t>
         </is>
       </c>
-      <c r="O56" s="16" t="inlineStr">
+      <c r="O59" s="24" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O56"/>
+  <autoFilter ref="A1:O59"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4512,6 +4705,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4556,21 +4752,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -4612,7 +4808,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -4674,7 +4870,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
@@ -4746,7 +4942,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4756,7 +4952,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -4766,7 +4962,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -4858,7 +5054,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -4888,7 +5084,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -4928,7 +5124,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4976,7 +5172,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4991,7 +5187,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5006,7 +5202,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5021,7 +5217,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-26 15:54
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 25/09/2026 às 16:37</t>
+          <t>Gerado em 26/09/2026 às 15:51</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -638,27 +638,27 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,11 +876,11 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146369</v>
+        <v>146373</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
+          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -890,13 +890,15 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
@@ -910,13 +912,13 @@
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46290</v>
+        <v>46295</v>
       </c>
       <c r="L2" s="15" t="n">
-        <v>120000</v>
+        <v>108000</v>
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
@@ -941,11 +943,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146370</v>
+        <v>146374</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -955,13 +957,15 @@
       </c>
       <c r="E3" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F3" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G3" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H3" s="19" t="inlineStr">
@@ -971,17 +975,17 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46290</v>
+        <v>46295</v>
       </c>
       <c r="L3" s="23" t="n">
-        <v>126000</v>
+        <v>120000</v>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
@@ -1006,11 +1010,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146373</v>
+        <v>146375</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1038,7 +1042,7 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
@@ -1048,7 +1052,7 @@
         <v>46295</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>108000</v>
+        <v>120000</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1073,11 +1077,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146374</v>
+        <v>146384</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1095,24 +1099,24 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="L5" s="23" t="n">
         <v>120000</v>
@@ -1124,7 +1128,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>dirp@mdh.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1140,11 +1144,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146375</v>
+        <v>146385</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1167,22 +1171,22 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46280</v>
+        <v>46289</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46295</v>
+        <v>46311</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1191,7 +1195,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1207,11 +1211,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146384</v>
+        <v>146386</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
+          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1229,27 +1233,27 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46296</v>
+        <v>46292</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>120000</v>
+        <v>92520</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1258,7 +1262,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>dirp@mdh.gov.br</t>
+          <t>processoseletivo.sat@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1274,11 +1278,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146385</v>
+        <v>146380</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1292,31 +1296,31 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46289</v>
+        <v>46287</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46311</v>
+        <v>46296</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>100000</v>
+        <v>126500</v>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
@@ -1325,7 +1329,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1341,11 +1345,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146386</v>
+        <v>146381</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
+          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1359,31 +1363,31 @@
         </is>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46282</v>
+        <v>46287</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46292</v>
+        <v>46296</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>92520</v>
+        <v>126500</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1392,7 +1396,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>processoseletivo.sat@trabalho.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
@@ -1408,11 +1412,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146380</v>
+        <v>146383</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
+          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1430,7 +1434,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1450,7 +1454,7 @@
         <v>46296</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>126500</v>
+        <v>86800</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1475,16 +1479,16 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146381</v>
+        <v>146357</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
@@ -1497,7 +1501,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1542,16 +1546,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146383</v>
+        <v>146358</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
+          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1564,7 +1568,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -1584,7 +1588,7 @@
         <v>46296</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>86800</v>
+        <v>126500</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1609,11 +1613,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146357</v>
+        <v>146390</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
+          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1627,31 +1631,31 @@
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46287</v>
+        <v>46282</v>
       </c>
       <c r="K13" s="22" t="n">
         <v>46296</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>126500</v>
+        <v>49580</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1660,7 +1664,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>selecaopnud0326@pge.ba.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1676,16 +1680,16 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146358</v>
+        <v>146394</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
+          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -1694,16 +1698,16 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
@@ -1712,13 +1716,13 @@
         </is>
       </c>
       <c r="J14" s="14" t="n">
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46296</v>
+        <v>46304</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>126500</v>
+        <v>90000</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
@@ -1727,7 +1731,7 @@
       </c>
       <c r="N14" s="12" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O14" s="16" t="inlineStr">
@@ -1743,16 +1747,16 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>146390</v>
+        <v>146396</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
@@ -1765,27 +1769,27 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Brasília, com disponibilidade para viagens</t>
         </is>
       </c>
       <c r="J15" s="22" t="n">
-        <v>46282</v>
+        <v>46290</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46296</v>
+        <v>46303</v>
       </c>
       <c r="L15" s="23" t="n">
-        <v>49580</v>
+        <v>208966.53</v>
       </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
@@ -1794,7 +1798,7 @@
       </c>
       <c r="N15" s="20" t="inlineStr">
         <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
+          <t>selecao.spt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O15" s="24" t="inlineStr">
@@ -1806,15 +1810,17 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="n">
-        <v>146394</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1824,64 +1830,54 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr"/>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46304</v>
-      </c>
-      <c r="L16" s="15" t="n">
-        <v>90000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr"/>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>146396</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1899,41 +1895,31 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>Brasília, com disponibilidade para viagens</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46303</v>
-      </c>
-      <c r="L17" s="23" t="n">
-        <v>208966.53</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr">
-        <is>
-          <t>selecao.spt@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr"/>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -1945,12 +1931,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1966,7 +1952,7 @@
       <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -2002,12 +1988,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2017,15 +2003,13 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2061,12 +2045,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2082,7 +2066,7 @@
       <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2118,12 +2102,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2175,12 +2159,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:5028b251-6c79-4f6d-f98d-08df189e5e5f</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ1102- Edital nº 39/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2190,13 +2174,15 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2206,10 +2192,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46286</v>
+        <v>46290</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46316</v>
+        <v>46294</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2232,12 +2218,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2247,13 +2233,15 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2263,10 +2251,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46286</v>
+        <v>46290</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46316</v>
+        <v>46295</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2289,12 +2277,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:5028b251-6c79-4f6d-f98d-08df189e5e5f</t>
+          <t>unesco:4d25520a-6684-41e6-3080-08df1a5635e8</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 39/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 02/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2312,7 +2300,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2322,10 +2310,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2348,12 +2336,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
+          <t>unesco:c0a1d55e-84e2-4c98-3081-08df1a5635e8</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 03/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2363,15 +2351,13 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2381,7 +2367,7 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="K25" s="22" t="n">
         <v>46295</v>
@@ -2940,28 +2926,30 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="n">
+        <v>0.343</v>
+      </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -2995,7 +2983,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3007,30 +2995,28 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="n">
-        <v>0.343</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3064,7 +3050,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3076,12 +3062,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3099,27 +3085,27 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>204000</v>
+        <v>288000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3133,7 +3119,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3145,12 +3131,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3168,27 +3154,27 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46237</v>
+        <v>46245</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>288000</v>
+        <v>204000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3202,7 +3188,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3214,12 +3200,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3237,7 +3223,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3271,7 +3257,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3283,12 +3269,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3306,7 +3292,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3316,7 +3302,7 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
@@ -3340,7 +3326,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3352,12 +3338,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3375,7 +3361,7 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3385,7 +3371,7 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
@@ -3409,7 +3395,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3490,12 +3476,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3505,37 +3491,37 @@
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F43" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F43" s="21" t="inlineStr"/>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L43" s="23" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L43" s="23" t="n">
+        <v>286000</v>
+      </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3545,7 +3531,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3557,12 +3543,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3572,37 +3558,37 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46252</v>
-      </c>
-      <c r="L44" s="15" t="n">
-        <v>286000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L44" s="15" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3612,7 +3598,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3624,12 +3610,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3647,7 +3633,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3681,7 +3667,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3693,12 +3679,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3716,7 +3702,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3750,7 +3736,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3900,17 +3886,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3923,41 +3909,41 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46246</v>
+        <v>46208</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46272</v>
+        <v>46259</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>54000</v>
+        <v>500000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3969,17 +3955,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -3992,41 +3978,41 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46208</v>
+        <v>46246</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46259</v>
+        <v>46272</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>500000</v>
+        <v>54000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -4038,22 +4024,22 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
@@ -4061,27 +4047,27 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46270</v>
+        <v>46288</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4095,7 +4081,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -4107,22 +4093,22 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
@@ -4130,27 +4116,27 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46288</v>
+        <v>46270</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4164,7 +4150,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -4176,12 +4162,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4195,11 +4181,11 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -4209,18 +4195,16 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
         <v>46275</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L53" s="23" t="n">
-        <v>50000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L53" s="23" t="inlineStr"/>
       <c r="M53" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4233,7 +4217,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4245,12 +4229,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4264,11 +4248,11 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4278,16 +4262,18 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
         <v>46275</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L54" s="15" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L54" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4300,7 +4286,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4450,17 +4436,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4469,45 +4455,43 @@
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46244</v>
+        <v>46278</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L57" s="23" t="n">
-        <v>350000</v>
-      </c>
+        <v>46289</v>
+      </c>
+      <c r="L57" s="23" t="inlineStr"/>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -4519,17 +4503,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4538,43 +4522,45 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46278</v>
+        <v>46244</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46289</v>
-      </c>
-      <c r="L58" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L58" s="15" t="n">
+        <v>350000</v>
+      </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4586,69 +4572,136 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F59" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>Porto Alegre - RS</t>
+        </is>
+      </c>
+      <c r="J59" s="22" t="n">
+        <v>46290</v>
+      </c>
+      <c r="K59" s="22" t="n">
+        <v>46294</v>
+      </c>
+      <c r="L59" s="23" t="inlineStr"/>
+      <c r="M59" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N59" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O59" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
           <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
-      <c r="C59" s="19" t="inlineStr">
+      <c r="C60" s="11" t="inlineStr">
         <is>
           <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
-      <c r="D59" s="19" t="inlineStr">
+      <c r="D60" s="11" t="inlineStr">
         <is>
           <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
-      <c r="E59" s="20" t="inlineStr">
+      <c r="E60" s="12" t="inlineStr">
         <is>
           <t>Analista Powerbi</t>
         </is>
       </c>
-      <c r="F59" s="21" t="n">
+      <c r="F60" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="G59" s="19" t="inlineStr">
+      <c r="G60" s="11" t="inlineStr">
         <is>
           <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
-      <c r="H59" s="19" t="inlineStr">
+      <c r="H60" s="11" t="inlineStr">
         <is>
           <t>OEI/MDHC</t>
         </is>
       </c>
-      <c r="I59" s="19" t="inlineStr">
+      <c r="I60" s="11" t="inlineStr">
         <is>
           <t>Nacional</t>
         </is>
       </c>
-      <c r="J59" s="22" t="n">
+      <c r="J60" s="14" t="n">
         <v>46244</v>
       </c>
-      <c r="K59" s="22" t="n">
+      <c r="K60" s="14" t="n">
         <v>46296</v>
       </c>
-      <c r="L59" s="23" t="n">
+      <c r="L60" s="15" t="n">
         <v>935000</v>
       </c>
-      <c r="M59" s="17" t="inlineStr">
+      <c r="M60" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
         </is>
       </c>
-      <c r="N59" s="20" t="inlineStr">
+      <c r="N60" s="12" t="inlineStr">
         <is>
           <t>compras.bra@oei.int</t>
         </is>
       </c>
-      <c r="O59" s="24" t="inlineStr">
+      <c r="O60" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O59"/>
+  <autoFilter ref="A1:O60"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4708,6 +4761,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4746,27 +4800,27 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -4808,7 +4862,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -4818,7 +4872,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -4890,7 +4944,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -4942,7 +4996,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -4952,7 +5006,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -4962,7 +5016,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -4972,7 +5026,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -5012,7 +5066,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -5054,7 +5108,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -5064,7 +5118,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -5080,21 +5134,21 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -5172,7 +5226,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5187,7 +5241,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5202,7 +5256,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5217,7 +5271,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-27 16:30
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 26/09/2026 às 15:51</t>
+          <t>Gerado em 27/09/2026 às 16:28</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>161778.5714285714</v>
+        <v>157103.7037037037</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>100000</v>
+        <v>86800</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -2682,12 +2682,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2697,13 +2697,15 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2713,10 +2715,10 @@
       </c>
       <c r="I31" s="19" t="inlineStr"/>
       <c r="J31" s="22" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46292</v>
+        <v>46299</v>
       </c>
       <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
@@ -2739,30 +2741,28 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
+          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
+          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F32" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr"/>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46287</v>
+        <v>46285</v>
       </c>
       <c r="K32" s="14" t="n">
         <v>46292</v>
@@ -2798,12 +2798,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
+          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Saúde</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="22" t="n">
-        <v>46285</v>
+        <v>46287</v>
       </c>
       <c r="K33" s="22" t="n">
         <v>46292</v>
@@ -2852,22 +2852,22 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2876,45 +2876,35 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I34" s="11" t="inlineStr">
-        <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr"/>
       <c r="J34" s="14" t="n">
-        <v>46224</v>
+        <v>46285</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46233</v>
-      </c>
-      <c r="L34" s="15" t="n">
-        <v>288000</v>
-      </c>
+        <v>46292</v>
+      </c>
+      <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N34" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N34" s="12" t="inlineStr"/>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2995,12 +2985,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3010,13 +3000,15 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3026,17 +3018,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3050,7 +3042,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3123,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3146,15 +3138,13 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F38" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr"/>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3164,17 +3154,17 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3188,7 +3178,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3200,12 +3190,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3223,7 +3213,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3257,7 +3247,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3338,12 +3328,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3353,35 +3343,33 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F41" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="inlineStr"/>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>80000</v>
+        <v>286000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3395,7 +3383,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3407,12 +3395,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3426,7 +3414,7 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
@@ -3440,21 +3428,19 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>100000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3464,7 +3450,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3476,12 +3462,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3491,33 +3477,35 @@
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F43" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F43" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>286000</v>
+        <v>80000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3531,7 +3519,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3543,12 +3531,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3562,33 +3550,35 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
         <v>46246</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L44" s="15" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L44" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3598,7 +3588,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3610,12 +3600,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3633,27 +3623,27 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>54000</v>
+        <v>100000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3667,7 +3657,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3748,17 +3738,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3771,7 +3761,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3781,17 +3771,17 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3805,7 +3795,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3817,17 +3807,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3840,7 +3830,7 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3850,17 +3840,17 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3874,7 +3864,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3955,12 +3945,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -3974,35 +3964,33 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L50" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L50" s="15" t="inlineStr"/>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
@@ -4012,7 +4000,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4024,22 +4012,22 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
@@ -4047,27 +4035,27 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46288</v>
+        <v>46270</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4081,7 +4069,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -4093,22 +4081,22 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
@@ -4116,7 +4104,7 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
@@ -4126,17 +4114,17 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46265</v>
+        <v>46275</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46270</v>
+        <v>46280</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4150,7 +4138,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4162,12 +4150,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4181,30 +4169,32 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L53" s="23" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L53" s="23" t="n">
+        <v>70000</v>
+      </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4217,7 +4207,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -4229,12 +4219,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4252,31 +4242,31 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46275</v>
+        <v>46246</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46280</v>
+        <v>46272</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4286,7 +4276,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -4298,17 +4288,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4321,41 +4311,41 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46281</v>
+        <v>46244</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>110000</v>
+        <v>350000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4367,12 +4357,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4382,15 +4372,15 @@
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
@@ -4400,31 +4390,29 @@
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46282</v>
+        <v>46278</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L56" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46289</v>
+      </c>
+      <c r="L56" s="15" t="inlineStr"/>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -4436,17 +4424,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4455,43 +4443,45 @@
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46289</v>
-      </c>
-      <c r="L57" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L57" s="23" t="n">
+        <v>110000</v>
+      </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -4503,22 +4493,22 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
@@ -4526,41 +4516,41 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46244</v>
+        <v>46282</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46300</v>
+        <v>46286</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>350000</v>
+        <v>30000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4790,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -4810,7 +4800,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -5006,7 +4996,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -5016,7 +5006,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -5036,23 +5026,23 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Direito / Jurídico</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -5062,7 +5052,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Direito / Jurídico</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
@@ -5108,7 +5098,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
@@ -5118,7 +5108,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -5256,7 +5246,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-28 19:20
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 27/09/2026 às 16:28</t>
+          <t>Gerado em 28/09/2026 às 19:18</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -638,27 +638,27 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="18">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>157103.7037037037</v>
+        <v>140806.0606060606</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>86800</v>
+        <v>93500</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,11 +876,11 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146373</v>
+        <v>146370</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
+          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -890,15 +890,13 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr"/>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
@@ -908,17 +906,17 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46280</v>
+        <v>46276</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="L2" s="15" t="n">
-        <v>108000</v>
+        <v>126000</v>
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
@@ -943,11 +941,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146374</v>
+        <v>146373</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -985,7 +983,7 @@
         <v>46295</v>
       </c>
       <c r="L3" s="23" t="n">
-        <v>120000</v>
+        <v>108000</v>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
@@ -1010,11 +1008,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146375</v>
+        <v>146374</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1042,7 +1040,7 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
@@ -1077,11 +1075,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146384</v>
+        <v>146375</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1099,24 +1097,24 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="L5" s="23" t="n">
         <v>120000</v>
@@ -1128,7 +1126,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>dirp@mdh.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1144,11 +1142,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146385</v>
+        <v>146384</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1166,7 +1164,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1176,17 +1174,17 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46289</v>
+        <v>46283</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46311</v>
+        <v>46296</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1195,7 +1193,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>dirp@mdh.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1211,11 +1209,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146386</v>
+        <v>146385</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 08/2026 – Contratação de 6 (seis) consultorias especializadas (pessoa física) para revisão, consolidação, simplificação e otimização de atos normativos trabalhistas infralegais no Brasil</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1233,27 +1231,27 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46292</v>
+        <v>46311</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>92520</v>
+        <v>100000</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1262,7 +1260,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>processoseletivo.sat@trabalho.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1479,11 +1477,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146357</v>
+        <v>146354</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1501,7 +1499,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1515,13 +1513,13 @@
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>126500</v>
+        <v>93500</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1546,11 +1544,11 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146358</v>
+        <v>146357</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
+          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1613,11 +1611,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146390</v>
+        <v>146358</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1631,31 +1629,31 @@
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46282</v>
+        <v>46287</v>
       </c>
       <c r="K13" s="22" t="n">
         <v>46296</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>49580</v>
+        <v>126500</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1664,7 +1662,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1680,11 +1678,11 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146394</v>
+        <v>146382</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1698,16 +1696,16 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
@@ -1716,13 +1714,13 @@
         </is>
       </c>
       <c r="J14" s="14" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>90000</v>
+        <v>91500</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
@@ -1731,7 +1729,7 @@
       </c>
       <c r="N14" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O14" s="16" t="inlineStr">
@@ -1747,16 +1745,16 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>146396</v>
+        <v>146379</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
@@ -1765,7 +1763,7 @@
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
@@ -1774,22 +1772,22 @@
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
-          <t>Brasília, com disponibilidade para viagens</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J15" s="22" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46303</v>
+        <v>46307</v>
       </c>
       <c r="L15" s="23" t="n">
-        <v>208966.53</v>
+        <v>121500</v>
       </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
@@ -1798,7 +1796,7 @@
       </c>
       <c r="N15" s="20" t="inlineStr">
         <is>
-          <t>selecao.spt@trabalho.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O15" s="24" t="inlineStr">
@@ -1810,79 +1808,87 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>146378</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr"/>
+          <t>IBGE</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J16" s="14" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L16" s="15" t="inlineStr"/>
+        <v>46307</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>121500</v>
+      </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>projetos.especiais@ibge.gov.br</t>
+        </is>
+      </c>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>146377</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
@@ -1891,223 +1897,261 @@
         </is>
       </c>
       <c r="F17" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr"/>
+          <t>IBGE</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L17" s="23" t="inlineStr"/>
+        <v>46307</v>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>93500</v>
+      </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>projetos.especiais@ibge.gov.br</t>
+        </is>
+      </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>146355</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr"/>
+          <t>IBGE</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J18" s="14" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L18" s="15" t="inlineStr"/>
+        <v>46307</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <v>93500</v>
+      </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>projetos.especiais@ibge.gov.br</t>
+        </is>
+      </c>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n">
+        <v>146376</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr"/>
+          <t>IBGE</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J19" s="22" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L19" s="23" t="inlineStr"/>
+        <v>46307</v>
+      </c>
+      <c r="L19" s="23" t="n">
+        <v>86800</v>
+      </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr">
+        <is>
+          <t>projetos.especiais@ibge.gov.br</t>
+        </is>
+      </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>146390</v>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>Salvador/BA</t>
+        </is>
+      </c>
       <c r="J20" s="14" t="n">
-        <v>46286</v>
+        <v>46282</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L20" s="15" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <v>49580</v>
+      </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>selecaopnud0326@pge.ba.gov.br</t>
+        </is>
+      </c>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="n">
+        <v>146394</v>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2117,54 +2161,64 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="inlineStr"/>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J21" s="22" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L21" s="23" t="inlineStr"/>
+        <v>46304</v>
+      </c>
+      <c r="L21" s="23" t="n">
+        <v>90000</v>
+      </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N21" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N21" s="20" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>unesco:5028b251-6c79-4f6d-f98d-08df189e5e5f</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>146396</v>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 39/2026 - 01 vaga - Consultor Individual</t>
+          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2182,31 +2236,41 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr"/>
+          <t>MTE</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Brasília, com disponibilidade para viagens</t>
+        </is>
+      </c>
       <c r="J22" s="14" t="n">
         <v>46290</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L22" s="15" t="inlineStr"/>
+        <v>46303</v>
+      </c>
+      <c r="L22" s="15" t="n">
+        <v>208966.53</v>
+      </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr">
+        <is>
+          <t>selecao.spt@trabalho.gov.br</t>
+        </is>
+      </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -2218,12 +2282,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2233,15 +2297,13 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr"/>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2251,10 +2313,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46295</v>
+        <v>46316</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2277,12 +2339,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:4d25520a-6684-41e6-3080-08df1a5635e8</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 02/2026 - 01 vaga - Consultor Individual</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2300,7 +2362,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2310,10 +2372,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46291</v>
+        <v>46286</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46295</v>
+        <v>46316</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2336,12 +2398,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:c0a1d55e-84e2-4c98-3081-08df1a5635e8</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 03/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2357,7 +2419,7 @@
       <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2367,10 +2429,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46291</v>
+        <v>46286</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46295</v>
+        <v>46316</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2393,12 +2455,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:6277cc83-3d55-4575-091b-08df172a76c5</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>14BRZ1163 - Publicação -  Edital 69/2026 - 01 Vaga consultor Individual</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2408,15 +2470,13 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr"/>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2426,10 +2486,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46294</v>
+        <v>46316</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2452,12 +2512,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:6c8e0acd-2d12-4dc7-e28e-08df14acbbca</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 36/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2483,10 +2543,10 @@
       </c>
       <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46293</v>
+        <v>46316</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2509,12 +2569,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:5f5ec6eb-c0e8-4e67-e28f-08df14acbbca</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 37/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2540,10 +2600,10 @@
       </c>
       <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46293</v>
+        <v>46316</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
@@ -2566,12 +2626,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:dceb9c82-2a2c-4ba9-e290-08df14acbbca</t>
+          <t>unesco:5028b251-6c79-4f6d-f98d-08df189e5e5f</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 38/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1102- Edital nº 39/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2581,13 +2641,15 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2597,10 +2659,10 @@
       </c>
       <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
@@ -2623,12 +2685,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
+          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2646,7 +2708,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2656,7 +2718,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="K30" s="14" t="n">
         <v>46295</v>
@@ -2682,17 +2744,17 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>unesco:4d25520a-6684-41e6-3080-08df1a5635e8</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>914BRZ1161.2 - Edital nº 02/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2705,7 +2767,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2715,10 +2777,10 @@
       </c>
       <c r="I31" s="19" t="inlineStr"/>
       <c r="J31" s="22" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46299</v>
+        <v>46295</v>
       </c>
       <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
@@ -2741,17 +2803,17 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>unesco:a4685014-44a0-4ec8-9b63-08df0ff5ff21</t>
+          <t>unesco:c0a1d55e-84e2-4c98-3081-08df1a5635e8</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 11/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1161.2 - Edital nº 03/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2772,10 +2834,10 @@
       </c>
       <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46285</v>
+        <v>46291</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46292</v>
+        <v>46295</v>
       </c>
       <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
@@ -2798,17 +2860,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>unesco:49fa6512-497b-43c7-9b65-08df0ff5ff21</t>
+          <t>unesco:6277cc83-3d55-4575-091b-08df172a76c5</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 04/2026 - 4 vagas - Consultores Individuais</t>
+          <t>14BRZ1163 - Publicação -  Edital 69/2026 - 01 Vaga consultor Individual</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2821,7 +2883,7 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2831,10 +2893,10 @@
       </c>
       <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="22" t="n">
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46292</v>
+        <v>46294</v>
       </c>
       <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
@@ -2857,30 +2919,28 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>unesco:f0e2f0e3-b50c-4695-6d11-08df126138f3</t>
+          <t>unesco:6c8e0acd-2d12-4dc7-e28e-08df14acbbca</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1102- Edital nº 36/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F34" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr"/>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2890,10 +2950,10 @@
       </c>
       <c r="I34" s="11" t="inlineStr"/>
       <c r="J34" s="14" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
@@ -2911,17 +2971,17 @@
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>unesco:5f5ec6eb-c0e8-4e67-e28f-08df14acbbca</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>914BRZ1102- Edital nº 37/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -2931,140 +2991,116 @@
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="n">
-        <v>0.343</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="inlineStr"/>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I35" s="19" t="inlineStr">
-        <is>
-          <t>Remoto, Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I35" s="19" t="inlineStr"/>
       <c r="J35" s="22" t="n">
-        <v>46232</v>
+        <v>46289</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L35" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46293</v>
+      </c>
+      <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N35" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N35" s="20" t="inlineStr"/>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>unesco:dceb9c82-2a2c-4ba9-e290-08df14acbbca</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>914BRZ1102- Edital nº 38/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I36" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr"/>
       <c r="J36" s="14" t="n">
-        <v>46240</v>
+        <v>46289</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L36" s="15" t="n">
-        <v>204000</v>
-      </c>
+        <v>46293</v>
+      </c>
+      <c r="L36" s="15" t="inlineStr"/>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N36" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N36" s="12" t="inlineStr"/>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3073,62 +3109,52 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I37" s="19" t="inlineStr">
-        <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I37" s="19" t="inlineStr"/>
       <c r="J37" s="22" t="n">
-        <v>46232</v>
+        <v>46289</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46237</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N37" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N37" s="20" t="inlineStr"/>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3138,47 +3164,39 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F38" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I38" s="11" t="inlineStr">
-        <is>
-          <t>Remoto, Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr"/>
       <c r="J38" s="14" t="n">
-        <v>46232</v>
+        <v>46292</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L38" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46299</v>
+      </c>
+      <c r="L38" s="15" t="inlineStr"/>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N38" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N38" s="12" t="inlineStr"/>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -3190,12 +3208,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3213,7 +3231,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3233,7 +3251,7 @@
         <v>46245</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>204000</v>
+        <v>100000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3247,7 +3265,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3259,12 +3277,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3282,7 +3300,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3302,7 +3320,7 @@
         <v>46245</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3316,7 +3334,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3328,12 +3346,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3343,33 +3361,35 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F41" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>286000</v>
+        <v>204000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3383,7 +3403,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3395,12 +3415,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3410,37 +3430,37 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="inlineStr"/>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L42" s="15" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <v>286000</v>
+      </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3450,7 +3470,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3531,12 +3551,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3554,27 +3574,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>54000</v>
+        <v>80000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3588,7 +3608,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3600,12 +3620,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3619,7 +3639,7 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
@@ -3633,21 +3653,19 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L45" s="23" t="n">
-        <v>100000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L45" s="23" t="inlineStr"/>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3657,7 +3675,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3738,12 +3756,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3761,7 +3779,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3771,17 +3789,17 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3795,7 +3813,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3876,17 +3894,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3904,36 +3922,36 @@
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46208</v>
+        <v>46252</v>
       </c>
       <c r="K49" s="22" t="n">
         <v>46259</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>500000</v>
+        <v>60000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3945,12 +3963,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -3964,33 +3982,35 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46275</v>
+        <v>46246</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L50" s="15" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
@@ -4000,7 +4020,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -4081,17 +4101,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4104,41 +4124,41 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46275</v>
+        <v>46208</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46280</v>
+        <v>46259</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>50000</v>
+        <v>500000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4219,12 +4239,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4242,31 +4262,31 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46272</v>
+        <v>46280</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4276,7 +4296,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4288,17 +4308,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4311,41 +4331,41 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46244</v>
+        <v>46281</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46300</v>
+        <v>46286</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>350000</v>
+        <v>110000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -4357,12 +4377,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4380,39 +4400,39 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46278</v>
+        <v>46275</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46289</v>
+        <v>46281</v>
       </c>
       <c r="L56" s="15" t="inlineStr"/>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4424,17 +4444,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4447,41 +4467,41 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46281</v>
+        <v>46244</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46286</v>
+        <v>46296</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>110000</v>
+        <v>935000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4629,69 +4649,274 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="J60" s="14" t="n">
+        <v>46278</v>
+      </c>
+      <c r="K60" s="14" t="n">
+        <v>46295</v>
+      </c>
+      <c r="L60" s="15" t="inlineStr"/>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N60" s="12" t="inlineStr">
+        <is>
+          <t>ugp@educacao.sp.gov.br</t>
+        </is>
+      </c>
+      <c r="O60" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F61" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+        </is>
+      </c>
+      <c r="J61" s="22" t="n">
+        <v>46293</v>
+      </c>
+      <c r="K61" s="22" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L61" s="23" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M61" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N61" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O61" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
+        </is>
+      </c>
+      <c r="J62" s="14" t="n">
+        <v>46293</v>
+      </c>
+      <c r="K62" s="14" t="n">
+        <v>46298</v>
+      </c>
+      <c r="L62" s="15" t="n">
+        <v>21000</v>
+      </c>
+      <c r="M62" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N62" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O62" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
           <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
-      <c r="E60" s="12" t="inlineStr">
+      <c r="E63" s="20" t="inlineStr">
         <is>
           <t>Analista Powerbi</t>
         </is>
       </c>
-      <c r="F60" s="13" t="n">
+      <c r="F63" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="G60" s="11" t="inlineStr">
+      <c r="G63" s="19" t="inlineStr">
         <is>
           <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
-      <c r="H60" s="11" t="inlineStr">
+      <c r="H63" s="19" t="inlineStr">
         <is>
           <t>OEI/MDHC</t>
         </is>
       </c>
-      <c r="I60" s="11" t="inlineStr">
+      <c r="I63" s="19" t="inlineStr">
         <is>
           <t>Nacional</t>
         </is>
       </c>
-      <c r="J60" s="14" t="n">
+      <c r="J63" s="22" t="n">
         <v>46244</v>
       </c>
-      <c r="K60" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L60" s="15" t="n">
-        <v>935000</v>
-      </c>
-      <c r="M60" s="9" t="inlineStr">
+      <c r="K63" s="22" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L63" s="23" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M63" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
         </is>
       </c>
-      <c r="N60" s="12" t="inlineStr">
+      <c r="N63" s="20" t="inlineStr">
         <is>
           <t>compras.bra@oei.int</t>
         </is>
       </c>
-      <c r="O60" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+      <c r="O63" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O60"/>
+  <autoFilter ref="A1:O63"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4752,6 +4977,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4790,27 +5018,27 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -4852,7 +5080,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -4862,7 +5090,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -4872,7 +5100,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4924,7 +5152,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -4934,7 +5162,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -4986,7 +5214,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3">
@@ -4996,7 +5224,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -5006,7 +5234,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -5016,7 +5244,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -5026,13 +5254,13 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -5046,17 +5274,17 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5098,37 +5326,37 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -5138,7 +5366,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -5168,7 +5396,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5216,7 +5444,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5231,7 +5459,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5246,7 +5474,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5261,7 +5489,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-29 17:45
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 28/09/2026 às 19:18</t>
+          <t>Gerado em 29/09/2026 às 17:42</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>140806.0606060606</v>
+        <v>137241.1428571429</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1047,7 +1047,7 @@
         <v>46280</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="L4" s="15" t="n">
         <v>120000</v>
@@ -1114,7 +1114,7 @@
         <v>46280</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="L5" s="23" t="n">
         <v>120000</v>
@@ -2919,12 +2919,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>unesco:6c8e0acd-2d12-4dc7-e28e-08df14acbbca</t>
+          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 36/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2934,13 +2934,15 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F34" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2953,7 +2955,7 @@
         <v>46289</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
@@ -2976,28 +2978,30 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>unesco:5f5ec6eb-c0e8-4e67-e28f-08df14acbbca</t>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 37/2026 - 01 vaga - Consultor Individual</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3007,10 +3011,10 @@
       </c>
       <c r="I35" s="19" t="inlineStr"/>
       <c r="J35" s="22" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46293</v>
+        <v>46299</v>
       </c>
       <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
@@ -3028,79 +3032,91 @@
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>unesco:dceb9c82-2a2c-4ba9-e290-08df14acbbca</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 38/2026 - 01 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I36" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J36" s="14" t="n">
-        <v>46289</v>
+        <v>46240</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46293</v>
-      </c>
-      <c r="L36" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>204000</v>
+      </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N36" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N36" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3109,52 +3125,62 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I37" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I37" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J37" s="22" t="n">
-        <v>46289</v>
+        <v>46240</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>204000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N37" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N37" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3168,35 +3194,45 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I38" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J38" s="14" t="n">
-        <v>46292</v>
+        <v>46240</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46299</v>
-      </c>
-      <c r="L38" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>100000</v>
+      </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N38" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N38" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3208,12 +3244,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3231,7 +3267,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3241,7 +3277,7 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
@@ -3251,7 +3287,7 @@
         <v>46245</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3265,7 +3301,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3277,12 +3313,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3300,7 +3336,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3320,7 +3356,7 @@
         <v>46245</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>204000</v>
+        <v>80000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3334,7 +3370,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3346,12 +3382,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3361,35 +3397,33 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F41" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="inlineStr"/>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>204000</v>
+        <v>286000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3403,7 +3437,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3415,12 +3449,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3430,13 +3464,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3446,17 +3482,17 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46227</v>
+        <v>46252</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>286000</v>
+        <v>60000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3470,7 +3506,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3482,12 +3518,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3505,27 +3541,27 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3539,7 +3575,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3551,17 +3587,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3574,27 +3610,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>80000</v>
+        <v>50000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3608,7 +3644,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3687,12 +3723,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3710,7 +3746,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3744,7 +3780,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3756,12 +3792,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3779,7 +3815,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3796,14 +3832,14 @@
         <v>46246</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46257</v>
+        <v>46272</v>
       </c>
       <c r="L47" s="23" t="n">
         <v>54000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3813,7 +3849,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3825,22 +3861,22 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
@@ -3848,27 +3884,27 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46251</v>
+        <v>46265</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46256</v>
+        <v>46270</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3882,7 +3918,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3894,17 +3930,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3922,36 +3958,36 @@
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46252</v>
+        <v>46208</v>
       </c>
       <c r="K49" s="22" t="n">
         <v>46259</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>60000</v>
+        <v>500000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3963,12 +3999,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -3986,7 +4022,7 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -3996,21 +4032,21 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46246</v>
+        <v>46266</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46272</v>
+        <v>46288</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>54000</v>
+        <v>70000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
@@ -4020,7 +4056,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -4032,17 +4068,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4055,12 +4091,12 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
@@ -4069,10 +4105,10 @@
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46265</v>
+        <v>46282</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46270</v>
+        <v>46286</v>
       </c>
       <c r="L51" s="23" t="n">
         <v>30000</v>
@@ -4089,7 +4125,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -4101,12 +4137,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4124,7 +4160,7 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
@@ -4138,17 +4174,17 @@
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46208</v>
+        <v>46244</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46259</v>
+        <v>46296</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>500000</v>
+        <v>935000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
@@ -4158,7 +4194,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4170,17 +4206,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4193,27 +4229,27 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>70000</v>
+        <v>110000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4227,7 +4263,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -4308,17 +4344,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4327,11 +4363,11 @@
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -4341,18 +4377,16 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K55" s="22" t="n">
         <v>46281</v>
       </c>
-      <c r="K55" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L55" s="23" t="n">
-        <v>110000</v>
-      </c>
+      <c r="L55" s="23" t="inlineStr"/>
       <c r="M55" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4365,7 +4399,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4377,17 +4411,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4400,7 +4434,7 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
@@ -4414,10 +4448,10 @@
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46275</v>
+        <v>46290</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46281</v>
+        <v>46294</v>
       </c>
       <c r="L56" s="15" t="inlineStr"/>
       <c r="M56" s="9" t="inlineStr">
@@ -4432,7 +4466,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -4444,22 +4478,22 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
@@ -4467,41 +4501,41 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46244</v>
+        <v>46293</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>935000</v>
+        <v>30000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -4513,12 +4547,12 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -4528,7 +4562,7 @@
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
@@ -4536,31 +4570,31 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46282</v>
+        <v>46294</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46286</v>
+        <v>46297</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>30000</v>
+        <v>600000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
@@ -4570,7 +4604,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -4582,17 +4616,17 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
@@ -4601,43 +4635,45 @@
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46290</v>
+        <v>46244</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L59" s="23" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L59" s="23" t="n">
+        <v>350000</v>
+      </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4716,12 +4752,12 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
@@ -4735,11 +4771,11 @@
         </is>
       </c>
       <c r="F61" s="21" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
@@ -4749,7 +4785,7 @@
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J61" s="22" t="n">
@@ -4759,11 +4795,11 @@
         <v>46298</v>
       </c>
       <c r="L61" s="23" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N61" s="20" t="inlineStr">
@@ -4773,7 +4809,7 @@
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -4785,12 +4821,12 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
@@ -4800,15 +4836,15 @@
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.335</v>
+        <v>0.4</v>
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
@@ -4818,21 +4854,21 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J62" s="14" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K62" s="14" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="L62" s="15" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N62" s="12" t="inlineStr">
@@ -4842,81 +4878,12 @@
       </c>
       <c r="O62" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C63" s="19" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E63" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F63" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G63" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H63" s="19" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I63" s="19" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J63" s="22" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K63" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L63" s="23" t="n">
-        <v>350000</v>
-      </c>
-      <c r="M63" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N63" s="20" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O63" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O63"/>
+  <autoFilter ref="A1:O62"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4979,7 +4946,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5018,7 +4984,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -5038,7 +5004,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -5080,7 +5046,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3">
@@ -5090,7 +5056,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -5142,7 +5108,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -5152,7 +5118,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -5214,7 +5180,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -5224,7 +5190,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
@@ -5240,7 +5206,7 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
@@ -5250,11 +5216,11 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -5326,7 +5292,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -5346,7 +5312,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -5356,7 +5322,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -5444,7 +5410,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5459,7 +5425,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5474,7 +5440,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5489,7 +5455,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-30 17:42
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$61</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 29/09/2026 às 17:42</t>
+          <t>Gerado em 30/09/2026 às 17:39</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>137241.1428571429</v>
+        <v>134956.6666666667</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2626,12 +2626,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:5028b251-6c79-4f6d-f98d-08df189e5e5f</t>
+          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1102- Edital nº 39/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2662,7 +2662,7 @@
         <v>46290</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
@@ -2685,12 +2685,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
+          <t>unesco:4d25520a-6684-41e6-3080-08df1a5635e8</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 02/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="K30" s="14" t="n">
         <v>46295</v>
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:4d25520a-6684-41e6-3080-08df1a5635e8</t>
+          <t>unesco:c0a1d55e-84e2-4c98-3081-08df1a5635e8</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 02/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1161.2 - Edital nº 03/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2759,15 +2759,13 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr"/>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2803,12 +2801,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>unesco:c0a1d55e-84e2-4c98-3081-08df1a5635e8</t>
+          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 03/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2818,13 +2816,15 @@
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F32" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="K32" s="14" t="n">
         <v>46295</v>
@@ -2860,17 +2860,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>unesco:6277cc83-3d55-4575-091b-08df172a76c5</t>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>14BRZ1163 - Publicação -  Edital 69/2026 - 01 Vaga consultor Individual</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2893,10 +2893,10 @@
       </c>
       <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="22" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46294</v>
+        <v>46299</v>
       </c>
       <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
@@ -2914,22 +2914,22 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2938,52 +2938,62 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I34" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J34" s="14" t="n">
-        <v>46289</v>
+        <v>46240</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L34" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>80000</v>
+      </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N34" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N34" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -2997,35 +3007,45 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I35" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I35" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J35" s="22" t="n">
-        <v>46292</v>
+        <v>46240</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46299</v>
-      </c>
-      <c r="L35" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L35" s="23" t="n">
+        <v>100000</v>
+      </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N35" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N35" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3037,12 +3057,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3060,7 +3080,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3094,7 +3114,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3106,12 +3126,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3129,7 +3149,7 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3163,7 +3183,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3175,12 +3195,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3198,7 +3218,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3208,7 +3228,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
@@ -3218,7 +3238,7 @@
         <v>46245</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3232,7 +3252,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3244,12 +3264,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3259,35 +3279,33 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F39" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F39" s="21" t="inlineStr"/>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>80000</v>
+        <v>286000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3301,7 +3319,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3313,17 +3331,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3336,27 +3354,27 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>80000</v>
+        <v>50000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3370,7 +3388,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3382,12 +3400,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3397,13 +3415,15 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F41" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3413,17 +3433,17 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46252</v>
+        <v>46257</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>286000</v>
+        <v>54000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3437,7 +3457,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3449,12 +3469,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3472,7 +3492,7 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3482,17 +3502,17 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3506,7 +3526,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3518,12 +3538,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3541,7 +3561,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3551,17 +3571,17 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3575,7 +3595,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3587,17 +3607,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3606,35 +3626,33 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L44" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L44" s="15" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3644,7 +3662,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3656,17 +3674,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3675,43 +3693,45 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46246</v>
+        <v>46208</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L45" s="23" t="inlineStr"/>
+        <v>46259</v>
+      </c>
+      <c r="L45" s="23" t="n">
+        <v>500000</v>
+      </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3723,12 +3743,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3746,7 +3766,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3763,14 +3783,14 @@
         <v>46246</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46257</v>
+        <v>46272</v>
       </c>
       <c r="L46" s="15" t="n">
         <v>54000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -3780,7 +3800,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3792,22 +3812,22 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
@@ -3815,31 +3835,31 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3849,7 +3869,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3861,22 +3881,22 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
@@ -3884,27 +3904,27 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46270</v>
+        <v>46288</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3918,7 +3938,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3930,17 +3950,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3953,41 +3973,41 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46208</v>
+        <v>46281</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46259</v>
+        <v>46286</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>500000</v>
+        <v>110000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3999,12 +4019,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4018,32 +4038,30 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46266</v>
+        <v>46275</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46288</v>
-      </c>
-      <c r="L50" s="15" t="n">
-        <v>70000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L50" s="15" t="inlineStr"/>
       <c r="M50" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4056,7 +4074,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4068,12 +4086,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4083,7 +4101,7 @@
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
@@ -4091,27 +4109,27 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46282</v>
+        <v>46275</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4125,7 +4143,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -4137,17 +4155,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4156,45 +4174,43 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46244</v>
+        <v>46290</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L52" s="15" t="n">
-        <v>935000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L52" s="15" t="inlineStr"/>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -4206,22 +4222,22 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
@@ -4229,27 +4245,27 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="K53" s="22" t="n">
         <v>46286</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>110000</v>
+        <v>30000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4263,7 +4279,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -4275,17 +4291,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4298,41 +4314,41 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46275</v>
+        <v>46244</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46280</v>
+        <v>46296</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>50000</v>
+        <v>935000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4344,12 +4360,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4359,37 +4375,39 @@
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.3</v>
+        <v>0.335</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46275</v>
+        <v>46293</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L55" s="23" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L55" s="23" t="n">
+        <v>21000</v>
+      </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
@@ -4399,7 +4417,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -4411,17 +4429,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4430,43 +4448,45 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46290</v>
+        <v>46244</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L56" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>350000</v>
+      </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4478,12 +4498,12 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -4493,15 +4513,15 @@
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
@@ -4511,31 +4531,29 @@
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46293</v>
+        <v>46278</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L57" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L57" s="23" t="inlineStr"/>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -4547,12 +4565,12 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -4562,7 +4580,7 @@
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
@@ -4570,31 +4588,31 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>600000</v>
+        <v>30000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
@@ -4604,7 +4622,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -4616,17 +4634,17 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
@@ -4639,41 +4657,41 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46244</v>
+        <v>46294</v>
       </c>
       <c r="K59" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>350000</v>
+        <v>55000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -4685,12 +4703,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -4704,43 +4722,45 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46278</v>
+        <v>46294</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L60" s="15" t="inlineStr"/>
+        <v>46297</v>
+      </c>
+      <c r="L60" s="15" t="n">
+        <v>600000</v>
+      </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -4752,12 +4772,12 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
@@ -4767,15 +4787,15 @@
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F61" s="21" t="n">
-        <v>0.335</v>
+        <v>0.4</v>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
@@ -4785,21 +4805,21 @@
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J61" s="22" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K61" s="22" t="n">
-        <v>46298</v>
+        <v>46302</v>
       </c>
       <c r="L61" s="23" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N61" s="20" t="inlineStr">
@@ -4809,81 +4829,12 @@
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F62" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J62" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="K62" s="14" t="n">
-        <v>46305</v>
-      </c>
-      <c r="L62" s="15" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M62" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N62" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O62" s="16" t="inlineStr">
-        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O62"/>
+  <autoFilter ref="A1:O61"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4945,7 +4896,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4984,7 +4934,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -5004,7 +4954,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -5046,7 +4996,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
@@ -5108,7 +5058,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -5118,7 +5068,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -5180,7 +5130,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -5200,7 +5150,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -5288,7 +5238,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5318,11 +5268,11 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -5410,7 +5360,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5425,7 +5375,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5440,7 +5390,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5455,7 +5405,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-01 18:12
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 30/09/2026 às 17:39</t>
+          <t>Gerado em 01/10/2026 às 18:09</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>134956.6666666667</v>
+        <v>123620.4878048781</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>93500</v>
+        <v>86800</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -941,11 +941,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146373</v>
+        <v>146374</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 26/2026 – Contratação de Consultoria Individual para aprimoramento de soluções analíticas e computacionais aplicadas ao Modelo de Mensuração de Custos da Digitalização de Serviços Públicos </t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -980,10 +980,10 @@
         <v>46280</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="L3" s="23" t="n">
-        <v>108000</v>
+        <v>120000</v>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
@@ -1008,11 +1008,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146374</v>
+        <v>146375</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
@@ -1075,11 +1075,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146375</v>
+        <v>146384</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1097,24 +1097,24 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46310</v>
+        <v>46296</v>
       </c>
       <c r="L5" s="23" t="n">
         <v>120000</v>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>dirp@mdh.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1142,11 +1142,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146384</v>
+        <v>146385</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1174,17 +1174,17 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46283</v>
+        <v>46289</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46296</v>
+        <v>46311</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>dirp@mdh.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1209,11 +1209,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146385</v>
+        <v>146380</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1227,31 +1227,31 @@
         </is>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46289</v>
+        <v>46287</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46311</v>
+        <v>46296</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>100000</v>
+        <v>126500</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1276,11 +1276,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146380</v>
+        <v>146381</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
+          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1343,11 +1343,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146381</v>
+        <v>146383</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1385,7 +1385,7 @@
         <v>46296</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>126500</v>
+        <v>86800</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1410,16 +1410,16 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146383</v>
+        <v>146354</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1446,13 +1446,13 @@
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>86800</v>
+        <v>93500</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1477,11 +1477,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146354</v>
+        <v>146357</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1513,13 +1513,13 @@
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46293</v>
+        <v>46287</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46307</v>
+        <v>46296</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>93500</v>
+        <v>126500</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1544,11 +1544,11 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146357</v>
+        <v>146358</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
+          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1611,16 +1611,16 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146358</v>
+        <v>146382</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1647,13 +1647,13 @@
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>126500</v>
+        <v>91500</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1678,16 +1678,16 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146382</v>
+        <v>146379</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1720,7 +1720,7 @@
         <v>46307</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>91500</v>
+        <v>121500</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
@@ -1745,11 +1745,11 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>146379</v>
+        <v>146378</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1812,11 +1812,11 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>146378</v>
+        <v>146377</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1854,7 +1854,7 @@
         <v>46307</v>
       </c>
       <c r="L16" s="15" t="n">
-        <v>121500</v>
+        <v>93500</v>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
@@ -1879,11 +1879,11 @@
         </is>
       </c>
       <c r="B17" s="18" t="n">
-        <v>146377</v>
+        <v>146355</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1946,11 +1946,11 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>146355</v>
+        <v>146376</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1988,7 +1988,7 @@
         <v>46307</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>93500</v>
+        <v>86800</v>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
@@ -2013,11 +2013,11 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>146376</v>
+        <v>146390</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2031,31 +2031,31 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="J19" s="22" t="n">
-        <v>46293</v>
+        <v>46282</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46307</v>
+        <v>46296</v>
       </c>
       <c r="L19" s="23" t="n">
-        <v>86800</v>
+        <v>49580</v>
       </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="N19" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>selecaopnud0326@pge.ba.gov.br</t>
         </is>
       </c>
       <c r="O19" s="24" t="inlineStr">
@@ -2080,16 +2080,16 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>146390</v>
+        <v>146394</v>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2102,27 +2102,27 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J20" s="14" t="n">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46296</v>
+        <v>46304</v>
       </c>
       <c r="L20" s="15" t="n">
-        <v>49580</v>
+        <v>90000</v>
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="N20" s="12" t="inlineStr">
         <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O20" s="16" t="inlineStr">
@@ -2147,11 +2147,11 @@
         </is>
       </c>
       <c r="B21" s="18" t="n">
-        <v>146394</v>
+        <v>146396</v>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
+          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2169,27 +2169,27 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I21" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília, com disponibilidade para viagens</t>
         </is>
       </c>
       <c r="J21" s="22" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="L21" s="23" t="n">
-        <v>90000</v>
+        <v>208966.53</v>
       </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="N21" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>selecao.spt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O21" s="24" t="inlineStr">
@@ -2210,15 +2210,17 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="n">
-        <v>146396</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2228,49 +2230,37 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>Brasília, com disponibilidade para viagens</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46303</v>
-      </c>
-      <c r="L22" s="15" t="n">
-        <v>208966.53</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr">
-        <is>
-          <t>selecao.spt@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr"/>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2282,12 +2272,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2297,13 +2287,15 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2339,12 +2331,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2354,15 +2346,13 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr"/>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2398,12 +2388,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2419,7 +2409,7 @@
       <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2455,12 +2445,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2512,12 +2502,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2569,28 +2559,30 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2600,10 +2592,10 @@
       </c>
       <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46286</v>
+        <v>46296</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46316</v>
+        <v>46303</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
@@ -2626,17 +2618,17 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:31acdc9f-bf0b-43fe-5017-08df1966cd05</t>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 01/2026 - 01 vaga - Consultor Individual</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2649,7 +2641,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2659,10 +2651,10 @@
       </c>
       <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46295</v>
+        <v>46299</v>
       </c>
       <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
@@ -2680,138 +2672,158 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:4d25520a-6684-41e6-3080-08df1a5635e8</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 02/2026 - 01 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+        </is>
+      </c>
       <c r="J30" s="14" t="n">
-        <v>46291</v>
+        <v>46227</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L30" s="15" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L30" s="15" t="n">
+        <v>286000</v>
+      </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:c0a1d55e-84e2-4c98-3081-08df1a5635e8</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1161.2 - Edital nº 03/2026 - 01 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J31" s="22" t="n">
-        <v>46291</v>
+        <v>46240</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L31" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L31" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>unesco:7f118a1a-eb71-48a2-e28d-08df14acbbca</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 40/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2820,52 +2832,62 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J32" s="14" t="n">
-        <v>46289</v>
+        <v>46240</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L32" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L32" s="15" t="n">
+        <v>204000</v>
+      </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2879,35 +2901,45 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I33" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J33" s="22" t="n">
-        <v>46292</v>
+        <v>46240</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46299</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>204000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N33" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2919,12 +2951,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2962,7 +2994,7 @@
         <v>46245</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>80000</v>
+        <v>100000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2976,7 +3008,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -2988,12 +3020,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3011,7 +3043,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3021,7 +3053,7 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
@@ -3031,7 +3063,7 @@
         <v>46245</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3045,7 +3077,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3057,12 +3089,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3080,27 +3112,27 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3114,7 +3146,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3126,12 +3158,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3149,27 +3181,27 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3183,7 +3215,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3195,17 +3227,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3218,27 +3250,27 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>80000</v>
+        <v>50000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3252,7 +3284,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3264,12 +3296,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3279,37 +3311,37 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F39" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F39" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46252</v>
-      </c>
-      <c r="L39" s="23" t="n">
-        <v>286000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L39" s="23" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3319,7 +3351,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3331,17 +3363,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3354,7 +3386,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3364,17 +3396,17 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3388,7 +3420,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3400,12 +3432,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3423,7 +3455,7 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3440,14 +3472,14 @@
         <v>46246</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46257</v>
+        <v>46272</v>
       </c>
       <c r="L41" s="23" t="n">
         <v>54000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3457,7 +3489,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3469,22 +3501,22 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
@@ -3492,27 +3524,27 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46257</v>
+        <v>46270</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3526,7 +3558,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3538,17 +3570,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3566,36 +3598,36 @@
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46252</v>
+        <v>46208</v>
       </c>
       <c r="K43" s="22" t="n">
         <v>46259</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>60000</v>
+        <v>500000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3607,12 +3639,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3626,33 +3658,35 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46246</v>
+        <v>46266</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L44" s="15" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L44" s="15" t="n">
+        <v>70000</v>
+      </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3662,7 +3696,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3674,17 +3708,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3697,41 +3731,41 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46208</v>
+        <v>46275</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>500000</v>
+        <v>50000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3743,17 +3777,17 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -3762,35 +3796,33 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46246</v>
+        <v>46290</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L46" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L46" s="15" t="inlineStr"/>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -3800,7 +3832,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3812,12 +3844,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3827,7 +3859,7 @@
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
@@ -3835,7 +3867,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3845,17 +3877,17 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46265</v>
+        <v>46281</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46270</v>
+        <v>46286</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>30000</v>
+        <v>110000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3869,7 +3901,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3881,12 +3913,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3896,7 +3928,7 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
@@ -3904,7 +3936,7 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3914,17 +3946,17 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46266</v>
+        <v>46282</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3938,7 +3970,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3950,17 +3982,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3969,11 +4001,11 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -3983,18 +4015,16 @@
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K49" s="22" t="n">
         <v>46281</v>
       </c>
-      <c r="K49" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L49" s="23" t="n">
-        <v>110000</v>
-      </c>
+      <c r="L49" s="23" t="inlineStr"/>
       <c r="M49" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4007,7 +4037,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4049,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4042,39 +4072,39 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46275</v>
+        <v>46278</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46281</v>
+        <v>46295</v>
       </c>
       <c r="L50" s="15" t="inlineStr"/>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -4086,17 +4116,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4109,41 +4139,41 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46275</v>
+        <v>46244</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46280</v>
+        <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>50000</v>
+        <v>350000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4155,17 +4185,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4174,30 +4204,32 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46290</v>
+        <v>46294</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L52" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L52" s="15" t="n">
+        <v>55000</v>
+      </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4210,7 +4242,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -4222,12 +4254,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4241,11 +4273,11 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -4255,21 +4287,21 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46282</v>
+        <v>46293</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46286</v>
+        <v>46298</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
@@ -4279,7 +4311,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -4291,22 +4323,22 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
@@ -4314,41 +4346,41 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46244</v>
+        <v>46293</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>935000</v>
+        <v>30000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -4360,12 +4392,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4375,35 +4407,35 @@
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.335</v>
+        <v>0.4</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>21000</v>
+        <v>600000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -4417,7 +4449,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -4429,17 +4461,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4457,36 +4489,36 @@
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46244</v>
+        <v>46294</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>350000</v>
+        <v>60000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -4498,12 +4530,12 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -4517,43 +4549,45 @@
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46278</v>
+        <v>46296</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L57" s="23" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L57" s="23" t="n">
+        <v>60000</v>
+      </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -4565,12 +4599,12 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -4580,7 +4614,7 @@
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
@@ -4598,17 +4632,17 @@
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
@@ -4622,7 +4656,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4634,12 +4668,12 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
@@ -4657,27 +4691,27 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K59" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>55000</v>
+        <v>36000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
@@ -4691,7 +4725,7 @@
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4703,12 +4737,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -4722,11 +4756,11 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
@@ -4736,21 +4770,21 @@
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>600000</v>
+        <v>21000</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
@@ -4760,7 +4794,7 @@
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4772,12 +4806,12 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
@@ -4791,50 +4825,119 @@
         </is>
       </c>
       <c r="F61" s="21" t="n">
+        <v>0.347</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>Vitória - ES</t>
+        </is>
+      </c>
+      <c r="J61" s="22" t="n">
+        <v>46296</v>
+      </c>
+      <c r="K61" s="22" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L61" s="23" t="n">
+        <v>33000</v>
+      </c>
+      <c r="M61" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N61" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O61" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="G61" s="19" t="inlineStr">
+      <c r="G62" s="11" t="inlineStr">
         <is>
           <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
-      <c r="H61" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J61" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="K61" s="22" t="n">
-        <v>46302</v>
-      </c>
-      <c r="L61" s="23" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M61" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N61" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O61" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+      <c r="H62" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J62" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K62" s="14" t="n">
+        <v>46296</v>
+      </c>
+      <c r="L62" s="15" t="n">
+        <v>935000</v>
+      </c>
+      <c r="M62" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N62" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O62" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O61"/>
+  <autoFilter ref="A1:O62"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4896,6 +4999,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4934,7 +5038,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -4944,7 +5048,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -4954,7 +5058,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -4996,7 +5100,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -5006,7 +5110,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -5054,21 +5158,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -5130,7 +5234,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -5140,7 +5244,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -5150,7 +5254,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -5160,7 +5264,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -5170,7 +5274,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -5190,7 +5294,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -5200,7 +5304,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5238,27 +5342,27 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
@@ -5272,7 +5376,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -5282,7 +5386,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -5360,7 +5464,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5375,7 +5479,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5390,7 +5494,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5405,7 +5509,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-03 15:53
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$56</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 01/10/2026 às 18:09</t>
+          <t>Gerado em 03/10/2026 às 15:47</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>123620.4878048781</v>
+        <v>121990.5263157895</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>86800</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,11 +876,11 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146370</v>
+        <v>146374</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -890,13 +890,15 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
@@ -906,17 +908,17 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46297</v>
+        <v>46310</v>
       </c>
       <c r="L2" s="15" t="n">
-        <v>126000</v>
+        <v>120000</v>
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
@@ -941,11 +943,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146374</v>
+        <v>146375</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -973,7 +975,7 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
@@ -1008,11 +1010,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146375</v>
+        <v>146385</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1035,22 +1037,22 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46280</v>
+        <v>46289</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1059,7 +1061,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1075,16 +1077,16 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146384</v>
+        <v>146354</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Edital 05/2026 - Estudos e análises para o fortalecimento da perspectiva de gênero nas políticas públicas de direitos humanos</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -1093,7 +1095,7 @@
         </is>
       </c>
       <c r="F5" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
@@ -1102,22 +1104,22 @@
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46283</v>
+        <v>46293</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>120000</v>
+        <v>93500</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1126,7 +1128,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>dirp@mdh.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1142,11 +1144,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146385</v>
+        <v>146382</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1160,31 +1162,31 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>100000</v>
+        <v>91500</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1193,7 +1195,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1209,16 +1211,16 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146380</v>
+        <v>146379</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 138/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A PROPOSIÇÃO DE PLATAFORMAS E DASHBOARDS DE VISUALIZAÇÃO DE DADOS PARA A AGENDA DE DESENVOLVIMENTO HUMANO</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -1245,13 +1247,13 @@
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>126500</v>
+        <v>121500</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1276,16 +1278,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146381</v>
+        <v>146378</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 139/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A SISTEMATIZAÇÃO E ELABORAÇÃO DO DOSSIÊ INSTITUCIONAL DA SÉRIE DIÁLOGOS NACIONAIS PARA O DESENVOLVIMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -1312,13 +1314,13 @@
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>126500</v>
+        <v>121500</v>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
@@ -1343,16 +1345,16 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146383</v>
+        <v>146377</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 145/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE ALGORITMO DE GEOCODIFICAÇÃO DE ENDEREÇOS BRASILEIROS.</t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
@@ -1365,7 +1367,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1379,13 +1381,13 @@
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>86800</v>
+        <v>93500</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1410,11 +1412,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146354</v>
+        <v>146355</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1432,7 +1434,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1477,11 +1479,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146357</v>
+        <v>146376</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 141/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA PARA ANÁLISE TERRITORIAL DO DESENVOLVIMENTO HUMANO.</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1499,7 +1501,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1513,13 +1515,13 @@
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46287</v>
+        <v>46293</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46296</v>
+        <v>46307</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>126500</v>
+        <v>86800</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1544,16 +1546,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146358</v>
+        <v>146394</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 142/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE METODOLOGIA DE MODELAGEM PREDITIVA COM FOCO NO PROCESSAMENTO E INTEGRAÇÃO DE DADOS GEOESPACIAIS.</t>
+          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1562,16 +1564,16 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -1580,13 +1582,13 @@
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46296</v>
+        <v>46304</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>126500</v>
+        <v>90000</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1595,7 +1597,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1611,11 +1613,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146382</v>
+        <v>146396</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1629,31 +1631,31 @@
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília, com disponibilidade para viagens</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46307</v>
+        <v>46303</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>91500</v>
+        <v>208966.53</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1662,7 +1664,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>selecao.spt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1674,87 +1676,79 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>146379</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr"/>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L14" s="15" t="n">
-        <v>121500</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr"/>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="n">
-        <v>146378</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
@@ -1763,333 +1757,285 @@
         </is>
       </c>
       <c r="F15" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L15" s="23" t="n">
-        <v>121500</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr"/>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="n">
-        <v>146377</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr"/>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L16" s="15" t="n">
-        <v>93500</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr"/>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>146355</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr"/>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L17" s="23" t="n">
-        <v>93500</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr"/>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="n">
-        <v>146376</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L18" s="15" t="n">
-        <v>86800</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr"/>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="n">
-        <v>146390</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>BRA/24/018 - CONTRATAÇÃO DE CONSULTOR ESPECIALIZADO EM POLÍTICA DE INOVAÇÃO E DE TRANSFORMAÇÃO DIGITAL</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr">
-        <is>
-          <t>Salvador/BA</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L19" s="23" t="n">
-        <v>49580</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr">
-        <is>
-          <t>selecaopnud0326@pge.ba.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr"/>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="n">
-        <v>146394</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+        </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
+          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2102,61 +2048,53 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46289</v>
+        <v>46296</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46304</v>
-      </c>
-      <c r="L20" s="15" t="n">
-        <v>90000</v>
-      </c>
+        <v>46303</v>
+      </c>
+      <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr">
-        <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr"/>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="n">
-        <v>146396</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+        </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
+          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2169,120 +2107,122 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="inlineStr">
-        <is>
-          <t>Brasília, com disponibilidade para viagens</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46303</v>
-      </c>
-      <c r="L21" s="23" t="n">
-        <v>208966.53</v>
-      </c>
+        <v>46299</v>
+      </c>
+      <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N21" s="20" t="inlineStr">
-        <is>
-          <t>selecao.spt@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N21" s="20" t="inlineStr"/>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J22" s="14" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L22" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L22" s="15" t="n">
+        <v>100000</v>
+      </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
@@ -2291,114 +2231,136 @@
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I23" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J23" s="22" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L23" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L23" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N23" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N23" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J24" s="14" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L24" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L24" s="15" t="n">
+        <v>204000</v>
+      </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N24" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2414,157 +2376,191 @@
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr">
+        <is>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+        </is>
+      </c>
       <c r="J25" s="22" t="n">
-        <v>46286</v>
+        <v>46227</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L25" s="23" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L25" s="23" t="n">
+        <v>286000</v>
+      </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N25" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N25" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J26" s="14" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L26" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L26" s="15" t="n">
+        <v>204000</v>
+      </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - Df</t>
+        </is>
+      </c>
       <c r="J27" s="22" t="n">
-        <v>46286</v>
+        <v>46240</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L27" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L27" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2582,48 +2578,56 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF | Híbrido</t>
+        </is>
+      </c>
       <c r="J28" s="14" t="n">
-        <v>46296</v>
+        <v>46246</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46303</v>
+        <v>46250</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2637,35 +2641,45 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>Porto Alegre/RS</t>
+        </is>
+      </c>
       <c r="J29" s="22" t="n">
-        <v>46292</v>
+        <v>46246</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46299</v>
-      </c>
-      <c r="L29" s="23" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L29" s="23" t="n">
+        <v>54000</v>
+      </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2677,12 +2691,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2692,13 +2706,15 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2708,17 +2724,17 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46227</v>
+        <v>46252</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>286000</v>
+        <v>60000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2732,7 +2748,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2760,17 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2767,27 +2783,27 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>80000</v>
+        <v>50000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2801,7 +2817,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2813,12 +2829,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2836,27 +2852,27 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2870,7 +2886,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2882,17 +2898,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2905,41 +2921,41 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46240</v>
+        <v>46208</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46245</v>
+        <v>46259</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>204000</v>
+        <v>500000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -2951,12 +2967,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2974,31 +2990,31 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46245</v>
+        <v>46272</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>100000</v>
+        <v>54000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -3008,7 +3024,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3020,22 +3036,22 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
@@ -3043,7 +3059,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3053,17 +3069,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46240</v>
+        <v>46265</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46245</v>
+        <v>46270</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>80000</v>
+        <v>30000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3077,7 +3093,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3089,12 +3105,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3112,7 +3128,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3122,17 +3138,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46246</v>
+        <v>46266</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46257</v>
+        <v>46288</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>54000</v>
+        <v>70000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3146,7 +3162,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3158,12 +3174,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3181,27 +3197,27 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46257</v>
+        <v>46280</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3215,7 +3231,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3227,17 +3243,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3246,32 +3262,30 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46251</v>
+        <v>46275</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L38" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L38" s="15" t="inlineStr"/>
       <c r="M38" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3284,7 +3298,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3296,12 +3310,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3311,37 +3325,39 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46246</v>
+        <v>46282</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L39" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L39" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3351,7 +3367,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3363,17 +3379,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3386,27 +3402,27 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46252</v>
+        <v>46281</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46259</v>
+        <v>46286</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>60000</v>
+        <v>110000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3420,7 +3436,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3432,12 +3448,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3451,11 +3467,11 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3465,31 +3481,29 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46246</v>
+        <v>46278</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L41" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3501,30 +3515,30 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3534,18 +3548,16 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46265</v>
+        <v>46290</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3558,7 +3570,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3570,12 +3582,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3593,7 +3605,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3607,17 +3619,17 @@
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46208</v>
+        <v>46244</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46259</v>
+        <v>46300</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>500000</v>
+        <v>350000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3627,7 +3639,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3639,12 +3651,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3654,15 +3666,15 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3672,21 +3684,21 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46266</v>
+        <v>46293</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46288</v>
+        <v>46298</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>70000</v>
+        <v>21000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3696,7 +3708,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3708,12 +3720,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3731,7 +3743,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3741,21 +3753,21 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46275</v>
+        <v>46294</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46280</v>
+        <v>46297</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>50000</v>
+        <v>600000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3765,7 +3777,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3777,49 +3789,51 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L46" s="15" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L46" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3832,7 +3846,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3844,17 +3858,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3867,7 +3881,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3877,17 +3891,17 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46281</v>
+        <v>46296</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>110000</v>
+        <v>60000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3901,7 +3915,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3913,12 +3927,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3928,7 +3942,7 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
@@ -3936,7 +3950,7 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3950,13 +3964,13 @@
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46282</v>
+        <v>46294</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>30000</v>
+        <v>55000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3970,7 +3984,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3982,12 +3996,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -4001,30 +4015,32 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46275</v>
+        <v>46294</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L49" s="23" t="inlineStr"/>
+        <v>46302</v>
+      </c>
+      <c r="L49" s="23" t="n">
+        <v>60000</v>
+      </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4037,7 +4053,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -4049,17 +4065,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4068,43 +4084,45 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46278</v>
+        <v>46244</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L50" s="15" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>935000</v>
+      </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4116,17 +4134,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4135,45 +4153,45 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K51" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>350000</v>
+        <v>33000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4185,12 +4203,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4208,7 +4226,7 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
@@ -4222,13 +4240,13 @@
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K52" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4242,7 +4260,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4254,12 +4272,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4269,39 +4287,39 @@
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.335</v>
+        <v>0.4</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>21000</v>
+        <v>36000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
@@ -4311,7 +4329,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4323,12 +4341,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4338,35 +4356,35 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
@@ -4380,7 +4398,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4392,12 +4410,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4415,31 +4433,31 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46297</v>
+        <v>46311</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>600000</v>
+        <v>90000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
@@ -4449,7 +4467,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4461,12 +4479,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4484,7 +4502,7 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
@@ -4498,13 +4516,13 @@
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46302</v>
+        <v>46311</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>60000</v>
+        <v>70000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
@@ -4518,426 +4536,12 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B57" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
-        </is>
-      </c>
-      <c r="C57" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
-        </is>
-      </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E57" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F57" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G57" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H57" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I57" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
-      <c r="J57" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K57" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L57" s="23" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M57" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N57" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O57" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
-        </is>
-      </c>
-      <c r="C58" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E58" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F58" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G58" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H58" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I58" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J58" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K58" s="14" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L58" s="15" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M58" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N58" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O58" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B59" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
-        </is>
-      </c>
-      <c r="C59" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
-        </is>
-      </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E59" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F59" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G59" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H59" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I59" s="19" t="inlineStr">
-        <is>
-          <t>Vitória - ES</t>
-        </is>
-      </c>
-      <c r="J59" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K59" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L59" s="23" t="n">
-        <v>36000</v>
-      </c>
-      <c r="M59" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N59" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O59" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
-        </is>
-      </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F60" s="13" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="G60" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H60" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I60" s="11" t="inlineStr">
-        <is>
-          <t>Vitória - ES</t>
-        </is>
-      </c>
-      <c r="J60" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K60" s="14" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L60" s="15" t="n">
-        <v>21000</v>
-      </c>
-      <c r="M60" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N60" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O60" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B61" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F61" s="21" t="n">
-        <v>0.347</v>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H61" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>Vitória - ES</t>
-        </is>
-      </c>
-      <c r="J61" s="22" t="n">
-        <v>46296</v>
-      </c>
-      <c r="K61" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L61" s="23" t="n">
-        <v>33000</v>
-      </c>
-      <c r="M61" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N61" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O61" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F62" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J62" s="14" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K62" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L62" s="15" t="n">
-        <v>935000</v>
-      </c>
-      <c r="M62" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N62" s="12" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O62" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O62"/>
+  <autoFilter ref="A1:O56"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4994,12 +4598,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5038,7 +4636,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -5048,7 +4646,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -5100,7 +4698,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -5110,7 +4708,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -5162,7 +4760,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -5172,7 +4770,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -5182,7 +4780,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -5234,7 +4832,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -5244,7 +4842,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -5254,7 +4852,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -5264,7 +4862,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -5274,7 +4872,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -5356,27 +4954,27 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -5386,13 +4984,13 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -5402,11 +5000,11 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -5464,7 +5062,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5479,7 +5077,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5494,7 +5092,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5509,7 +5107,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-06 18:06
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 03/10/2026 às 15:47</t>
+          <t>Gerado em 06/10/2026 às 17:59</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>121990.5263157895</v>
+        <v>116902.8988571428</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>80000</v>
+        <v>62500</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1676,17 +1676,15 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>146401</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1696,37 +1694,49 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Território Nacional</t>
+        </is>
+      </c>
       <c r="J14" s="14" t="n">
-        <v>46286</v>
+        <v>46301</v>
       </c>
       <c r="K14" s="14" t="n">
         <v>46316</v>
       </c>
-      <c r="L14" s="15" t="inlineStr"/>
+      <c r="L14" s="15" t="n">
+        <v>120000</v>
+      </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr">
+        <is>
+          <t>cgti@mdh.gov.br</t>
+        </is>
+      </c>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1738,12 +1748,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1761,7 +1771,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1771,10 +1781,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46316</v>
+        <v>46304</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1797,12 +1807,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1818,7 +1828,7 @@
       <c r="F16" s="13" t="inlineStr"/>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1854,12 +1864,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1869,13 +1879,15 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1911,12 +1923,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1932,7 +1944,7 @@
       <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1968,12 +1980,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2025,30 +2037,28 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2058,10 +2068,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46296</v>
+        <v>46286</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46303</v>
+        <v>46316</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2084,30 +2094,28 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:80185502-579b-44a1-e3c6-08df13ea9ffe</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 22/2026</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr"/>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2117,10 +2125,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46292</v>
+        <v>46286</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46299</v>
+        <v>46316</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2138,17 +2146,17 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2162,45 +2170,35 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46240</v>
+        <v>46296</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L22" s="15" t="n">
-        <v>100000</v>
-      </c>
+        <v>46303</v>
+      </c>
+      <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr"/>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2212,12 +2210,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2235,27 +2233,27 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2269,7 +2267,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2281,12 +2279,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2304,7 +2302,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2324,7 +2322,7 @@
         <v>46245</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>204000</v>
+        <v>100000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -2338,7 +2336,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -2350,12 +2348,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2365,13 +2363,15 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2381,17 +2381,17 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46252</v>
+        <v>46257</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>286000</v>
+        <v>54000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2417,12 +2417,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2436,11 +2436,11 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2450,21 +2450,19 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L26" s="15" t="n">
-        <v>204000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
@@ -2474,7 +2472,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2486,12 +2484,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2501,35 +2499,33 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="inlineStr"/>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>80000</v>
+        <v>286000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2543,7 +2539,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2555,17 +2551,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2574,33 +2570,35 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L28" s="15" t="inlineStr"/>
+        <v>46256</v>
+      </c>
+      <c r="L28" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N28" s="12" t="inlineStr">
@@ -2610,7 +2608,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2622,12 +2620,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2645,7 +2643,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2655,17 +2653,17 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2679,7 +2677,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2691,12 +2689,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2714,7 +2712,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2724,21 +2722,21 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46259</v>
+        <v>46272</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2748,7 +2746,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -2760,17 +2758,17 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2783,7 +2781,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2793,17 +2791,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46251</v>
+        <v>46266</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46256</v>
+        <v>46288</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>50000</v>
+        <v>70000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2817,7 +2815,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -2829,22 +2827,22 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
@@ -2852,27 +2850,27 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46257</v>
+        <v>46270</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2886,7 +2884,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -2898,17 +2896,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2917,45 +2915,43 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46208</v>
+        <v>46275</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>500000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -2967,12 +2963,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2982,7 +2978,7 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
@@ -2990,7 +2986,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -3000,21 +2996,21 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46246</v>
+        <v>46282</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46272</v>
+        <v>46286</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -3024,7 +3020,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3036,22 +3032,22 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
@@ -3059,7 +3055,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3069,17 +3065,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46265</v>
+        <v>46275</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46270</v>
+        <v>46280</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3093,7 +3089,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3105,17 +3101,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3128,27 +3124,27 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>70000</v>
+        <v>110000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3162,7 +3158,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3174,17 +3170,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3193,11 +3189,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3207,18 +3203,16 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46275</v>
+        <v>46290</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>50000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3231,7 +3225,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3243,12 +3237,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3266,39 +3260,39 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46275</v>
+        <v>46278</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46281</v>
+        <v>46295</v>
       </c>
       <c r="L38" s="15" t="inlineStr"/>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3310,12 +3304,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3325,7 +3319,7 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
@@ -3333,7 +3327,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3343,17 +3337,17 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46282</v>
+        <v>46294</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46286</v>
+        <v>46302</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3367,7 +3361,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3379,54 +3373,54 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46281</v>
+        <v>46293</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46286</v>
+        <v>46298</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>110000</v>
+        <v>21000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3436,7 +3430,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3448,12 +3442,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3463,15 +3457,15 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3481,29 +3475,31 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46278</v>
+        <v>46293</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L41" s="23" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L41" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3515,17 +3511,17 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -3534,30 +3530,32 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46290</v>
+        <v>46294</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L42" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <v>55000</v>
+      </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3570,7 +3568,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3582,17 +3580,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3605,27 +3603,27 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46244</v>
+        <v>46294</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>350000</v>
+        <v>600000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3634,12 +3632,12 @@
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3651,12 +3649,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3666,39 +3664,39 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.335</v>
+        <v>0.4</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3708,7 +3706,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3720,12 +3718,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3739,11 +3737,11 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3753,21 +3751,21 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>600000</v>
+        <v>33000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3777,7 +3775,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -3789,12 +3787,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3804,7 +3802,7 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
@@ -3822,17 +3820,17 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3846,7 +3844,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3858,12 +3856,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3877,11 +3875,11 @@
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3891,7 +3889,7 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
@@ -3901,7 +3899,7 @@
         <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3915,7 +3913,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -3927,12 +3925,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3950,27 +3948,27 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K48" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>55000</v>
+        <v>36000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3984,7 +3982,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -3996,12 +3994,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -4019,7 +4017,7 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -4033,13 +4031,13 @@
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46302</v>
+        <v>46311</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>60000</v>
+        <v>70000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4053,7 +4051,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4134,17 +4132,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4153,7 +4151,7 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
@@ -4162,36 +4160,36 @@
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46300</v>
+        <v>46315</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>33000</v>
+        <v>600000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4203,17 +4201,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4226,27 +4224,27 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>60000</v>
+        <v>62500</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4260,7 +4258,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4272,12 +4270,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4295,31 +4293,31 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>36000</v>
+        <v>90000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
@@ -4329,7 +4327,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4341,17 +4339,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4360,188 +4358,50 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46296</v>
+        <v>46244</v>
       </c>
       <c r="K54" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>21000</v>
+        <v>350000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B55" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
-        </is>
-      </c>
-      <c r="C55" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
-        </is>
-      </c>
-      <c r="D55" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E55" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F55" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G55" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H55" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I55" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J55" s="22" t="n">
-        <v>46297</v>
-      </c>
-      <c r="K55" s="22" t="n">
-        <v>46311</v>
-      </c>
-      <c r="L55" s="23" t="n">
-        <v>90000</v>
-      </c>
-      <c r="M55" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N55" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O55" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
-        </is>
-      </c>
-      <c r="C56" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E56" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F56" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G56" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H56" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I56" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J56" s="14" t="n">
-        <v>46297</v>
-      </c>
-      <c r="K56" s="14" t="n">
-        <v>46311</v>
-      </c>
-      <c r="L56" s="15" t="n">
-        <v>70000</v>
-      </c>
-      <c r="M56" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N56" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O56" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O56"/>
+  <autoFilter ref="A1:O54"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4596,8 +4456,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4636,7 +4494,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -4646,7 +4504,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -4698,7 +4556,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -4760,7 +4618,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -4770,7 +4628,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -4832,7 +4690,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4842,7 +4700,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -4862,7 +4720,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -4878,7 +4736,7 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Direito / Jurídico</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -4888,17 +4746,17 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Direito / Jurídico</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
@@ -4918,7 +4776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4940,7 +4798,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -4950,11 +4808,11 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -4990,21 +4848,21 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -5017,8 +4875,18 @@
         <v>1</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>OEI/SECULT</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5062,7 +4930,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5077,7 +4945,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5092,7 +4960,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5107,7 +4975,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-07 18:37
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,17 +17,17 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$55</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Por_Perfil'!$A$1:$B$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Por_Perfil'!$A$1:$B$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Por_Perfil'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Por_Tipo'!$A$1:$B$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 06/10/2026 às 17:59</t>
+          <t>Gerado em 07/10/2026 às 18:29</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>935000</v>
+        <v>2778901.38</v>
       </c>
     </row>
     <row r="19">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>116902.8988571428</v>
+        <v>191958.4122222222</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>62500</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -755,6 +755,16 @@
       </c>
       <c r="B25" s="6" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Pesquisador Computacao</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -772,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2210,17 +2220,17 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
@@ -2233,7 +2243,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2243,17 +2253,17 @@
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2267,7 +2277,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2289,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2302,27 +2312,27 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>100000</v>
+        <v>54000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -2336,7 +2346,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2348,12 +2358,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2363,15 +2373,13 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2381,17 +2389,17 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46257</v>
+        <v>46252</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>54000</v>
+        <v>286000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
@@ -2405,7 +2413,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2484,12 +2492,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2499,13 +2507,15 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2515,17 +2525,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46252</v>
+        <v>46257</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>286000</v>
+        <v>54000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2539,7 +2549,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2551,17 +2561,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2574,7 +2584,7 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2584,17 +2594,17 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2608,7 +2618,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2620,12 +2630,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2643,7 +2653,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2653,21 +2663,21 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46259</v>
+        <v>46272</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2677,7 +2687,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -2689,17 +2699,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2712,31 +2722,31 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46246</v>
+        <v>46281</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46272</v>
+        <v>46286</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>54000</v>
+        <v>110000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2746,7 +2756,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -2758,12 +2768,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2777,32 +2787,30 @@
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46266</v>
+        <v>46275</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46288</v>
-      </c>
-      <c r="L31" s="23" t="n">
-        <v>70000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2815,7 +2823,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -2896,12 +2904,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2915,30 +2923,32 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>70000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2951,7 +2961,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3101,17 +3111,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3124,7 +3134,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3134,21 +3144,21 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46281</v>
+        <v>46294</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46286</v>
+        <v>46297</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>110000</v>
+        <v>600000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3158,7 +3168,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3170,52 +3180,54 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.335</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>21000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3225,7 +3237,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3237,12 +3249,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3252,15 +3264,15 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3270,29 +3282,31 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46278</v>
+        <v>46293</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L38" s="15" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3304,12 +3318,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3323,11 +3337,11 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3341,27 +3355,25 @@
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46294</v>
+        <v>46278</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46302</v>
-      </c>
-      <c r="L39" s="23" t="n">
-        <v>60000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L39" s="23" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3373,54 +3385,52 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.335</v>
+        <v>0.3</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L40" s="15" t="n">
-        <v>21000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L40" s="15" t="inlineStr"/>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3430,7 +3440,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3442,12 +3452,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3457,7 +3467,7 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
@@ -3465,7 +3475,7 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3475,17 +3485,17 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>30000</v>
+        <v>55000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3499,7 +3509,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3511,12 +3521,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3534,7 +3544,7 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3544,17 +3554,17 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
         <v>46294</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3568,7 +3578,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3580,12 +3590,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3603,31 +3613,31 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>600000</v>
+        <v>60000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3637,7 +3647,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3718,17 +3728,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3737,45 +3747,45 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K45" s="22" t="n">
         <v>46296</v>
       </c>
-      <c r="K45" s="22" t="n">
-        <v>46300</v>
-      </c>
       <c r="L45" s="23" t="n">
-        <v>33000</v>
+        <v>935000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3787,12 +3797,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3806,21 +3816,21 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
@@ -3830,7 +3840,7 @@
         <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>60000</v>
+        <v>33000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3844,7 +3854,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4063,12 +4073,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4103,10 +4113,10 @@
         <v>46244</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>935000</v>
+        <v>350000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4120,7 +4130,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4201,17 +4211,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4224,31 +4234,31 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46305</v>
+        <v>46311</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>62500</v>
+        <v>90000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
@@ -4258,7 +4268,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4270,17 +4280,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4293,31 +4303,31 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46311</v>
+        <v>46305</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>90000</v>
+        <v>62500</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
@@ -4327,7 +4337,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4339,17 +4349,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4362,46 +4372,115 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46244</v>
+        <v>46302</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>350000</v>
+        <v>140000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O54" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>Pesquisador Computacao</t>
+        </is>
+      </c>
+      <c r="F55" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G55" s="19" t="inlineStr">
+        <is>
+          <t>Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H55" s="19" t="inlineStr">
+        <is>
+          <t>OEI/FPOS</t>
+        </is>
+      </c>
+      <c r="I55" s="19" t="inlineStr">
+        <is>
+          <t>Território Nacional</t>
+        </is>
+      </c>
+      <c r="J55" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K55" s="22" t="n">
+        <v>46322</v>
+      </c>
+      <c r="L55" s="23" t="n">
+        <v>2778901.38</v>
+      </c>
+      <c r="M55" s="17" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N55" s="20" t="inlineStr">
+        <is>
           <t>compras.bra@oei.int</t>
         </is>
       </c>
-      <c r="O54" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+      <c r="O55" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O54"/>
+  <autoFilter ref="A1:O55"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4456,6 +4535,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4494,7 +4574,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -4530,7 +4610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4579,8 +4659,18 @@
         <v>4</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>Pesquisador Computacao</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B4"/>
+  <autoFilter ref="A1:B5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4618,7 +4708,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -4638,7 +4728,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -4648,7 +4738,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4690,7 +4780,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -4700,7 +4790,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -4710,7 +4800,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -4720,7 +4810,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -4776,7 +4866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4802,7 +4892,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -4812,7 +4902,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -4885,8 +4975,18 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>OEI/FPOS</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4975,7 +5075,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-08 18:35
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$58</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 07/10/2026 às 18:29</t>
+          <t>Gerado em 08/10/2026 às 18:28</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>191958.4122222222</v>
+        <v>186276.3905263158</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1758,12 +1758,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1773,15 +1773,13 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F15" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="inlineStr"/>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1791,10 +1789,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1817,12 +1815,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1832,13 +1830,15 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1848,10 +1848,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46316</v>
+        <v>46304</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1874,12 +1874,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1889,15 +1889,13 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr"/>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1933,12 +1931,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1948,13 +1946,15 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1990,12 +1990,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2011,7 +2011,7 @@
       <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2047,12 +2047,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2104,12 +2104,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2161,30 +2161,28 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2194,10 +2192,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46296</v>
+        <v>46286</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46303</v>
+        <v>46316</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2215,22 +2213,22 @@
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
@@ -2239,45 +2237,35 @@
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I23" s="19" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46251</v>
+        <v>46296</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L23" s="23" t="n">
-        <v>50000</v>
-      </c>
+        <v>46303</v>
+      </c>
+      <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N23" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N23" s="20" t="inlineStr"/>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2277,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2312,7 +2300,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2346,7 +2334,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2492,17 +2480,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2515,7 +2503,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2525,17 +2513,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2549,7 +2537,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2561,12 +2549,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2584,7 +2572,7 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2594,17 +2582,17 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2618,7 +2606,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2630,12 +2618,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2653,7 +2641,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2663,21 +2651,21 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46272</v>
+        <v>46259</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2687,7 +2675,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2699,17 +2687,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2722,31 +2710,31 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46281</v>
+        <v>46246</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46286</v>
+        <v>46272</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>110000</v>
+        <v>54000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2756,7 +2744,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -2768,30 +2756,30 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2801,16 +2789,18 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46275</v>
+        <v>46265</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L31" s="23" t="inlineStr"/>
+        <v>46270</v>
+      </c>
+      <c r="L31" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2823,7 +2813,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -2835,22 +2825,22 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
@@ -2858,27 +2848,27 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46270</v>
+        <v>46288</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2892,7 +2882,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -2904,12 +2894,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2927,27 +2917,27 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46266</v>
+        <v>46275</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46288</v>
+        <v>46280</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>70000</v>
+        <v>50000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2961,7 +2951,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -2973,12 +2963,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2988,36 +2978,34 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46282</v>
+        <v>46275</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L34" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3030,7 +3018,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3042,17 +3030,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3065,7 +3053,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3075,17 +3063,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46275</v>
+        <v>46281</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>50000</v>
+        <v>110000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3099,7 +3087,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3111,12 +3099,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3130,32 +3118,30 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46294</v>
+        <v>46278</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46297</v>
-      </c>
-      <c r="L36" s="15" t="n">
-        <v>600000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L36" s="15" t="inlineStr"/>
       <c r="M36" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3163,12 +3149,12 @@
       </c>
       <c r="N36" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3180,54 +3166,52 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.335</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>21000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3237,7 +3221,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3249,12 +3233,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3268,11 +3252,11 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3282,7 +3266,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
@@ -3292,11 +3276,11 @@
         <v>46298</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3306,7 +3290,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3318,12 +3302,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3333,15 +3317,15 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3351,29 +3335,31 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46278</v>
+        <v>46282</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L39" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L39" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3385,49 +3371,51 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3440,7 +3428,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3452,12 +3440,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3475,7 +3463,7 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3489,13 +3477,13 @@
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K41" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3509,7 +3497,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3521,12 +3509,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3544,24 +3532,24 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L42" s="15" t="n">
         <v>60000</v>
@@ -3578,7 +3566,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3590,12 +3578,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3613,7 +3601,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3623,14 +3611,14 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L43" s="23" t="n">
         <v>60000</v>
@@ -3647,7 +3635,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3659,12 +3647,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3682,7 +3670,7 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3692,21 +3680,21 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>60000</v>
+        <v>600000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3716,7 +3704,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3728,17 +3716,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3751,41 +3739,41 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46244</v>
+        <v>46294</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>935000</v>
+        <v>55000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3797,12 +3785,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3816,7 +3804,7 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.347</v>
+        <v>0.33</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
@@ -3840,7 +3828,7 @@
         <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>33000</v>
+        <v>21000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3854,7 +3842,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -3866,12 +3854,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3885,7 +3873,7 @@
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.33</v>
+        <v>0.347</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
@@ -3909,7 +3897,7 @@
         <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>21000</v>
+        <v>33000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3923,7 +3911,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4073,12 +4061,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4113,10 +4101,10 @@
         <v>46244</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46300</v>
+        <v>46296</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>350000</v>
+        <v>935000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4130,7 +4118,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4142,12 +4130,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4165,27 +4153,27 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46301</v>
+        <v>46244</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>600000</v>
+        <v>350000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4199,7 +4187,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4280,17 +4268,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4303,41 +4291,41 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
         <v>46301</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46305</v>
+        <v>46315</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>62500</v>
+        <v>600000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4349,17 +4337,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4372,27 +4360,27 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>140000</v>
+        <v>62500</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
@@ -4406,7 +4394,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4418,69 +4406,276 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K55" s="22" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L55" s="23" t="n">
+        <v>27000</v>
+      </c>
+      <c r="M55" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N55" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O55" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F56" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+        </is>
+      </c>
+      <c r="J56" s="14" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K56" s="14" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>140000</v>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N56" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O56" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+        </is>
+      </c>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>Pesquisador Computacao</t>
+        </is>
+      </c>
+      <c r="F57" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G57" s="19" t="inlineStr">
+        <is>
+          <t>Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H57" s="19" t="inlineStr">
+        <is>
+          <t>OEI/FPOS</t>
+        </is>
+      </c>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>Território Nacional</t>
+        </is>
+      </c>
+      <c r="J57" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K57" s="22" t="n">
         <v>46322</v>
       </c>
-      <c r="L55" s="23" t="n">
+      <c r="L57" s="23" t="n">
         <v>2778901.38</v>
       </c>
-      <c r="M55" s="17" t="inlineStr">
+      <c r="M57" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N57" s="20" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O57" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H58" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J58" s="14" t="n">
+        <v>46303</v>
+      </c>
+      <c r="K58" s="14" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L58" s="15" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M58" s="9" t="inlineStr">
         <is>
           <t>En presentación</t>
         </is>
       </c>
-      <c r="N55" s="20" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O55" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+      <c r="N58" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O58" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O55"/>
+  <autoFilter ref="A1:O58"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4536,6 +4731,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4574,7 +4772,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -4594,7 +4792,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -4636,7 +4834,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3">
@@ -4646,7 +4844,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -4656,7 +4854,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -4708,7 +4906,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -4718,7 +4916,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -4780,7 +4978,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -4790,7 +4988,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -4800,7 +4998,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -4810,7 +5008,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -4820,7 +5018,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -4902,7 +5100,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -4912,7 +5110,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -5030,7 +5228,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5045,7 +5243,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5060,7 +5258,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5075,7 +5273,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-09 18:04
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 08/10/2026 às 18:28</t>
+          <t>Gerado em 09/10/2026 às 18:00</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24">
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1126,7 +1126,7 @@
         <v>46293</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L5" s="23" t="n">
         <v>93500</v>
@@ -1193,7 +1193,7 @@
         <v>46293</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L6" s="15" t="n">
         <v>91500</v>
@@ -1260,7 +1260,7 @@
         <v>46293</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L7" s="23" t="n">
         <v>121500</v>
@@ -1327,7 +1327,7 @@
         <v>46293</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L8" s="15" t="n">
         <v>121500</v>
@@ -1394,7 +1394,7 @@
         <v>46293</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L9" s="23" t="n">
         <v>93500</v>
@@ -1461,7 +1461,7 @@
         <v>46293</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L10" s="15" t="n">
         <v>93500</v>
@@ -1528,7 +1528,7 @@
         <v>46293</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46307</v>
+        <v>46313</v>
       </c>
       <c r="L11" s="23" t="n">
         <v>86800</v>
@@ -1623,11 +1623,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146396</v>
+        <v>146401</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>BRA/25/024 - Edital nº 013/2026 – Contratação de consultoria especializada (pessoa física) para desenvolvimento de estudo e análise sobre os efeitos econômicos e sociais dos recursos mobilizados pelo FAT e pelo FGTS</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1645,27 +1645,27 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Brasília, com disponibilidade para viagens</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46290</v>
+        <v>46301</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46303</v>
+        <v>46316</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>208966.53</v>
+        <v>120000</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>selecao.spt@trabalho.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1686,15 +1686,17 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>146401</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
+        </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1704,49 +1706,37 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr"/>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>Território Nacional</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L14" s="15" t="n">
-        <v>120000</v>
-      </c>
+        <v>46309</v>
+      </c>
+      <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr">
-        <is>
-          <t>cgti@mdh.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr"/>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -1758,12 +1748,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
+          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1773,13 +1763,15 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F15" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1789,7 +1781,7 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="K15" s="22" t="n">
         <v>46309</v>
@@ -1815,12 +1807,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
+          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1838,7 +1830,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1848,10 +1840,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1874,12 +1866,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1889,13 +1881,15 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1905,10 +1899,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1931,12 +1925,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1954,7 +1948,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1964,10 +1958,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1990,12 +1984,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2005,13 +1999,15 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2021,10 +2017,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46316</v>
+        <v>46304</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2047,12 +2043,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2104,12 +2100,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2119,13 +2115,15 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2161,12 +2159,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2182,7 +2180,7 @@
       <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2218,30 +2216,28 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:ec486dce-4c41-4830-4e64-08df1817d7a0</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 05/2026 - 02 vagas - Consultores Individuais</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr"/>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2251,10 +2247,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46296</v>
+        <v>46286</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46303</v>
+        <v>46316</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2272,91 +2268,79 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr"/>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L24" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N24" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr"/>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2372,36 +2356,26 @@
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr">
-        <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46227</v>
+        <v>46286</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46252</v>
-      </c>
-      <c r="L25" s="23" t="n">
-        <v>286000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N25" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N25" s="20" t="inlineStr"/>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2413,17 +2387,17 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -2432,33 +2406,35 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L26" s="15" t="inlineStr"/>
+        <v>46256</v>
+      </c>
+      <c r="L26" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
@@ -2468,7 +2444,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2480,17 +2456,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2503,7 +2479,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2513,17 +2489,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2537,7 +2513,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2525,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2572,7 +2548,7 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2606,7 +2582,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2618,12 +2594,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2637,35 +2613,33 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L29" s="23" t="n">
-        <v>60000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2675,7 +2649,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2687,12 +2661,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2702,15 +2676,13 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2720,21 +2692,21 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46272</v>
+        <v>46252</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>54000</v>
+        <v>286000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2744,7 +2716,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -2756,22 +2728,22 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F31" s="21" t="n">
@@ -2779,27 +2751,27 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46265</v>
+        <v>46252</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2813,7 +2785,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2825,12 +2797,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2848,7 +2820,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2858,21 +2830,21 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46266</v>
+        <v>46246</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46288</v>
+        <v>46272</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>70000</v>
+        <v>54000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N32" s="12" t="inlineStr">
@@ -2882,7 +2854,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -2894,22 +2866,22 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F33" s="21" t="n">
@@ -2917,7 +2889,7 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2927,17 +2899,17 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46275</v>
+        <v>46265</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2951,7 +2923,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -2963,12 +2935,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2982,30 +2954,32 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L34" s="15" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>70000</v>
+      </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3018,7 +2992,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3030,17 +3004,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3053,7 +3027,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3063,17 +3037,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46281</v>
+        <v>46275</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>110000</v>
+        <v>50000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3087,7 +3061,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3099,12 +3073,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3122,39 +3096,39 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46278</v>
+        <v>46275</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46295</v>
+        <v>46281</v>
       </c>
       <c r="L36" s="15" t="inlineStr"/>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3166,17 +3140,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3185,11 +3159,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3199,16 +3173,18 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46290</v>
+        <v>46281</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>110000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3221,7 +3197,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3233,12 +3209,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3252,11 +3228,11 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.335</v>
+        <v>0.4</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3266,21 +3242,21 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46293</v>
+        <v>46282</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46298</v>
+        <v>46286</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>21000</v>
+        <v>30000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3290,7 +3266,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3302,51 +3278,49 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46282</v>
+        <v>46290</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L39" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L39" s="23" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3359,7 +3333,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3371,12 +3345,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3386,15 +3360,15 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3404,31 +3378,29 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46293</v>
+        <v>46278</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L40" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L40" s="15" t="inlineStr"/>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3440,12 +3412,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3455,15 +3427,15 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3473,21 +3445,21 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46296</v>
+        <v>46293</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3497,7 +3469,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3509,12 +3481,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3524,7 +3496,7 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
@@ -3532,27 +3504,27 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46296</v>
+        <v>46293</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3566,7 +3538,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3578,12 +3550,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3601,7 +3573,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3611,17 +3583,17 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3635,7 +3607,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3716,12 +3688,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3739,7 +3711,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3749,17 +3721,17 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3773,7 +3745,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3785,12 +3757,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3804,11 +3776,11 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3818,7 +3790,7 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
@@ -3828,7 +3800,7 @@
         <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3842,7 +3814,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3854,12 +3826,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3873,21 +3845,21 @@
         </is>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
@@ -3897,7 +3869,7 @@
         <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>33000</v>
+        <v>60000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3911,7 +3883,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3923,12 +3895,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3942,11 +3914,11 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3966,7 +3938,7 @@
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>36000</v>
+        <v>33000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3980,7 +3952,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -3992,12 +3964,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -4011,31 +3983,31 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>70000</v>
+        <v>21000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4049,7 +4021,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4130,17 +4102,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4153,41 +4125,41 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46244</v>
+        <v>46297</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>350000</v>
+        <v>70000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4199,12 +4171,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4222,31 +4194,31 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>90000</v>
+        <v>36000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
@@ -4256,7 +4228,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4268,12 +4240,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4291,27 +4263,27 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46301</v>
+        <v>46244</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>600000</v>
+        <v>350000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4325,7 +4297,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4337,17 +4309,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4360,31 +4332,31 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46305</v>
+        <v>46311</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>62500</v>
+        <v>90000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4394,7 +4366,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4406,64 +4378,64 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.345</v>
+        <v>0.4</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46307</v>
+        <v>46315</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>27000</v>
+        <v>600000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4475,17 +4447,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4498,27 +4470,27 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>140000</v>
+        <v>62500</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
@@ -4532,7 +4504,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4544,64 +4516,64 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46322</v>
+        <v>46307</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>2778901.38</v>
+        <v>27000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
         </is>
       </c>
     </row>
@@ -4613,17 +4585,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4636,46 +4608,184 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="K58" s="14" t="n">
         <v>46307</v>
       </c>
       <c r="L58" s="15" t="n">
+        <v>140000</v>
+      </c>
+      <c r="M58" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N58" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O58" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F59" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J59" s="22" t="n">
+        <v>46303</v>
+      </c>
+      <c r="K59" s="22" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L59" s="23" t="n">
         <v>600000</v>
       </c>
-      <c r="M58" s="9" t="inlineStr">
+      <c r="M59" s="17" t="inlineStr">
         <is>
           <t>En presentación</t>
         </is>
       </c>
-      <c r="N58" s="12" t="inlineStr">
+      <c r="N59" s="20" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O58" s="16" t="inlineStr">
+      <c r="O59" s="24" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>Pesquisador Computacao</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>OEI/FPOS</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>Território Nacional</t>
+        </is>
+      </c>
+      <c r="J60" s="14" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K60" s="14" t="n">
+        <v>46322</v>
+      </c>
+      <c r="L60" s="15" t="n">
+        <v>2778901.38</v>
+      </c>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N60" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O60" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O58"/>
+  <autoFilter ref="A1:O60"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4734,6 +4844,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4782,7 +4894,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -4792,7 +4904,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -4834,7 +4946,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -4906,7 +5018,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -4916,7 +5028,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -4978,7 +5090,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -4988,7 +5100,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -4998,7 +5110,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -5034,7 +5146,7 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -5044,11 +5156,11 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5064,7 +5176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5110,7 +5222,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -5156,7 +5268,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
@@ -5166,25 +5278,15 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>OEI/FPOS</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5228,7 +5330,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5243,7 +5345,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5258,7 +5360,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5273,7 +5375,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-10 17:04
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 09/10/2026 às 18:00</t>
+          <t>Gerado em 10/10/2026 às 17:01</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>186276.3905263158</v>
+        <v>183581.1578378378</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>70000</v>
+        <v>62500</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1556,11 +1556,11 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146394</v>
+        <v>146401</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 30/2026 – Contratação de Consultoria Individual para realizar estudo de caso sobre a Secretaria de Serviços Compartilhados</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1578,27 +1578,27 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46289</v>
+        <v>46301</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46304</v>
+        <v>46316</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>90000</v>
+        <v>120000</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1623,11 +1623,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146401</v>
+        <v>146421</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1655,17 +1655,17 @@
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Híbrido</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46316</v>
+        <v>46313</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>cgti@mdh.gov.br</t>
+          <t>dga@mj.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1686,17 +1686,15 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>146422</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1706,59 +1704,69 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Híbrido</t>
+        </is>
+      </c>
       <c r="J14" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L14" s="15" t="inlineStr"/>
+        <v>46313</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <v>60000</v>
+      </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr">
+        <is>
+          <t>dga@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>146423</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
+          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
@@ -1771,48 +1779,56 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
+        <is>
+          <t>Híbrido</t>
+        </is>
+      </c>
       <c r="J15" s="22" t="n">
         <v>46304</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L15" s="23" t="inlineStr"/>
+        <v>46313</v>
+      </c>
+      <c r="L15" s="23" t="n">
+        <v>102000</v>
+      </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr">
+        <is>
+          <t>dga@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>146424</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
+          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1830,48 +1846,56 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Híbrido</t>
+        </is>
+      </c>
       <c r="J16" s="14" t="n">
         <v>46304</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L16" s="15" t="inlineStr"/>
+        <v>46313</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>60000</v>
+      </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>dga@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>146425</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
+          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1889,31 +1913,41 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Híbrido</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="n">
         <v>46304</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46310</v>
-      </c>
-      <c r="L17" s="23" t="inlineStr"/>
+        <v>46313</v>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>40000</v>
+      </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>dpagi@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1925,12 +1959,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1940,15 +1974,13 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1958,10 +1990,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1984,12 +2016,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:375ed309-bb72-44ae-7d86-08df1d6278dd</t>
+          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 41/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2007,7 +2039,7 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2017,10 +2049,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2043,12 +2075,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2058,13 +2090,15 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2074,10 +2108,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2100,12 +2134,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2123,7 +2157,7 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2133,10 +2167,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2159,12 +2193,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2174,13 +2208,15 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2190,10 +2226,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2216,12 +2252,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2273,12 +2309,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2288,13 +2324,15 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2330,12 +2368,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2351,7 +2389,7 @@
       <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2382,207 +2420,171 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr"/>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46251</v>
+        <v>46286</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L26" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr"/>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="inlineStr"/>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L27" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr"/>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L28" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr"/>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2596,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2613,33 +2615,35 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
         <v>46246</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L29" s="23" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L29" s="23" t="n">
+        <v>54000</v>
+      </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2649,7 +2653,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -2661,12 +2665,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2676,37 +2680,37 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46252</v>
-      </c>
-      <c r="L30" s="15" t="n">
-        <v>286000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2716,7 +2720,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2728,12 +2732,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2751,7 +2755,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2761,17 +2765,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2785,7 +2789,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -2797,12 +2801,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2820,7 +2824,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2830,21 +2834,21 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46272</v>
+        <v>46259</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N32" s="12" t="inlineStr">
@@ -2854,7 +2858,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2866,22 +2870,22 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F33" s="21" t="n">
@@ -2889,27 +2893,27 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46265</v>
+        <v>46251</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46270</v>
+        <v>46256</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2923,7 +2927,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2935,12 +2939,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2958,7 +2962,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2968,21 +2972,21 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46266</v>
+        <v>46246</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46288</v>
+        <v>46272</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>70000</v>
+        <v>54000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2992,7 +2996,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3004,22 +3008,22 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
@@ -3027,7 +3031,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3037,17 +3041,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46275</v>
+        <v>46265</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3061,7 +3065,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3073,12 +3077,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3092,30 +3096,32 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L36" s="15" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>70000</v>
+      </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3128,7 +3134,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3215,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3224,36 +3230,34 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46282</v>
+        <v>46275</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L38" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L38" s="15" t="inlineStr"/>
       <c r="M38" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3266,7 +3270,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3278,17 +3282,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3297,11 +3301,11 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3311,16 +3315,18 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46290</v>
+        <v>46275</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L39" s="23" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L39" s="23" t="n">
+        <v>50000</v>
+      </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3333,7 +3339,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3345,12 +3351,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3360,15 +3366,15 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3378,29 +3384,31 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46278</v>
+        <v>46282</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3412,54 +3420,52 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.335</v>
+        <v>0.3</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L41" s="23" t="n">
-        <v>21000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3469,7 +3475,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3481,12 +3487,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3496,15 +3502,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3514,31 +3520,29 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46293</v>
+        <v>46278</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3550,12 +3554,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3565,15 +3569,15 @@
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3583,21 +3587,21 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>55000</v>
+        <v>21000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3607,7 +3611,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3619,12 +3623,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3634,7 +3638,7 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
@@ -3642,31 +3646,31 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>600000</v>
+        <v>30000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3676,7 +3680,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3688,12 +3692,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3711,31 +3715,31 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>60000</v>
+        <v>600000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3745,7 +3749,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3757,12 +3761,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3780,27 +3784,27 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K46" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3814,7 +3818,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3826,12 +3830,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3849,7 +3853,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3859,14 +3863,14 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L47" s="23" t="n">
         <v>60000</v>
@@ -3883,7 +3887,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3895,12 +3899,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3914,11 +3918,11 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3928,7 +3932,7 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
@@ -3938,7 +3942,7 @@
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>33000</v>
+        <v>60000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3952,7 +3956,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3964,12 +3968,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3983,21 +3987,21 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
@@ -4007,7 +4011,7 @@
         <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4021,7 +4025,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4033,17 +4037,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4052,45 +4056,45 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>935000</v>
+        <v>21000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4102,17 +4106,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4125,41 +4129,41 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46311</v>
+        <v>46296</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>70000</v>
+        <v>935000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4240,17 +4244,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4259,45 +4263,45 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K53" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>350000</v>
+        <v>33000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4309,12 +4313,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4332,7 +4336,7 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4352,11 +4356,11 @@
         <v>46311</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>90000</v>
+        <v>70000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4366,7 +4370,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4378,12 +4382,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4401,27 +4405,27 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46301</v>
+        <v>46244</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>600000</v>
+        <v>350000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -4435,7 +4439,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4447,17 +4451,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4470,31 +4474,31 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46305</v>
+        <v>46311</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>62500</v>
+        <v>90000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -4504,7 +4508,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4516,30 +4520,30 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.345</v>
+        <v>0.4</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
@@ -4549,17 +4553,17 @@
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>27000</v>
+        <v>62500</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4573,7 +4577,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4585,17 +4589,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4608,41 +4612,41 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46307</v>
+        <v>46315</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>140000</v>
+        <v>600000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4654,22 +4658,22 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
@@ -4677,41 +4681,41 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46307</v>
+        <v>46322</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>600000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4723,69 +4727,207 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
         <v>46302</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46322</v>
+        <v>46307</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>2778901.38</v>
+        <v>27000</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F61" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+        </is>
+      </c>
+      <c r="J61" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K61" s="22" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L61" s="23" t="n">
+        <v>140000</v>
+      </c>
+      <c r="M61" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N61" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O61" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J62" s="14" t="n">
+        <v>46303</v>
+      </c>
+      <c r="K62" s="14" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L62" s="15" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M62" s="9" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N62" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O62" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O60"/>
+  <autoFilter ref="A1:O62"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4846,6 +4988,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4884,7 +5028,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -4894,7 +5038,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -4904,7 +5048,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -4946,7 +5090,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3">
@@ -4956,7 +5100,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -5028,7 +5172,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -5090,7 +5234,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -5100,7 +5244,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -5110,7 +5254,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -5130,7 +5274,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -5140,7 +5284,7 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -5202,7 +5346,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -5222,13 +5366,13 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
@@ -5238,17 +5382,17 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -5330,7 +5474,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5345,7 +5489,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5360,7 +5504,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5375,7 +5519,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-13 18:59
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 10/10/2026 às 17:01</t>
+          <t>Gerado em 13/10/2026 às 18:55</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>183581.1578378378</v>
+        <v>197696.8566666667</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>62500</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1954,22 +1954,20 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>146427</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1985,85 +1983,101 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>HOME OFFICE</t>
+        </is>
+      </c>
       <c r="J18" s="14" t="n">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L18" s="15" t="inlineStr"/>
+        <v>46316</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <v>208000</v>
+      </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>curriculos@consorcionordeste.gov.br</t>
+        </is>
+      </c>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n">
+        <v>146428</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>HOME OFFICE</t>
+        </is>
+      </c>
       <c r="J19" s="22" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46309</v>
-      </c>
-      <c r="L19" s="23" t="inlineStr"/>
+        <v>46316</v>
+      </c>
+      <c r="L19" s="23" t="n">
+        <v>28000</v>
+      </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr">
+        <is>
+          <t>curriculos@consorcionordeste.gov.br</t>
+        </is>
+      </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -2075,12 +2089,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
+          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
+          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2090,15 +2104,13 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2108,10 +2120,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46309</v>
+        <v>46313</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2134,12 +2146,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2149,15 +2161,13 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr"/>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2167,10 +2177,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2193,12 +2203,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
+          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2216,7 +2226,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2229,7 +2239,7 @@
         <v>46304</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2252,12 +2262,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2267,13 +2277,15 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2283,10 +2295,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2309,12 +2321,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2332,7 +2344,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2342,10 +2354,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2368,12 +2380,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2383,13 +2395,15 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2399,10 +2413,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2425,12 +2439,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2482,12 +2496,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2497,13 +2511,15 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2539,12 +2555,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2560,7 +2576,7 @@
       <c r="F28" s="13" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2591,205 +2607,171 @@
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="inlineStr"/>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L29" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr"/>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF | Híbrido</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46250</v>
+        <v>46316</v>
       </c>
       <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr"/>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr"/>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr"/>
       <c r="J31" s="22" t="n">
-        <v>46246</v>
+        <v>46286</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L31" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr"/>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2801,17 +2783,17 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2824,7 +2806,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2834,17 +2816,17 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2858,7 +2840,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2870,17 +2852,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2893,7 +2875,7 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2903,17 +2885,17 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2927,7 +2909,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3146,17 +3128,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3169,7 +3151,7 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3179,17 +3161,17 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46281</v>
+        <v>46275</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>110000</v>
+        <v>50000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3203,7 +3185,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3282,17 +3264,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3305,7 +3287,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3315,17 +3297,17 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46275</v>
+        <v>46281</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>50000</v>
+        <v>110000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3339,7 +3321,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -4037,12 +4019,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4056,7 +4038,7 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.33</v>
+        <v>0.347</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
@@ -4080,7 +4062,7 @@
         <v>46300</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>21000</v>
+        <v>33000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4094,7 +4076,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4106,17 +4088,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4125,45 +4107,45 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>935000</v>
+        <v>21000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4175,17 +4157,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4198,41 +4180,41 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K52" s="14" t="n">
         <v>46296</v>
       </c>
-      <c r="K52" s="14" t="n">
-        <v>46300</v>
-      </c>
       <c r="L52" s="15" t="n">
-        <v>36000</v>
+        <v>935000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4244,12 +4226,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4263,11 +4245,11 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -4287,7 +4269,7 @@
         <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>33000</v>
+        <v>36000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4301,7 +4283,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4520,17 +4502,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4543,41 +4525,41 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
         <v>46301</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46305</v>
+        <v>46315</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>62500</v>
+        <v>600000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4589,17 +4571,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4612,41 +4594,41 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
         <v>46301</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46315</v>
+        <v>46305</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>600000</v>
+        <v>62500</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4658,64 +4640,64 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46322</v>
+        <v>46307</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>2778901.38</v>
+        <v>27000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
         </is>
       </c>
     </row>
@@ -4727,64 +4709,64 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.345</v>
+        <v>0.4</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
         <v>46302</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46307</v>
+        <v>46322</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>27000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4926,8 +4908,77 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F63" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>OEI/SECULT</t>
+        </is>
+      </c>
+      <c r="I63" s="19" t="inlineStr">
+        <is>
+          <t>Vitória/ES.</t>
+        </is>
+      </c>
+      <c r="J63" s="22" t="n">
+        <v>46308</v>
+      </c>
+      <c r="K63" s="22" t="n">
+        <v>46321</v>
+      </c>
+      <c r="L63" s="23" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M63" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N63" s="20" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O63" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O62"/>
+  <autoFilter ref="A1:O63"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4990,6 +5041,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5028,7 +5080,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -5038,7 +5090,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -5048,7 +5100,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -5090,7 +5142,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -5100,7 +5152,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -5158,21 +5210,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -5182,7 +5234,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -5192,7 +5244,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5234,7 +5286,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -5244,7 +5296,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -5254,7 +5306,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -5274,7 +5326,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -5346,7 +5398,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -5356,7 +5408,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -5366,7 +5418,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -5376,7 +5428,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -5416,7 +5468,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -5474,7 +5526,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5489,7 +5541,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5504,7 +5556,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5519,7 +5571,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-14 16:44
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$65</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 13/10/2026 às 18:55</t>
+          <t>Gerado em 14/10/2026 às 16:36</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24">
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2089,12 +2089,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
+          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2104,13 +2104,15 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2120,10 +2122,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2146,12 +2148,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
+          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2161,13 +2163,15 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2177,10 +2181,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46303</v>
+        <v>46309</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2203,12 +2207,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
+          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
+          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2218,15 +2222,13 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2236,10 +2238,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46309</v>
+        <v>46313</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2262,12 +2264,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
+          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
+          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2277,15 +2279,13 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr"/>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K23" s="22" t="n">
         <v>46309</v>
@@ -2321,12 +2321,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
+          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2357,7 +2357,7 @@
         <v>46304</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2380,12 +2380,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
+          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2416,7 +2416,7 @@
         <v>46304</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2439,12 +2439,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2454,13 +2454,15 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2470,10 +2472,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2496,12 +2498,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2519,7 +2521,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2529,10 +2531,10 @@
       </c>
       <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46286</v>
+        <v>46304</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2555,12 +2557,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2576,7 +2578,7 @@
       <c r="F28" s="13" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2612,12 +2614,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2627,13 +2629,15 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2669,12 +2673,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2690,7 +2694,7 @@
       <c r="F30" s="13" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2726,12 +2730,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2778,138 +2782,114 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F32" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr"/>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46251</v>
+        <v>46286</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L32" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr"/>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="inlineStr"/>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I33" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="22" t="n">
-        <v>46252</v>
+        <v>46286</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>60000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N33" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr"/>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2921,17 +2901,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2944,7 +2924,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2954,21 +2934,21 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46272</v>
+        <v>46256</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2978,7 +2958,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2990,22 +2970,22 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
@@ -3013,27 +2993,27 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46265</v>
+        <v>46252</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3047,7 +3027,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3059,12 +3039,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3082,7 +3062,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3092,21 +3072,21 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46266</v>
+        <v>46246</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46288</v>
+        <v>46272</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>70000</v>
+        <v>54000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3116,7 +3096,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3128,22 +3108,22 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
@@ -3151,7 +3131,7 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3161,17 +3141,17 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46275</v>
+        <v>46265</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3185,7 +3165,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3197,12 +3177,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3216,30 +3196,32 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L38" s="15" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>70000</v>
+      </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3252,7 +3234,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3264,17 +3246,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3287,7 +3269,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3297,17 +3279,17 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46281</v>
+        <v>46275</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>110000</v>
+        <v>50000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3321,7 +3303,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3333,12 +3315,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3348,36 +3330,34 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46282</v>
+        <v>46275</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L40" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L40" s="15" t="inlineStr"/>
       <c r="M40" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3390,7 +3370,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3402,17 +3382,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3421,11 +3401,11 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3435,16 +3415,18 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46290</v>
+        <v>46281</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L41" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L41" s="23" t="n">
+        <v>110000</v>
+      </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3457,7 +3439,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3469,12 +3451,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3484,15 +3466,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3502,29 +3484,31 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46278</v>
+        <v>46282</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L42" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3536,54 +3520,52 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.335</v>
+        <v>0.3</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L43" s="23" t="n">
-        <v>21000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L43" s="23" t="inlineStr"/>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3593,7 +3575,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3605,12 +3587,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3620,15 +3602,15 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3638,31 +3620,29 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46293</v>
+        <v>46278</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L44" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L44" s="15" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3674,12 +3654,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3689,35 +3669,35 @@
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>600000</v>
+        <v>21000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3731,7 +3711,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3743,12 +3723,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3758,7 +3738,7 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
@@ -3766,7 +3746,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3776,17 +3756,17 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>55000</v>
+        <v>30000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3800,7 +3780,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3812,12 +3792,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3835,31 +3815,31 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>60000</v>
+        <v>600000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3869,7 +3849,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -3881,12 +3861,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3904,27 +3884,27 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K48" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3938,7 +3918,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3950,12 +3930,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3969,21 +3949,21 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
@@ -3993,7 +3973,7 @@
         <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>60000</v>
+        <v>33000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4007,7 +3987,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4019,12 +3999,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4038,31 +4018,31 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>33000</v>
+        <v>60000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4076,7 +4056,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -4088,12 +4068,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4107,21 +4087,21 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
@@ -4131,7 +4111,7 @@
         <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4145,7 +4125,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4157,17 +4137,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4180,41 +4160,41 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>935000</v>
+        <v>60000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -4226,12 +4206,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4245,11 +4225,11 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -4269,7 +4249,7 @@
         <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>36000</v>
+        <v>21000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4283,7 +4263,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4295,17 +4275,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4318,41 +4298,41 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46311</v>
+        <v>46296</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>70000</v>
+        <v>935000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4364,17 +4344,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4387,41 +4367,41 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K55" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>350000</v>
+        <v>36000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4433,12 +4413,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4456,7 +4436,7 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
@@ -4476,11 +4456,11 @@
         <v>46311</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>90000</v>
+        <v>70000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -4490,7 +4470,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4502,12 +4482,12 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -4525,27 +4505,27 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46301</v>
+        <v>46244</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>600000</v>
+        <v>350000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4559,7 +4539,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4571,17 +4551,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4594,31 +4574,31 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46305</v>
+        <v>46311</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>62500</v>
+        <v>90000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
@@ -4628,7 +4608,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4640,64 +4620,64 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.345</v>
+        <v>0.4</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46307</v>
+        <v>46315</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>27000</v>
+        <v>600000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4709,22 +4689,22 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
@@ -4732,41 +4712,41 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46322</v>
+        <v>46305</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>2778901.38</v>
+        <v>62500</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4778,22 +4758,22 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="F61" s="21" t="n">
@@ -4801,41 +4781,41 @@
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J61" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K61" s="22" t="n">
-        <v>46307</v>
+        <v>46322</v>
       </c>
       <c r="L61" s="23" t="n">
-        <v>140000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N61" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4847,17 +4827,17 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
@@ -4870,31 +4850,31 @@
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J62" s="14" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="K62" s="14" t="n">
         <v>46307</v>
       </c>
       <c r="L62" s="15" t="n">
-        <v>600000</v>
+        <v>140000</v>
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N62" s="12" t="inlineStr">
@@ -4904,7 +4884,7 @@
       </c>
       <c r="O62" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4916,69 +4896,207 @@
       </c>
       <c r="B63" s="18" t="inlineStr">
         <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F63" s="21" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I63" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J63" s="22" t="n">
+        <v>46302</v>
+      </c>
+      <c r="K63" s="22" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L63" s="23" t="n">
+        <v>27000</v>
+      </c>
+      <c r="M63" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N63" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O63" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E64" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G64" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H64" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I64" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J64" s="14" t="n">
+        <v>46303</v>
+      </c>
+      <c r="K64" s="14" t="n">
+        <v>46307</v>
+      </c>
+      <c r="L64" s="15" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M64" s="9" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N64" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O64" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
           <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
         </is>
       </c>
-      <c r="C63" s="19" t="inlineStr">
+      <c r="C65" s="19" t="inlineStr">
         <is>
           <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
         </is>
       </c>
-      <c r="D63" s="19" t="inlineStr">
+      <c r="D65" s="19" t="inlineStr">
         <is>
           <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
-      <c r="E63" s="20" t="inlineStr">
+      <c r="E65" s="20" t="inlineStr">
         <is>
           <t>Analista Powerbi</t>
         </is>
       </c>
-      <c r="F63" s="21" t="n">
+      <c r="F65" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="G63" s="19" t="inlineStr">
+      <c r="G65" s="19" t="inlineStr">
         <is>
           <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
-      <c r="H63" s="19" t="inlineStr">
+      <c r="H65" s="19" t="inlineStr">
         <is>
           <t>OEI/SECULT</t>
         </is>
       </c>
-      <c r="I63" s="19" t="inlineStr">
+      <c r="I65" s="19" t="inlineStr">
         <is>
           <t>Vitória/ES.</t>
         </is>
       </c>
-      <c r="J63" s="22" t="n">
+      <c r="J65" s="22" t="n">
         <v>46308</v>
       </c>
-      <c r="K63" s="22" t="n">
+      <c r="K65" s="22" t="n">
         <v>46321</v>
       </c>
-      <c r="L63" s="23" t="n">
+      <c r="L65" s="23" t="n">
         <v>600000</v>
       </c>
-      <c r="M63" s="17" t="inlineStr">
+      <c r="M65" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
         </is>
       </c>
-      <c r="N63" s="20" t="inlineStr">
+      <c r="N65" s="20" t="inlineStr">
         <is>
           <t>compras.bra@oei.int</t>
         </is>
       </c>
-      <c r="O63" s="24" t="inlineStr">
+      <c r="O65" s="24" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O63"/>
+  <autoFilter ref="A1:O65"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -5042,6 +5160,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5100,7 +5220,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -5142,7 +5262,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3">
@@ -5214,7 +5334,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -5286,7 +5406,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -5296,7 +5416,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -5306,7 +5426,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -5394,7 +5514,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5404,21 +5524,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -5526,7 +5646,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5541,7 +5661,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5556,7 +5676,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5571,7 +5691,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-15 16:27
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 14/10/2026 às 16:36</t>
+          <t>Gerado em 15/10/2026 às 16:22</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -886,11 +886,11 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146374</v>
+        <v>146334</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Consultoria individual para estudo sobre os impactos regulatórios da Reforma Tributária no setor de saneamento básico</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -908,27 +908,27 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>brasília</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46280</v>
+        <v>46310</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46310</v>
+        <v>46320</v>
       </c>
       <c r="L2" s="15" t="n">
-        <v>120000</v>
+        <v>53610.42</v>
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
@@ -937,7 +937,7 @@
       </c>
       <c r="N2" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>cotar@ssb.gov.br</t>
         </is>
       </c>
       <c r="O2" s="16" t="inlineStr">
@@ -953,11 +953,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146375</v>
+        <v>146374</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
@@ -1020,11 +1020,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146385</v>
+        <v>146375</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1047,22 +1047,22 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46289</v>
+        <v>46280</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1087,16 +1087,16 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146354</v>
+        <v>146385</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -1105,31 +1105,31 @@
         </is>
       </c>
       <c r="F5" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46293</v>
+        <v>46289</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46313</v>
+        <v>46311</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>93500</v>
+        <v>100000</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1154,16 +1154,16 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146382</v>
+        <v>146354</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1196,7 +1196,7 @@
         <v>46313</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>91500</v>
+        <v>93500</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146379</v>
+        <v>146382</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
@@ -1263,7 +1263,7 @@
         <v>46313</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>121500</v>
+        <v>91500</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1288,11 +1288,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146378</v>
+        <v>146379</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1355,11 +1355,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146377</v>
+        <v>146378</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1397,7 +1397,7 @@
         <v>46313</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>93500</v>
+        <v>121500</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1422,11 +1422,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146355</v>
+        <v>146377</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1489,11 +1489,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146376</v>
+        <v>146355</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1531,7 +1531,7 @@
         <v>46313</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>86800</v>
+        <v>93500</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146401</v>
+        <v>146376</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1574,31 +1574,31 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46301</v>
+        <v>46293</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46316</v>
+        <v>46313</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>120000</v>
+        <v>86800</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>cgti@mdh.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1623,11 +1623,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146421</v>
+        <v>146401</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1655,17 +1655,17 @@
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Híbrido</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>dga@mj.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1690,11 +1690,11 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146422</v>
+        <v>146421</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
+          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1732,7 +1732,7 @@
         <v>46313</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>60000</v>
+        <v>100000</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
@@ -1757,16 +1757,16 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>146423</v>
+        <v>146422</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
+          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
@@ -1799,7 +1799,7 @@
         <v>46313</v>
       </c>
       <c r="L15" s="23" t="n">
-        <v>102000</v>
+        <v>60000</v>
       </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
@@ -1824,16 +1824,16 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>146424</v>
+        <v>146423</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
+          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1866,7 +1866,7 @@
         <v>46313</v>
       </c>
       <c r="L16" s="15" t="n">
-        <v>60000</v>
+        <v>102000</v>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
@@ -1891,11 +1891,11 @@
         </is>
       </c>
       <c r="B17" s="18" t="n">
-        <v>146425</v>
+        <v>146424</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
+          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1933,7 +1933,7 @@
         <v>46313</v>
       </c>
       <c r="L17" s="23" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="N17" s="20" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>dga@mj.gov.br</t>
         </is>
       </c>
       <c r="O17" s="24" t="inlineStr">
@@ -1958,27 +1958,29 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>146427</v>
+        <v>146425</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
+          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1988,17 +1990,17 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t>Híbrido</t>
         </is>
       </c>
       <c r="J18" s="14" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46316</v>
+        <v>46313</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>208000</v>
+        <v>40000</v>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
@@ -2007,7 +2009,7 @@
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>dpagi@mj.gov.br</t>
         </is>
       </c>
       <c r="O18" s="16" t="inlineStr">
@@ -2023,11 +2025,11 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>146428</v>
+        <v>146427</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2063,7 +2065,7 @@
         <v>46316</v>
       </c>
       <c r="L19" s="23" t="n">
-        <v>28000</v>
+        <v>208000</v>
       </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
@@ -2084,59 +2086,65 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>146428</v>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>HOME OFFICE</t>
+        </is>
+      </c>
       <c r="J20" s="14" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46314</v>
-      </c>
-      <c r="L20" s="15" t="inlineStr"/>
+        <v>46316</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <v>28000</v>
+      </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>curriculos@consorcionordeste.gov.br</t>
+        </is>
+      </c>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -2148,12 +2156,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
+          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2171,7 +2179,7 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2184,7 +2192,7 @@
         <v>46309</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2207,12 +2215,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
+          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2222,13 +2230,15 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2238,10 +2248,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46313</v>
+        <v>46315</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2264,12 +2274,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:8e654be2-3b1f-4782-d2b4-08df1fb02468</t>
+          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 57/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2295,10 +2305,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46309</v>
+        <v>46313</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2321,12 +2331,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:d8649b2a-6267-450d-bf98-08df23ad085e</t>
+          <t>unesco:5e9b99bd-04d4-46aa-60df-08df20839863</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 56/2026 - Arquitetura e Urbanismo - Iphan-SP</t>
+          <t>A2101B5102 | Edital 01/2026 – 01 vaga - Consultor individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2344,7 +2354,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2354,10 +2364,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2380,12 +2390,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:ec3e284f-74b2-4ad2-bf99-08df23ad085e</t>
+          <t>unesco:4e03075d-fa9c-444b-bf96-08df23ad085e</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 57/2026 - Arquitetura e Urbanismo - Centro Vivo</t>
+          <t>570BRZ2005 - Edital 01/2026 - Consultor individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2395,15 +2405,13 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2413,10 +2421,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2901,17 +2909,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2924,7 +2932,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2934,17 +2942,17 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2958,7 +2966,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -2970,17 +2978,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -2993,7 +3001,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3003,17 +3011,17 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3027,7 +3035,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3039,22 +3047,22 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
@@ -3062,31 +3070,31 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3096,7 +3104,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3108,22 +3116,22 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
@@ -3131,31 +3139,31 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46270</v>
+        <v>46272</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>30000</v>
+        <v>54000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3165,7 +3173,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3177,12 +3185,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3200,27 +3208,27 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46266</v>
+        <v>46275</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46288</v>
+        <v>46280</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>70000</v>
+        <v>50000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3234,7 +3242,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3246,12 +3254,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3269,27 +3277,27 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46280</v>
+        <v>46288</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>50000</v>
+        <v>70000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3303,7 +3311,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3654,12 +3662,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3673,11 +3681,11 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.335</v>
+        <v>0.4</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3687,7 +3695,7 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
@@ -3697,11 +3705,11 @@
         <v>46298</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>21000</v>
+        <v>30000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3711,7 +3719,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3723,12 +3731,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3742,11 +3750,11 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3756,7 +3764,7 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
@@ -3766,11 +3774,11 @@
         <v>46298</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -3780,7 +3788,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3792,12 +3800,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3815,31 +3823,31 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
         <v>46294</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>600000</v>
+        <v>55000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3849,7 +3857,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3861,12 +3869,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3884,27 +3892,27 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K48" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3918,7 +3926,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3930,12 +3938,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3949,31 +3957,31 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>33000</v>
+        <v>60000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -3987,7 +3995,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3999,12 +4007,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4022,7 +4030,7 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -4032,14 +4040,14 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L50" s="15" t="n">
         <v>60000</v>
@@ -4056,7 +4064,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4068,12 +4076,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4087,21 +4095,21 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
@@ -4111,7 +4119,7 @@
         <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>60000</v>
+        <v>33000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4125,7 +4133,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4137,12 +4145,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4156,11 +4164,11 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
@@ -4170,7 +4178,7 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
@@ -4180,7 +4188,7 @@
         <v>46300</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4194,7 +4202,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4206,17 +4214,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4225,45 +4233,45 @@
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K53" s="22" t="n">
         <v>46296</v>
       </c>
-      <c r="K53" s="22" t="n">
-        <v>46300</v>
-      </c>
       <c r="L53" s="23" t="n">
-        <v>21000</v>
+        <v>935000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4275,17 +4283,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4298,41 +4306,41 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>935000</v>
+        <v>36000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4344,12 +4352,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4372,22 +4380,22 @@
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>36000</v>
+        <v>70000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -4401,7 +4409,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4413,17 +4421,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4436,41 +4444,41 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>70000</v>
+        <v>350000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4482,17 +4490,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4505,41 +4513,41 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46244</v>
+        <v>46297</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>350000</v>
+        <v>90000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4551,17 +4559,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4574,41 +4582,41 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>90000</v>
+        <v>600000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4620,17 +4628,17 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
@@ -4643,41 +4651,41 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
         <v>46301</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46315</v>
+        <v>46305</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>600000</v>
+        <v>62500</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4689,22 +4697,22 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
@@ -4712,41 +4720,41 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46305</v>
+        <v>46322</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>62500</v>
+        <v>2778901.38</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4758,22 +4766,22 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F61" s="21" t="n">
@@ -4781,41 +4789,41 @@
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J61" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K61" s="22" t="n">
-        <v>46322</v>
+        <v>46307</v>
       </c>
       <c r="L61" s="23" t="n">
-        <v>2778901.38</v>
+        <v>140000</v>
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N61" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4827,40 +4835,40 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J62" s="14" t="n">
@@ -4870,7 +4878,7 @@
         <v>46307</v>
       </c>
       <c r="L62" s="15" t="n">
-        <v>140000</v>
+        <v>27000</v>
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
@@ -4884,7 +4892,7 @@
       </c>
       <c r="O62" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
         </is>
       </c>
     </row>
@@ -4896,64 +4904,64 @@
       </c>
       <c r="B63" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
         </is>
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E63" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F63" s="21" t="n">
-        <v>0.345</v>
+        <v>0.4</v>
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H63" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I63" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória/ES.</t>
         </is>
       </c>
       <c r="J63" s="22" t="n">
-        <v>46302</v>
+        <v>46308</v>
       </c>
       <c r="K63" s="22" t="n">
-        <v>46307</v>
+        <v>46321</v>
       </c>
       <c r="L63" s="23" t="n">
-        <v>27000</v>
+        <v>600000</v>
       </c>
       <c r="M63" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N63" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O63" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4978,7 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
@@ -5005,7 +5013,7 @@
         <v>46303</v>
       </c>
       <c r="K64" s="14" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="L64" s="15" t="n">
         <v>600000</v>
@@ -5034,17 +5042,17 @@
       </c>
       <c r="B65" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E65" s="20" t="inlineStr">
@@ -5057,24 +5065,24 @@
       </c>
       <c r="G65" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H65" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I65" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES.</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J65" s="22" t="n">
-        <v>46308</v>
+        <v>46294</v>
       </c>
       <c r="K65" s="22" t="n">
-        <v>46321</v>
+        <v>46311</v>
       </c>
       <c r="L65" s="23" t="n">
         <v>600000</v>
@@ -5086,12 +5094,12 @@
       </c>
       <c r="N65" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O65" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -5210,7 +5218,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -5220,7 +5228,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -5406,7 +5414,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3">
@@ -5416,7 +5424,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -5426,7 +5434,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -5436,7 +5444,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -5466,7 +5474,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -5514,7 +5522,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5524,11 +5532,11 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -5548,7 +5556,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -5661,7 +5669,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5676,7 +5684,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-16 16:13
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 15/10/2026 às 16:22</t>
+          <t>Gerado em 16/10/2026 às 16:09</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>197696.8566666667</v>
+        <v>188660.18</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26">
@@ -953,11 +953,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146374</v>
+        <v>146385</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 27/2026 – Contratação de Consultoria Individual II - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Servidões de Passagem para Orlas e Praias</t>
+          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -980,22 +980,22 @@
       </c>
       <c r="H3" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Home-based</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46280</v>
+        <v>46289</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="L3" s="23" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="N3" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>prodocbra016@mj.gov.br</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1020,16 +1020,16 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146375</v>
+        <v>146354</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 28/2026 - Contratação de Consultoria Individual I - para produção de material técnico de apoio à elaboração de projetos de acessibilidade em praias – Manual de Acessibilidade em Orlas e Praias</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -1038,31 +1038,31 @@
         </is>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46280</v>
+        <v>46293</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>120000</v>
+        <v>93500</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1087,11 +1087,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146385</v>
+        <v>146382</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1105,31 +1105,31 @@
         </is>
       </c>
       <c r="F5" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>100000</v>
+        <v>91500</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1154,11 +1154,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146354</v>
+        <v>146379</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1196,7 +1196,7 @@
         <v>46313</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>93500</v>
+        <v>121500</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146382</v>
+        <v>146378</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
@@ -1263,7 +1263,7 @@
         <v>46313</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>91500</v>
+        <v>121500</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1288,11 +1288,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146379</v>
+        <v>146377</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1330,7 +1330,7 @@
         <v>46313</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>121500</v>
+        <v>93500</v>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
@@ -1355,11 +1355,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146378</v>
+        <v>146355</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1397,7 +1397,7 @@
         <v>46313</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>121500</v>
+        <v>93500</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1422,11 +1422,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146377</v>
+        <v>146376</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1464,7 +1464,7 @@
         <v>46313</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>93500</v>
+        <v>86800</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1489,16 +1489,16 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146355</v>
+        <v>146401</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
@@ -1507,31 +1507,31 @@
         </is>
       </c>
       <c r="F11" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>93500</v>
+        <v>120000</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146376</v>
+        <v>146421</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
@@ -1583,22 +1583,22 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Híbrido</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46293</v>
+        <v>46304</v>
       </c>
       <c r="K12" s="14" t="n">
         <v>46313</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>86800</v>
+        <v>100000</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>dga@mj.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1623,11 +1623,11 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146401</v>
+        <v>146422</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1655,17 +1655,17 @@
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Híbrido</t>
         </is>
       </c>
       <c r="J13" s="22" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46316</v>
+        <v>46313</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="N13" s="20" t="inlineStr">
         <is>
-          <t>cgti@mdh.gov.br</t>
+          <t>dga@mj.gov.br</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
@@ -1690,16 +1690,16 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146421</v>
+        <v>146423</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
+          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1732,7 +1732,7 @@
         <v>46313</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>100000</v>
+        <v>102000</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
@@ -1757,11 +1757,11 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>146422</v>
+        <v>146424</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
+          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1824,16 +1824,16 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>146423</v>
+        <v>146425</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
+          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -1866,7 +1866,7 @@
         <v>46313</v>
       </c>
       <c r="L16" s="15" t="n">
-        <v>102000</v>
+        <v>40000</v>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="N16" s="12" t="inlineStr">
         <is>
-          <t>dga@mj.gov.br</t>
+          <t>dpagi@mj.gov.br</t>
         </is>
       </c>
       <c r="O16" s="16" t="inlineStr">
@@ -1891,29 +1891,27 @@
         </is>
       </c>
       <c r="B17" s="18" t="n">
-        <v>146424</v>
+        <v>146427</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr"/>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1923,17 +1921,17 @@
       </c>
       <c r="I17" s="19" t="inlineStr">
         <is>
-          <t>Híbrido</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J17" s="22" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L17" s="23" t="n">
-        <v>60000</v>
+        <v>208000</v>
       </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
@@ -1942,7 +1940,7 @@
       </c>
       <c r="N17" s="20" t="inlineStr">
         <is>
-          <t>dga@mj.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O17" s="24" t="inlineStr">
@@ -1958,29 +1956,27 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>146425</v>
+        <v>146428</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1990,17 +1986,17 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>Híbrido</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J18" s="14" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>40000</v>
+        <v>28000</v>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
@@ -2009,7 +2005,7 @@
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O18" s="16" t="inlineStr">
@@ -2025,47 +2021,49 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>146427</v>
+        <v>146419</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
+          <t>UNDP-BR/25/024 - Edital nº 9/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização dos instrumentos coletivos de trabalho registrados no Sistema Mediador nas ações ajuizadas nos anos de 2023, 2024 e 2025.</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t xml:space="preserve">Híbrido, com eventuais reuniões presenciais em Brasília/DF </t>
         </is>
       </c>
       <c r="J19" s="22" t="n">
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="L19" s="23" t="n">
-        <v>208000</v>
+        <v>116812.8</v>
       </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
@@ -2074,7 +2072,7 @@
       </c>
       <c r="N19" s="20" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>processoseletivosrt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O19" s="24" t="inlineStr">
@@ -2090,47 +2088,49 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>146428</v>
+        <v>146420</v>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
+          <t>PNUD BRA/25/024 - Edital nº 10/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização e da atuação jurídica governamental federal nas ações judiciais ajuizadas nos anos de 2024 e 2025 relacionadas a pedidos de registro de entidades sindicais e aos respectivos processos administrativos.</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
         </is>
       </c>
       <c r="J20" s="14" t="n">
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="L20" s="15" t="n">
-        <v>28000</v>
+        <v>116812.8</v>
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="N20" s="12" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>processoseletivosrt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O20" s="16" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:fb72c64e-511e-4325-60e3-08df20839863</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 05/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2462,15 +2462,13 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr"/>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2480,10 +2478,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46304</v>
+        <v>46286</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2506,12 +2504,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:df21a7d3-d7d5-44ad-60e4-08df20839863</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 06/2026 - 01 vaga - Consultor Individual</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2529,7 +2527,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2539,10 +2537,10 @@
       </c>
       <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46304</v>
+        <v>46286</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2565,12 +2563,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2586,7 +2584,7 @@
       <c r="F28" s="13" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2622,12 +2620,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2637,15 +2635,13 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="inlineStr"/>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2681,12 +2677,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2702,7 +2698,7 @@
       <c r="F30" s="13" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2738,12 +2734,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2790,114 +2786,138 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F32" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
       <c r="J32" s="14" t="n">
-        <v>46286</v>
+        <v>46252</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L32" s="15" t="inlineStr"/>
+        <v>46259</v>
+      </c>
+      <c r="L32" s="15" t="n">
+        <v>60000</v>
+      </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I33" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr">
+        <is>
+          <t>Recife - PE</t>
+        </is>
+      </c>
       <c r="J33" s="22" t="n">
-        <v>46286</v>
+        <v>46251</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46256</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>50000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N33" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -2909,12 +2929,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2928,32 +2948,30 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46252</v>
+        <v>46275</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L34" s="15" t="n">
-        <v>60000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2966,7 +2984,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -2978,17 +2996,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3001,7 +3019,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3011,21 +3029,21 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46256</v>
+        <v>46272</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3035,7 +3053,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3047,22 +3065,22 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
@@ -3070,7 +3088,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3080,17 +3098,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46265</v>
+        <v>46275</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46270</v>
+        <v>46280</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3104,7 +3122,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3116,22 +3134,22 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
@@ -3139,31 +3157,31 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3173,7 +3191,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3185,12 +3203,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3208,27 +3226,27 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46280</v>
+        <v>46288</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>50000</v>
+        <v>70000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3242,7 +3260,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -3254,17 +3272,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3277,27 +3295,27 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>70000</v>
+        <v>110000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3311,7 +3329,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3323,12 +3341,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3338,34 +3356,36 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3378,7 +3398,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3410,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3409,11 +3429,11 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3423,18 +3443,16 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46281</v>
+        <v>46290</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L41" s="23" t="n">
-        <v>110000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3447,7 +3465,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3459,12 +3477,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3474,15 +3492,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3492,31 +3510,29 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46282</v>
+        <v>46278</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3528,52 +3544,54 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.3</v>
+        <v>0.335</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L43" s="23" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L43" s="23" t="n">
+        <v>21000</v>
+      </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3583,7 +3601,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3595,12 +3613,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3614,11 +3632,11 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3628,29 +3646,31 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46278</v>
+        <v>46294</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L44" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L44" s="15" t="n">
+        <v>55000</v>
+      </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3731,12 +3751,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3746,15 +3766,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.335</v>
+        <v>0.4</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3764,21 +3784,21 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46298</v>
+        <v>46302</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -3788,7 +3808,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3800,17 +3820,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3823,41 +3843,41 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46294</v>
+        <v>46244</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46300</v>
+        <v>46296</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>55000</v>
+        <v>935000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3869,12 +3889,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3888,11 +3908,11 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3902,7 +3922,7 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
@@ -3912,7 +3932,7 @@
         <v>46300</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3926,7 +3946,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -3938,12 +3958,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3957,31 +3977,31 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>60000</v>
+        <v>33000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -3995,7 +4015,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -4007,12 +4027,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4030,17 +4050,17 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
@@ -4064,7 +4084,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -4076,12 +4096,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4095,11 +4115,11 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -4119,7 +4139,7 @@
         <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>33000</v>
+        <v>36000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4133,7 +4153,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -4145,12 +4165,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4164,21 +4184,21 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
@@ -4188,7 +4208,7 @@
         <v>46300</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4202,7 +4222,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -4214,17 +4234,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4237,41 +4257,41 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46244</v>
+        <v>46297</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46296</v>
+        <v>46311</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>935000</v>
+        <v>70000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4283,12 +4303,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4306,31 +4326,31 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>36000</v>
+        <v>90000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4340,7 +4360,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -4352,17 +4372,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4375,41 +4395,41 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>70000</v>
+        <v>600000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4490,12 +4510,12 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -4505,39 +4525,39 @@
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46297</v>
+        <v>46302</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>90000</v>
+        <v>27000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
@@ -4547,7 +4567,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
         </is>
       </c>
     </row>
@@ -4559,17 +4579,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4582,41 +4602,41 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="L58" s="15" t="n">
         <v>600000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
         </is>
       </c>
     </row>
@@ -4835,64 +4855,64 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.345</v>
+        <v>0.4</v>
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória/ES.</t>
         </is>
       </c>
       <c r="J62" s="14" t="n">
-        <v>46302</v>
+        <v>46308</v>
       </c>
       <c r="K62" s="14" t="n">
-        <v>46307</v>
+        <v>46321</v>
       </c>
       <c r="L62" s="15" t="n">
-        <v>27000</v>
+        <v>600000</v>
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N62" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O62" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4904,47 +4924,47 @@
       </c>
       <c r="B63" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327</t>
         </is>
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13327</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E63" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F63" s="21" t="n">
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H63" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I63" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES.</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="J63" s="22" t="n">
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="K63" s="22" t="n">
-        <v>46321</v>
+        <v>46315</v>
       </c>
       <c r="L63" s="23" t="n">
         <v>600000</v>
@@ -4956,12 +4976,12 @@
       </c>
       <c r="N63" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O63" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327/</t>
         </is>
       </c>
     </row>
@@ -4973,12 +4993,12 @@
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13326</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
@@ -4988,15 +5008,15 @@
       </c>
       <c r="E64" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G64" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H64" s="11" t="inlineStr">
@@ -5006,21 +5026,21 @@
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Salvador - BA</t>
         </is>
       </c>
       <c r="J64" s="14" t="n">
-        <v>46303</v>
+        <v>46311</v>
       </c>
       <c r="K64" s="14" t="n">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="L64" s="15" t="n">
         <v>600000</v>
       </c>
       <c r="M64" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N64" s="12" t="inlineStr">
@@ -5030,7 +5050,7 @@
       </c>
       <c r="O64" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326/</t>
         </is>
       </c>
     </row>
@@ -5208,7 +5228,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -5228,7 +5248,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -5270,7 +5290,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -5290,7 +5310,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -5342,7 +5362,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -5352,7 +5372,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -5434,7 +5454,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -5464,7 +5484,7 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -5522,31 +5542,31 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -5572,7 +5592,7 @@
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -5669,7 +5689,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5684,7 +5704,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-17 15:08
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$64</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 16/10/2026 às 16:09</t>
+          <t>Gerado em 17/10/2026 às 15:00</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>188660.18</v>
+        <v>192407.7524324324</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O65"/>
+  <dimension ref="A1:O64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -953,16 +953,16 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146385</v>
+        <v>146354</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor para elaborar o Caderno Temático de Referência: Investigação de Crimes contra Jornalistas e Comunicadores</t>
+          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E3" s="20" t="inlineStr">
@@ -971,31 +971,31 @@
         </is>
       </c>
       <c r="F3" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G3" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H3" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Home-based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46289</v>
+        <v>46293</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
       <c r="L3" s="23" t="n">
-        <v>100000</v>
+        <v>93500</v>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="N3" s="20" t="inlineStr">
         <is>
-          <t>prodocbra016@mj.gov.br</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1020,16 +1020,16 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146354</v>
+        <v>146382</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
@@ -1062,7 +1062,7 @@
         <v>46313</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>93500</v>
+        <v>91500</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1087,16 +1087,16 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146382</v>
+        <v>146379</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
@@ -1129,7 +1129,7 @@
         <v>46313</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>91500</v>
+        <v>121500</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1154,11 +1154,11 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146379</v>
+        <v>146378</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1221,11 +1221,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146378</v>
+        <v>146377</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1263,7 +1263,7 @@
         <v>46313</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>121500</v>
+        <v>93500</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1288,11 +1288,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146377</v>
+        <v>146355</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1355,11 +1355,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146355</v>
+        <v>146376</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1397,7 +1397,7 @@
         <v>46313</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>93500</v>
+        <v>86800</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1422,16 +1422,16 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146376</v>
+        <v>146401</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -1440,31 +1440,31 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>86800</v>
+        <v>120000</v>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr">
@@ -1489,11 +1489,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146401</v>
+        <v>146421</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Híbrido</t>
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46316</v>
+        <v>46313</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>cgti@mdh.gov.br</t>
+          <t>dga@mj.gov.br</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
@@ -1556,11 +1556,11 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146421</v>
+        <v>146422</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
+          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -1598,7 +1598,7 @@
         <v>46313</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>100000</v>
+        <v>60000</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1623,16 +1623,16 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>146422</v>
+        <v>146423</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
+          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
@@ -1665,7 +1665,7 @@
         <v>46313</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>60000</v>
+        <v>102000</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -1690,16 +1690,16 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>146423</v>
+        <v>146424</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
+          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1732,7 +1732,7 @@
         <v>46313</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>102000</v>
+        <v>60000</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
@@ -1757,11 +1757,11 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>146424</v>
+        <v>146425</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
+          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1799,7 +1799,7 @@
         <v>46313</v>
       </c>
       <c r="L15" s="23" t="n">
-        <v>60000</v>
+        <v>40000</v>
       </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="N15" s="20" t="inlineStr">
         <is>
-          <t>dga@mj.gov.br</t>
+          <t>dpagi@mj.gov.br</t>
         </is>
       </c>
       <c r="O15" s="24" t="inlineStr">
@@ -1824,29 +1824,27 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>146425</v>
+        <v>146427</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr"/>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1856,17 +1854,17 @@
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Híbrido</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J16" s="14" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L16" s="15" t="n">
-        <v>40000</v>
+        <v>208000</v>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
@@ -1875,7 +1873,7 @@
       </c>
       <c r="N16" s="12" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O16" s="16" t="inlineStr">
@@ -1891,11 +1889,11 @@
         </is>
       </c>
       <c r="B17" s="18" t="n">
-        <v>146427</v>
+        <v>146428</v>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1931,7 +1929,7 @@
         <v>46316</v>
       </c>
       <c r="L17" s="23" t="n">
-        <v>208000</v>
+        <v>28000</v>
       </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
@@ -1956,47 +1954,49 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>146428</v>
+        <v>146419</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
+          <t>UNDP-BR/25/024 - Edital nº 9/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização dos instrumentos coletivos de trabalho registrados no Sistema Mediador nas ações ajuizadas nos anos de 2023, 2024 e 2025.</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t xml:space="preserve">Híbrido, com eventuais reuniões presenciais em Brasília/DF </t>
         </is>
       </c>
       <c r="J18" s="14" t="n">
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>28000</v>
+        <v>116812.8</v>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>processoseletivosrt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O18" s="16" t="inlineStr">
@@ -2021,11 +2021,11 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>146419</v>
+        <v>146420</v>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>UNDP-BR/25/024 - Edital nº 9/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização dos instrumentos coletivos de trabalho registrados no Sistema Mediador nas ações ajuizadas nos anos de 2023, 2024 e 2025.</t>
+          <t>PNUD BRA/25/024 - Edital nº 10/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização e da atuação jurídica governamental federal nas ações judiciais ajuizadas nos anos de 2024 e 2025 relacionadas a pedidos de registro de entidades sindicais e aos respectivos processos administrativos.</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Híbrido, com eventuais reuniões presenciais em Brasília/DF </t>
+          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
         </is>
       </c>
       <c r="J19" s="22" t="n">
@@ -2084,15 +2084,17 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="n">
-        <v>146420</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
+        </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 10/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização e da atuação jurídica governamental federal nas ações judiciais ajuizadas nos anos de 2024 e 2025 relacionadas a pedidos de registro de entidades sindicais e aos respectivos processos administrativos.</t>
+          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2110,41 +2112,31 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46322</v>
-      </c>
-      <c r="L20" s="15" t="n">
-        <v>116812.8</v>
-      </c>
+        <v>46314</v>
+      </c>
+      <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr">
-        <is>
-          <t>processoseletivosrt@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr"/>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2156,12 +2148,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
+          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2179,7 +2171,7 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2192,7 +2184,7 @@
         <v>46309</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2215,12 +2207,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
+          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2230,15 +2222,13 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2248,10 +2238,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46315</v>
+        <v>46313</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2274,12 +2264,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
+          <t>unesco:0f405e12-70d9-40e9-ff3b-08df246fb477</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1156 - Edital 09/2026 - Consultor Individual - 01 vaga</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2305,10 +2295,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46313</v>
+        <v>46320</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2860,17 +2850,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2883,7 +2873,7 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2893,21 +2883,21 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46256</v>
+        <v>46272</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2917,7 +2907,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -2929,12 +2919,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2948,30 +2938,32 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L34" s="15" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>70000</v>
+      </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2984,7 +2976,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -2996,22 +2988,22 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
@@ -3019,31 +3011,31 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3053,7 +3045,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3134,30 +3126,30 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3167,18 +3159,16 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46265</v>
+        <v>46275</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3191,7 +3181,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -3203,17 +3193,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3226,27 +3216,27 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>70000</v>
+        <v>110000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3260,7 +3250,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -3272,22 +3262,22 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
@@ -3295,27 +3285,27 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="K39" s="22" t="n">
         <v>46286</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>110000</v>
+        <v>30000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3329,7 +3319,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -3341,51 +3331,49 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46282</v>
+        <v>46290</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L40" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L40" s="15" t="inlineStr"/>
       <c r="M40" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3398,7 +3386,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3410,17 +3398,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3433,39 +3421,39 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46290</v>
+        <v>46278</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3477,12 +3465,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3492,15 +3480,15 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3510,29 +3498,31 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46278</v>
+        <v>46293</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L42" s="15" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3682,12 +3672,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3697,7 +3687,7 @@
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
@@ -3705,7 +3695,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3715,17 +3705,17 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46298</v>
+        <v>46302</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3739,7 +3729,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3751,12 +3741,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3774,7 +3764,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3784,14 +3774,14 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
         <v>60000</v>
@@ -3808,7 +3798,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3820,17 +3810,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3843,41 +3833,41 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>935000</v>
+        <v>60000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3889,17 +3879,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3908,45 +3898,45 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K48" s="14" t="n">
         <v>46296</v>
       </c>
-      <c r="K48" s="14" t="n">
-        <v>46300</v>
-      </c>
       <c r="L48" s="15" t="n">
-        <v>21000</v>
+        <v>935000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4027,12 +4017,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4046,11 +4036,11 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -4060,7 +4050,7 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
@@ -4070,7 +4060,7 @@
         <v>46300</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>60000</v>
+        <v>21000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4084,7 +4074,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -4165,12 +4155,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4188,7 +4178,7 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
@@ -4198,17 +4188,17 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>60000</v>
+        <v>70000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4222,7 +4212,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -4234,17 +4224,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4257,41 +4247,41 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>70000</v>
+        <v>350000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4372,12 +4362,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4387,7 +4377,7 @@
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
@@ -4395,27 +4385,27 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>600000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -4429,7 +4419,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4441,12 +4431,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4464,27 +4454,27 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46244</v>
+        <v>46301</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46300</v>
+        <v>46315</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>350000</v>
+        <v>600000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
@@ -4498,7 +4488,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -4510,30 +4500,30 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
-        <v>0.345</v>
+        <v>0.4</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
@@ -4543,17 +4533,17 @@
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>27000</v>
+        <v>62500</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4567,7 +4557,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4579,17 +4569,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4602,31 +4592,31 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>600000</v>
+        <v>140000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
@@ -4636,7 +4626,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4648,30 +4638,30 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
-        <v>0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
@@ -4681,17 +4671,17 @@
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>62500</v>
+        <v>27000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
@@ -4705,7 +4695,7 @@
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
         </is>
       </c>
     </row>
@@ -4717,12 +4707,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -4732,7 +4722,7 @@
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F60" s="13" t="n">
@@ -4740,27 +4730,27 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Vitória/ES.</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46302</v>
+        <v>46308</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>2778901.38</v>
+        <v>600000</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
@@ -4774,7 +4764,7 @@
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4786,17 +4776,17 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E61" s="20" t="inlineStr">
@@ -4809,31 +4799,31 @@
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J61" s="22" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="K61" s="22" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="L61" s="23" t="n">
-        <v>140000</v>
+        <v>600000</v>
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N61" s="20" t="inlineStr">
@@ -4843,7 +4833,7 @@
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
         </is>
       </c>
     </row>
@@ -4855,17 +4845,17 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
@@ -4878,24 +4868,24 @@
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Vitória/ES.</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J62" s="14" t="n">
-        <v>46308</v>
+        <v>46294</v>
       </c>
       <c r="K62" s="14" t="n">
-        <v>46321</v>
+        <v>46311</v>
       </c>
       <c r="L62" s="15" t="n">
         <v>600000</v>
@@ -4907,12 +4897,12 @@
       </c>
       <c r="N62" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O62" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -4924,12 +4914,12 @@
       </c>
       <c r="B63" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326</t>
         </is>
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13327</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13326</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
@@ -4943,7 +4933,7 @@
         </is>
       </c>
       <c r="F63" s="21" t="n">
-        <v>0.34</v>
+        <v>0.347</v>
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
@@ -4957,7 +4947,7 @@
       </c>
       <c r="I63" s="19" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Salvador - BA</t>
         </is>
       </c>
       <c r="J63" s="22" t="n">
@@ -4981,7 +4971,7 @@
       </c>
       <c r="O63" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326/</t>
         </is>
       </c>
     </row>
@@ -4993,12 +4983,12 @@
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13326</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13327</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
@@ -5012,7 +5002,7 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.347</v>
+        <v>0.34</v>
       </c>
       <c r="G64" s="11" t="inlineStr">
         <is>
@@ -5026,7 +5016,7 @@
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>Salvador - BA</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="J64" s="14" t="n">
@@ -5050,81 +5040,12 @@
       </c>
       <c r="O64" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326/</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B65" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
-        </is>
-      </c>
-      <c r="C65" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
-        </is>
-      </c>
-      <c r="D65" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E65" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F65" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G65" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H65" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I65" s="19" t="inlineStr">
-        <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
-        </is>
-      </c>
-      <c r="J65" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="K65" s="22" t="n">
-        <v>46311</v>
-      </c>
-      <c r="L65" s="23" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M65" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N65" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O65" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O65"/>
+  <autoFilter ref="A1:O64"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -5189,7 +5110,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5228,7 +5148,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -5238,7 +5158,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -5248,7 +5168,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -5290,7 +5210,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -5300,7 +5220,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -5382,7 +5302,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -5434,7 +5354,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -5444,7 +5364,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -5454,7 +5374,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -5474,7 +5394,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -5484,7 +5404,7 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -5556,7 +5476,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -5566,7 +5486,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -5576,7 +5496,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -5674,7 +5594,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5689,7 +5609,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5704,7 +5624,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5719,7 +5639,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-19 18:29
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$55</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 17/10/2026 às 15:00</t>
+          <t>Gerado em 19/10/2026 às 18:23</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>63</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -638,27 +638,27 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>192407.7524324324</v>
+        <v>213242.8946666667</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>70000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -953,16 +953,16 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146354</v>
+        <v>146401</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 88/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA PROPOSIÇÃO DE SOLUÇÕES DE CIÊNCIA DE DADOS EM SENSORIAMENTO REMOTO.</t>
+          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E3" s="20" t="inlineStr">
@@ -971,31 +971,31 @@
         </is>
       </c>
       <c r="F3" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G3" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H3" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L3" s="23" t="n">
-        <v>93500</v>
+        <v>120000</v>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="N3" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>cgti@mdh.gov.br</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1020,49 +1020,47 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146382</v>
+        <v>146427</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 140/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA A AVALIAÇÃO DA OPERAÇÕES CENSITÁRIAS EM TERRAS INDÍGENAS DE RORAIMA.</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr"/>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>91500</v>
+        <v>208000</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1071,7 +1069,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1087,11 +1085,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146379</v>
+        <v>146428</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 132/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ANÁLISE DOS MÉTODOS DE ROTEAMENTO PARA OPERAÇÕES DE PESQUISA EM CAMPO.</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1101,35 +1099,33 @@
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F5" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr"/>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>121500</v>
+        <v>28000</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1138,7 +1134,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1154,16 +1150,16 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146378</v>
+        <v>146434</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 131/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE GEOPROCESSAMENTO.</t>
+          <t>Edital 07/2026 - Curso “Direito à Identidade, Cidadania e Documentação" para a Plataforma EV.G/Enap.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1176,27 +1172,27 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46293</v>
+        <v>46314</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46313</v>
+        <v>46330</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>121500</v>
+        <v>40000</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1205,7 +1201,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>rcn_cidadania@mdh.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1221,16 +1217,16 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146377</v>
+        <v>146419</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 130/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA O DESENVOLVIMENTO DE PROPOSTA DE SOLUÇÕES DE CIÊNCIA DE DADOS E SENSORIAMENTO REMOTO.</t>
+          <t>UNDP-BR/25/024 - Edital nº 9/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização dos instrumentos coletivos de trabalho registrados no Sistema Mediador nas ações ajuizadas nos anos de 2023, 2024 e 2025.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -1239,31 +1235,31 @@
         </is>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t xml:space="preserve">Híbrido, com eventuais reuniões presenciais em Brasília/DF </t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46293</v>
+        <v>46311</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46313</v>
+        <v>46322</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>93500</v>
+        <v>116812.8</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1272,7 +1268,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>processoseletivosrt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1288,16 +1284,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146355</v>
+        <v>146420</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 119/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA DESENVOLVIMENTO DE PROPOSTA DE APRIMORAMENTO DO SISTEMA INTEGRADO DE PESQUISAS DOMICILIARES.</t>
+          <t>PNUD BRA/25/024 - Edital nº 10/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização e da atuação jurídica governamental federal nas ações judiciais ajuizadas nos anos de 2024 e 2025 relacionadas a pedidos de registro de entidades sindicais e aos respectivos processos administrativos.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -1306,31 +1302,31 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46293</v>
+        <v>46311</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46313</v>
+        <v>46322</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>93500</v>
+        <v>116812.8</v>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
@@ -1339,7 +1335,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>processoseletivosrt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1351,20 +1347,22 @@
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="n">
-        <v>146376</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>unesco:8e0c9386-3ad1-41de-cc73-08df25fc88d5</t>
+        </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 116/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA MAPEAMENTO DE INOVAÇÕES NO PROCESSO DE PRODUÇÃO ESTATÍSTICA.</t>
+          <t>UNESCO 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
@@ -1373,60 +1371,52 @@
         </is>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="I9" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr"/>
       <c r="J9" s="22" t="n">
-        <v>46293</v>
+        <v>46314</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46313</v>
-      </c>
-      <c r="L9" s="23" t="n">
-        <v>86800</v>
-      </c>
+        <v>46320</v>
+      </c>
+      <c r="L9" s="23" t="inlineStr"/>
       <c r="M9" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N9" s="20" t="inlineStr">
-        <is>
-          <t>projetos.especiais@ibge.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N9" s="20" t="inlineStr"/>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="n">
-        <v>146401</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
+        </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Edital 06/2026 - Programa de Privacidade e Segurança da Informação</t>
+          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1444,56 +1434,48 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I10" s="11" t="inlineStr">
-        <is>
-          <t>Território Nacional</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr"/>
       <c r="J10" s="14" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L10" s="15" t="n">
-        <v>120000</v>
-      </c>
+        <v>46314</v>
+      </c>
+      <c r="L10" s="15" t="inlineStr"/>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N10" s="12" t="inlineStr">
-        <is>
-          <t>cgti@mdh.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N10" s="12" t="inlineStr"/>
       <c r="O10" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="n">
-        <v>146421</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
+        </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Edital 9/2026 - Levantamento SIGAP - SENAD/MJSP</t>
+          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1511,56 +1493,48 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I11" s="19" t="inlineStr">
-        <is>
-          <t>Híbrido</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="inlineStr"/>
       <c r="J11" s="22" t="n">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46313</v>
-      </c>
-      <c r="L11" s="23" t="n">
-        <v>100000</v>
-      </c>
+        <v>46315</v>
+      </c>
+      <c r="L11" s="23" t="inlineStr"/>
       <c r="M11" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N11" s="20" t="inlineStr">
-        <is>
-          <t>dga@mj.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N11" s="20" t="inlineStr"/>
       <c r="O11" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="n">
-        <v>146422</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>unesco:0f405e12-70d9-40e9-ff3b-08df246fb477</t>
+        </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Edital 10/2026 - Reformulação painéis POWER BI</t>
+          <t>914BRZ1156 - Edital 09/2026 - Consultor Individual - 01 vaga</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1570,69 +1544,59 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr"/>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>Híbrido</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="14" t="n">
-        <v>46304</v>
+        <v>46311</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46313</v>
-      </c>
-      <c r="L12" s="15" t="n">
-        <v>60000</v>
-      </c>
+        <v>46320</v>
+      </c>
+      <c r="L12" s="15" t="inlineStr"/>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N12" s="12" t="inlineStr">
-        <is>
-          <t>dga@mj.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr"/>
       <c r="O12" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="n">
-        <v>146423</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>unesco:5e9b99bd-04d4-46aa-60df-08df20839863</t>
+        </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>EDITAL 11/2026 - Padrões decisões judiciais destinação bens FUNAD</t>
+          <t>A2101B5102 | Edital 01/2026 – 01 vaga - Consultor individual</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
@@ -1645,56 +1609,48 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="inlineStr">
-        <is>
-          <t>Híbrido</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46313</v>
-      </c>
-      <c r="L13" s="23" t="n">
-        <v>102000</v>
-      </c>
+        <v>46317</v>
+      </c>
+      <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr">
-        <is>
-          <t>dga@mj.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr"/>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>146424</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>unesco:4e03075d-fa9c-444b-bf96-08df23ad085e</t>
+        </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>EDITAL 12/2026 - DIAGNÓSTICO COMPARADO RELACIONADO À DESTINAÇÃO DE BENS FUNAD</t>
+          <t>570BRZ2005 - Edital 01/2026 - Consultor individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1704,64 +1660,54 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr"/>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>Híbrido</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46313</v>
-      </c>
-      <c r="L14" s="15" t="n">
-        <v>60000</v>
-      </c>
+        <v>46315</v>
+      </c>
+      <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr">
-        <is>
-          <t>dga@mj.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr"/>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="n">
-        <v>146425</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>unesco:bb750b64-4229-4e0c-7b7f-08df26180ec9</t>
+        </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>EDITAL 13/2026 - Metodologia realização do Levantamento Nacional de Álcool e Drogas (LENAD)</t>
+          <t>570BRZ3012 - Edital 01/2026 - Consultor individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1779,126 +1725,112 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr">
-        <is>
-          <t>Híbrido</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46304</v>
+        <v>46314</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46313</v>
-      </c>
-      <c r="L15" s="23" t="n">
-        <v>40000</v>
-      </c>
+        <v>46318</v>
+      </c>
+      <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr">
-        <is>
-          <t>dpagi@mj.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr"/>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="n">
-        <v>146427</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>unesco:27856fe5-63c2-4c4c-7b80-08df26180ec9</t>
+        </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
+          <t>914BRZ4027 - Edital 58/2026 - Arquitetura e Urbanismo - Iphan-PB</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>HOME OFFICE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L16" s="15" t="n">
-        <v>208000</v>
-      </c>
+        <v>46318</v>
+      </c>
+      <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr"/>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>146428</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
@@ -1914,51 +1846,43 @@
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>HOME OFFICE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46308</v>
+        <v>46286</v>
       </c>
       <c r="K17" s="22" t="n">
         <v>46316</v>
       </c>
-      <c r="L17" s="23" t="n">
-        <v>28000</v>
-      </c>
+      <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr">
-        <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr"/>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="n">
-        <v>146419</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>UNDP-BR/25/024 - Edital nº 9/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização dos instrumentos coletivos de trabalho registrados no Sistema Mediador nas ações ajuizadas nos anos de 2023, 2024 e 2025.</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1976,56 +1900,48 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Híbrido, com eventuais reuniões presenciais em Brasília/DF </t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46311</v>
+        <v>46286</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46322</v>
-      </c>
-      <c r="L18" s="15" t="n">
-        <v>116812.8</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr">
-        <is>
-          <t>processoseletivosrt@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr"/>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="n">
-        <v>146420</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+        </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 10/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização e da atuação jurídica governamental federal nas ações judiciais ajuizadas nos anos de 2024 e 2025 relacionadas a pedidos de registro de entidades sindicais e aos respectivos processos administrativos.</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2035,49 +1951,37 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr">
-        <is>
-          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46311</v>
+        <v>46286</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46322</v>
-      </c>
-      <c r="L19" s="23" t="n">
-        <v>116812.8</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr">
-        <is>
-          <t>processoseletivosrt@trabalho.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr"/>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2089,12 +1993,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2104,15 +2008,13 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2122,10 +2024,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46309</v>
+        <v>46286</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2148,12 +2050,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2163,15 +2065,13 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr"/>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2181,10 +2081,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46309</v>
+        <v>46286</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2207,12 +2107,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:1b397c59-629f-47bf-bf95-08df23ad085e</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Republicação - Edital 33/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2238,10 +2138,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46308</v>
+        <v>46286</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46313</v>
+        <v>46316</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2264,28 +2164,30 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:0f405e12-70d9-40e9-ff3b-08df246fb477</t>
+          <t>unesco:006fb387-0b8e-43ce-7b81-08df26180ec9</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1156 - Edital 09/2026 - Consultor Individual - 01 vaga</t>
+          <t>914BRZ4027 - Edital 59/2026 - Fotografia - Iphan-Sede</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2295,10 +2197,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46320</v>
+        <v>46318</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2316,22 +2218,22 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:5e9b99bd-04d4-46aa-60df-08df20839863</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>A2101B5102 | Edital 01/2026 – 01 vaga - Consultor individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -2340,52 +2242,62 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J24" s="14" t="n">
-        <v>46310</v>
+        <v>46275</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46317</v>
-      </c>
-      <c r="L24" s="15" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L24" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N24" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:4e03075d-fa9c-444b-bf96-08df23ad085e</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>570BRZ2005 - Edital 01/2026 - Consultor individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2395,116 +2307,140 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="inlineStr"/>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J25" s="22" t="n">
-        <v>46310</v>
+        <v>46265</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46315</v>
-      </c>
-      <c r="L25" s="23" t="inlineStr"/>
+        <v>46270</v>
+      </c>
+      <c r="L25" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N25" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N25" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F26" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>Porto Alegre/RS</t>
+        </is>
+      </c>
       <c r="J26" s="14" t="n">
-        <v>46286</v>
+        <v>46246</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L26" s="15" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L26" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2513,263 +2449,315 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
       <c r="J27" s="22" t="n">
-        <v>46286</v>
+        <v>46266</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L27" s="23" t="inlineStr"/>
+        <v>46288</v>
+      </c>
+      <c r="L27" s="23" t="n">
+        <v>70000</v>
+      </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Porto Alegre - RS</t>
+        </is>
+      </c>
       <c r="J28" s="14" t="n">
-        <v>46286</v>
+        <v>46275</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46316</v>
+        <v>46281</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
       <c r="J29" s="22" t="n">
-        <v>46286</v>
+        <v>46278</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46316</v>
+        <v>46295</v>
       </c>
       <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr">
+        <is>
+          <t>ugp@educacao.sp.gov.br</t>
+        </is>
+      </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="inlineStr"/>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J30" s="14" t="n">
+        <v>46282</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>46286</v>
       </c>
-      <c r="K30" s="14" t="n">
-        <v>46316</v>
-      </c>
-      <c r="L30" s="15" t="inlineStr"/>
+      <c r="L30" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>Porto Alegre - RS</t>
+        </is>
+      </c>
       <c r="J31" s="22" t="n">
-        <v>46286</v>
+        <v>46290</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46316</v>
+        <v>46294</v>
       </c>
       <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -2781,17 +2769,17 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2804,27 +2792,27 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46252</v>
+        <v>46281</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46259</v>
+        <v>46286</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>60000</v>
+        <v>110000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2838,7 +2826,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -2850,12 +2838,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2865,7 +2853,7 @@
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F33" s="21" t="n">
@@ -2873,7 +2861,7 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2883,21 +2871,21 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46246</v>
+        <v>46293</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46272</v>
+        <v>46298</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2907,7 +2895,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -2919,12 +2907,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2934,15 +2922,15 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2952,21 +2940,21 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46266</v>
+        <v>46293</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46288</v>
+        <v>46298</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>70000</v>
+        <v>21000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2976,7 +2964,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -2988,22 +2976,22 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
@@ -3011,12 +2999,12 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
@@ -3025,13 +3013,13 @@
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46265</v>
+        <v>46294</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46270</v>
+        <v>46300</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>30000</v>
+        <v>55000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3045,7 +3033,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3057,12 +3045,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3080,7 +3068,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3094,13 +3082,13 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46275</v>
+        <v>46296</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46280</v>
+        <v>46300</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3114,7 +3102,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3126,12 +3114,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3145,30 +3133,32 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46275</v>
+        <v>46296</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>60000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3181,7 +3171,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3193,17 +3183,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3216,27 +3206,27 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46281</v>
+        <v>46294</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46286</v>
+        <v>46302</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>110000</v>
+        <v>60000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3250,7 +3240,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3262,12 +3252,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3277,35 +3267,35 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46282</v>
+        <v>46296</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>30000</v>
+        <v>33000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3319,7 +3309,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -3331,17 +3321,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3350,11 +3340,11 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3364,16 +3354,18 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46290</v>
+        <v>46296</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>21000</v>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3386,7 +3378,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -3398,17 +3390,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3417,30 +3409,32 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46278</v>
+        <v>46244</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L41" s="23" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="L41" s="23" t="n">
+        <v>935000</v>
+      </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3448,12 +3442,12 @@
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3465,12 +3459,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3480,7 +3474,7 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F42" s="13" t="n">
@@ -3488,27 +3482,27 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>30000</v>
+        <v>36000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3522,7 +3516,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -3534,12 +3528,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3549,15 +3543,15 @@
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.335</v>
+        <v>0.4</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3567,21 +3561,21 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46293</v>
+        <v>46297</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46298</v>
+        <v>46311</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>21000</v>
+        <v>70000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3591,7 +3585,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -3603,17 +3597,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3626,41 +3620,41 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46294</v>
+        <v>46244</v>
       </c>
       <c r="K44" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>55000</v>
+        <v>350000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3672,17 +3666,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3695,41 +3689,41 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46294</v>
+        <v>46301</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46302</v>
+        <v>46315</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>60000</v>
+        <v>600000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -3741,12 +3735,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3764,7 +3758,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3774,21 +3768,21 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>60000</v>
+        <v>90000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -3798,7 +3792,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -3810,17 +3804,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3833,7 +3827,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3843,17 +3837,17 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>60000</v>
+        <v>62500</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3867,7 +3861,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -3879,12 +3873,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3894,7 +3888,7 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
@@ -3902,27 +3896,27 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46244</v>
+        <v>46302</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46296</v>
+        <v>46322</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>935000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3936,7 +3930,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -3948,17 +3942,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3967,31 +3961,31 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46296</v>
+        <v>46302</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>33000</v>
+        <v>140000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4005,7 +3999,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4017,17 +4011,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4036,7 +4030,7 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
@@ -4045,36 +4039,36 @@
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Vitória/ES.</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46300</v>
+        <v>46321</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>21000</v>
+        <v>600000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4086,12 +4080,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4109,7 +4103,7 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -4119,21 +4113,21 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46296</v>
+        <v>46303</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46300</v>
+        <v>46311</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>36000</v>
+        <v>600000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
@@ -4143,7 +4137,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
         </is>
       </c>
     </row>
@@ -4155,12 +4149,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4170,35 +4164,35 @@
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46297</v>
+        <v>46302</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>70000</v>
+        <v>27000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4212,7 +4206,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
         </is>
       </c>
     </row>
@@ -4224,50 +4218,50 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13327</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46244</v>
+        <v>46311</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46300</v>
+        <v>46315</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>350000</v>
+        <v>600000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4276,12 +4270,12 @@
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327/</t>
         </is>
       </c>
     </row>
@@ -4293,12 +4287,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4316,31 +4310,31 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="K54" s="14" t="n">
         <v>46311</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>90000</v>
+        <v>600000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4350,7 +4344,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -4362,50 +4356,50 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13326</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Salvador - BA</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46302</v>
+        <v>46311</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46322</v>
+        <v>46315</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>2778901.38</v>
+        <v>600000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -4414,638 +4408,17 @@
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
-        </is>
-      </c>
-      <c r="C56" s="11" t="inlineStr">
-        <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E56" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F56" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G56" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H56" s="11" t="inlineStr">
-        <is>
-          <t>OEI/SECULT</t>
-        </is>
-      </c>
-      <c r="I56" s="11" t="inlineStr">
-        <is>
-          <t>Vitória/ES</t>
-        </is>
-      </c>
-      <c r="J56" s="14" t="n">
-        <v>46301</v>
-      </c>
-      <c r="K56" s="14" t="n">
-        <v>46315</v>
-      </c>
-      <c r="L56" s="15" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M56" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N56" s="12" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O56" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B57" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
-        </is>
-      </c>
-      <c r="C57" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
-        </is>
-      </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Física (PF)</t>
-        </is>
-      </c>
-      <c r="E57" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F57" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G57" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H57" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I57" s="19" t="inlineStr">
-        <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
-        </is>
-      </c>
-      <c r="J57" s="22" t="n">
-        <v>46301</v>
-      </c>
-      <c r="K57" s="22" t="n">
-        <v>46305</v>
-      </c>
-      <c r="L57" s="23" t="n">
-        <v>62500</v>
-      </c>
-      <c r="M57" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N57" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O57" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
-        </is>
-      </c>
-      <c r="C58" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
-        </is>
-      </c>
-      <c r="E58" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F58" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G58" s="11" t="inlineStr">
-        <is>
-          <t>Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H58" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I58" s="11" t="inlineStr">
-        <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
-        </is>
-      </c>
-      <c r="J58" s="14" t="n">
-        <v>46302</v>
-      </c>
-      <c r="K58" s="14" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L58" s="15" t="n">
-        <v>140000</v>
-      </c>
-      <c r="M58" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N58" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O58" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B59" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
-        </is>
-      </c>
-      <c r="C59" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
-        </is>
-      </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E59" s="20" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F59" s="21" t="n">
-        <v>0.345</v>
-      </c>
-      <c r="G59" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H59" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I59" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J59" s="22" t="n">
-        <v>46302</v>
-      </c>
-      <c r="K59" s="22" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L59" s="23" t="n">
-        <v>27000</v>
-      </c>
-      <c r="M59" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N59" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O59" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
-        </is>
-      </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F60" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G60" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H60" s="11" t="inlineStr">
-        <is>
-          <t>OEI/SECULT</t>
-        </is>
-      </c>
-      <c r="I60" s="11" t="inlineStr">
-        <is>
-          <t>Vitória/ES.</t>
-        </is>
-      </c>
-      <c r="J60" s="14" t="n">
-        <v>46308</v>
-      </c>
-      <c r="K60" s="14" t="n">
-        <v>46321</v>
-      </c>
-      <c r="L60" s="15" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M60" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N60" s="12" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O60" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B61" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F61" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H61" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J61" s="22" t="n">
-        <v>46303</v>
-      </c>
-      <c r="K61" s="22" t="n">
-        <v>46311</v>
-      </c>
-      <c r="L61" s="23" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M61" s="17" t="inlineStr">
-        <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N61" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O61" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F62" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
-        </is>
-      </c>
-      <c r="J62" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="K62" s="14" t="n">
-        <v>46311</v>
-      </c>
-      <c r="L62" s="15" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M62" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N62" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O62" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326</t>
-        </is>
-      </c>
-      <c r="C63" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13326</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E63" s="20" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F63" s="21" t="n">
-        <v>0.347</v>
-      </c>
-      <c r="G63" s="19" t="inlineStr">
-        <is>
-          <t>Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H63" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I63" s="19" t="inlineStr">
-        <is>
-          <t>Salvador - BA</t>
-        </is>
-      </c>
-      <c r="J63" s="22" t="n">
-        <v>46311</v>
-      </c>
-      <c r="K63" s="22" t="n">
-        <v>46315</v>
-      </c>
-      <c r="L63" s="23" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M63" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N63" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O63" s="24" t="inlineStr">
-        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326/</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327</t>
-        </is>
-      </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13327</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F64" s="13" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="G64" s="11" t="inlineStr">
-        <is>
-          <t>Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H64" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I64" s="11" t="inlineStr">
-        <is>
-          <t>Salvador/BA</t>
-        </is>
-      </c>
-      <c r="J64" s="14" t="n">
-        <v>46311</v>
-      </c>
-      <c r="K64" s="14" t="n">
-        <v>46315</v>
-      </c>
-      <c r="L64" s="15" t="n">
-        <v>600000</v>
-      </c>
-      <c r="M64" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N64" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O64" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327/</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O64"/>
+  <autoFilter ref="A1:O55"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -5101,15 +4474,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5148,27 +4512,27 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -5210,7 +4574,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -5220,7 +4584,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -5278,7 +4642,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5288,31 +4652,31 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -5354,27 +4718,27 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -5384,7 +4748,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -5394,7 +4758,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -5404,7 +4768,7 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -5440,7 +4804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5462,7 +4826,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5472,17 +4836,17 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
@@ -5496,23 +4860,23 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -5522,7 +4886,7 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -5532,25 +4896,15 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>OEI/FPOS</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5594,7 +4948,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5609,7 +4963,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5624,7 +4978,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5639,7 +4993,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-20 16:32
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$57</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 19/10/2026 às 18:23</t>
+          <t>Gerado em 20/10/2026 às 16:24</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -730,37 +730,37 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -900,7 +900,7 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F2" s="13" t="n">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
@@ -1347,17 +1347,15 @@
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>unesco:8e0c9386-3ad1-41de-cc73-08df25fc88d5</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>146438</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>UNESCO 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
+          <t xml:space="preserve"> Contratação de 1 (um) Consultor para elaborar estudo técnico especializado para projeção de oferta e demanda de combustíveis, conforme produtos descritos no item 6 deste Termo de Referência. A contratação está vinculada ao Projeto BRA/26/002 e ao fortalecimento institucional da Infra S.A., com foco na elaboração de estudos técnicos estratégicos</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1367,7 +1365,7 @@
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F9" s="21" t="n">
@@ -1375,31 +1373,41 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I9" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>BRASÍLIA DF</t>
+        </is>
+      </c>
       <c r="J9" s="22" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46320</v>
-      </c>
-      <c r="L9" s="23" t="inlineStr"/>
+        <v>46321</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>116000</v>
+      </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N9" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N9" s="20" t="inlineStr">
+        <is>
+          <t>processoseletivo.pnud@infrasa.gov.br</t>
+        </is>
+      </c>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1411,22 +1419,22 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>unesco:048a1d3b-843f-4613-60de-08df20839863</t>
+          <t>unesco:8e0c9386-3ad1-41de-cc73-08df25fc88d5</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 42/2026 - 1 vaga - Consultor Individual</t>
+          <t>UNESCO 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
@@ -1434,7 +1442,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1444,10 +1452,10 @@
       </c>
       <c r="I10" s="11" t="inlineStr"/>
       <c r="J10" s="14" t="n">
-        <v>46309</v>
+        <v>46314</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46314</v>
+        <v>46320</v>
       </c>
       <c r="L10" s="15" t="inlineStr"/>
       <c r="M10" s="9" t="inlineStr">
@@ -1485,7 +1493,7 @@
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F11" s="21" t="n">
@@ -1717,7 +1725,7 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F15" s="21" t="n">
@@ -1776,7 +1784,7 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
@@ -1820,12 +1828,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:bcb9ad69-010a-48cb-2c80-08df29fb4e16</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ3061 - EDITAL Nº 16/2026 - 01 VAGA - CONSULTOR INDIVIDUAL</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1835,13 +1843,15 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="inlineStr"/>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1851,10 +1861,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46286</v>
+        <v>46315</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46316</v>
+        <v>46325</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1877,12 +1887,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:1c199ce7-1aec-45f2-2c7f-08df29fb4e16</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ3061 - EDITAL Nº 14/2026-REPUBLICAÇÃO - 01 VAGA - CONSULTOR INDIVIDUAL</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1892,15 +1902,13 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1910,10 +1918,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46286</v>
+        <v>46315</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1936,12 +1944,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1957,7 +1965,7 @@
       <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1993,12 +2001,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2008,13 +2016,15 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2050,12 +2060,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2071,7 +2081,7 @@
       <c r="F21" s="21" t="inlineStr"/>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2107,12 +2117,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2164,30 +2174,28 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:006fb387-0b8e-43ce-7b81-08df26180ec9</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 59/2026 - Fotografia - Iphan-Sede</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr"/>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2197,10 +2205,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46314</v>
+        <v>46286</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2218,91 +2226,79 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr"/>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46275</v>
+        <v>46286</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L24" s="15" t="n">
-        <v>50000</v>
-      </c>
+        <v>46316</v>
+      </c>
+      <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N24" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr"/>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>unesco:006fb387-0b8e-43ce-7b81-08df26180ec9</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>914BRZ4027 - Edital 59/2026 - Fotografia - Iphan-Sede</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2311,45 +2307,35 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46265</v>
+        <v>46314</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L25" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46318</v>
+      </c>
+      <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N25" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N25" s="20" t="inlineStr"/>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2362,7 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
@@ -2430,12 +2416,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2445,7 +2431,7 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F27" s="21" t="n">
@@ -2453,27 +2439,27 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46266</v>
+        <v>46275</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46288</v>
+        <v>46280</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>70000</v>
+        <v>50000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2487,7 +2473,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2500,7 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
@@ -2566,62 +2552,64 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46278</v>
+        <v>46265</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46295</v>
-      </c>
-      <c r="L29" s="23" t="inlineStr"/>
+        <v>46270</v>
+      </c>
+      <c r="L29" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
         <is>
-          <t>ugp@educacao.sp.gov.br</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -2633,12 +2621,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2656,7 +2644,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2666,17 +2654,17 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46282</v>
+        <v>46266</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2690,7 +2678,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -2702,17 +2690,17 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2721,11 +2709,11 @@
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2735,16 +2723,18 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46290</v>
+        <v>46281</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L31" s="23" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L31" s="23" t="n">
+        <v>110000</v>
+      </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2757,7 +2747,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -2769,30 +2759,30 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2802,18 +2792,16 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46281</v>
+        <v>46290</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46286</v>
-      </c>
-      <c r="L32" s="15" t="n">
-        <v>110000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2826,7 +2814,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -2838,12 +2826,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13242</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2871,14 +2859,14 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46293</v>
+        <v>46282</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46298</v>
+        <v>46286</v>
       </c>
       <c r="L33" s="23" t="n">
         <v>30000</v>
@@ -2895,7 +2883,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13242/</t>
         </is>
       </c>
     </row>
@@ -2976,12 +2964,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR 13236</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -2991,15 +2979,15 @@
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3009,31 +2997,29 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46294</v>
+        <v>46278</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L35" s="23" t="n">
-        <v>55000</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>ugp@educacao.sp.gov.br</t>
         </is>
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr-13236/</t>
         </is>
       </c>
     </row>
@@ -3045,12 +3031,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3060,7 +3046,7 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
@@ -3068,27 +3054,27 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46296</v>
+        <v>46293</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3102,7 +3088,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3114,12 +3100,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3137,7 +3123,7 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3151,13 +3137,13 @@
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K37" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3171,7 +3157,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3183,12 +3169,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3198,7 +3184,7 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
@@ -3206,24 +3192,24 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L38" s="15" t="n">
         <v>60000</v>
@@ -3240,7 +3226,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3252,12 +3238,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3267,25 +3253,25 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
@@ -3295,7 +3281,7 @@
         <v>46300</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>33000</v>
+        <v>60000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3309,7 +3295,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3321,12 +3307,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3336,35 +3322,35 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>21000</v>
+        <v>60000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3378,7 +3364,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3376,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3409,45 +3395,45 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>935000</v>
+        <v>33000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -3459,12 +3445,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3478,11 +3464,11 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3502,7 +3488,7 @@
         <v>46300</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>36000</v>
+        <v>21000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3516,7 +3502,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -3528,22 +3514,22 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
@@ -3551,41 +3537,41 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46297</v>
+        <v>46244</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46311</v>
+        <v>46300</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>70000</v>
+        <v>350000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3597,22 +3583,22 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
@@ -3620,41 +3606,41 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K44" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>350000</v>
+        <v>36000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -3666,12 +3652,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3681,7 +3667,7 @@
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F45" s="21" t="n">
@@ -3689,27 +3675,27 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46301</v>
+        <v>46244</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46315</v>
+        <v>46296</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>600000</v>
+        <v>935000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3723,7 +3709,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3735,12 +3721,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13221</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3750,7 +3736,7 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F46" s="13" t="n">
@@ -3758,7 +3744,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3778,11 +3764,11 @@
         <v>46311</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>90000</v>
+        <v>70000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>Suspendida</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -3792,7 +3778,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13221/</t>
         </is>
       </c>
     </row>
@@ -3804,22 +3790,22 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13304</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F47" s="21" t="n">
@@ -3827,31 +3813,31 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46305</v>
+        <v>46311</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>62500</v>
+        <v>90000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Suspendida</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3861,7 +3847,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13304/</t>
         </is>
       </c>
     </row>
@@ -3873,12 +3859,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:procedimento-simplificado-no-13307-2026-oei-secult-es</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Procedimento Simplificado nº 13307/2026 – OEI/SECULT-ES</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3888,7 +3874,7 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
@@ -3896,27 +3882,27 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Vitória/ES</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46322</v>
+        <v>46315</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>2778901.38</v>
+        <v>600000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3930,7 +3916,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13307-2026-oei-secult-es/</t>
         </is>
       </c>
     </row>
@@ -3942,22 +3928,22 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F49" s="21" t="n">
@@ -3965,27 +3951,27 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>140000</v>
+        <v>62500</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -3999,7 +3985,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4011,12 +3997,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4026,7 +4012,7 @@
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
@@ -4034,27 +4020,27 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Vitória/ES.</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>600000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4068,7 +4054,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4080,22 +4066,22 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
@@ -4103,31 +4089,31 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>600000</v>
+        <v>140000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
@@ -4137,7 +4123,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4218,47 +4204,47 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327</t>
+          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13327</t>
+          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.34</v>
+        <v>0.4</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/SECULT</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Vitória/ES.</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46315</v>
+        <v>46321</v>
       </c>
       <c r="L53" s="23" t="n">
         <v>600000</v>
@@ -4270,12 +4256,12 @@
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4287,12 +4273,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13312</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13312 REPUBLICADO</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4302,7 +4288,7 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
@@ -4310,7 +4296,7 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4320,11 +4306,11 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Remota e/ou presencial em Brasília - DF</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46294</v>
+        <v>46303</v>
       </c>
       <c r="K54" s="14" t="n">
         <v>46311</v>
@@ -4334,7 +4320,7 @@
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4344,7 +4330,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13312/</t>
         </is>
       </c>
     </row>
@@ -4356,12 +4342,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13326</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13327</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4375,7 +4361,7 @@
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.347</v>
+        <v>0.34</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
@@ -4389,7 +4375,7 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Salvador - BA</t>
+          <t>Salvador/BA</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
@@ -4413,12 +4399,150 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F56" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>Remota e/ou presencial em Brasília - DF</t>
+        </is>
+      </c>
+      <c r="J56" s="14" t="n">
+        <v>46294</v>
+      </c>
+      <c r="K56" s="14" t="n">
+        <v>46311</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N56" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O56" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326</t>
+        </is>
+      </c>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13326</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F57" s="21" t="n">
+        <v>0.347</v>
+      </c>
+      <c r="G57" s="19" t="inlineStr">
+        <is>
+          <t>Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H57" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>Salvador - BA</t>
+        </is>
+      </c>
+      <c r="J57" s="22" t="n">
+        <v>46311</v>
+      </c>
+      <c r="K57" s="22" t="n">
+        <v>46315</v>
+      </c>
+      <c r="L57" s="23" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M57" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N57" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O57" s="24" t="inlineStr">
+        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O55"/>
+  <autoFilter ref="A1:O57"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4474,6 +4598,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4522,7 +4648,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -4532,7 +4658,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -4570,37 +4696,37 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
@@ -4646,7 +4772,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -4656,7 +4782,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -4718,7 +4844,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -4738,7 +4864,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -4758,13 +4884,13 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Direito / Jurídico</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -4774,11 +4900,11 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Direito / Jurídico</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -4830,7 +4956,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -4860,7 +4986,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -4944,60 +5070,60 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
+          <t>Economista com stack técnica em análise de dados e políticas públicas, sem pós-graduação</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
+          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Economista com stack técnica em análise de dados e políticas públicas, sem pós-graduação</t>
+          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
+          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-10-21 16:48
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 20/10/2026 às 16:24</t>
+          <t>Gerado em 21/10/2026 às 16:40</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>21000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="18">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>213242.8946666667</v>
+        <v>214958.1225</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1020,47 +1020,49 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146427</v>
+        <v>146426</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
+          <t xml:space="preserve">Edital nº 31/2026 - Contratação de Consultoria Individual para realizar estudo sobre alternativas organizacionais para assistência técnica a Estados e Municípios </t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr"/>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46316</v>
+        <v>46332</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>208000</v>
+        <v>80000</v>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
@@ -1069,7 +1071,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1085,11 +1087,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146428</v>
+        <v>146427</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM COMUNICAÇÃO E PRODUÇÃO DE CONTEÚDO</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1125,7 +1127,7 @@
         <v>46316</v>
       </c>
       <c r="L5" s="23" t="n">
-        <v>28000</v>
+        <v>208000</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1150,29 +1152,27 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146434</v>
+        <v>146428</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Edital 07/2026 - Curso “Direito à Identidade, Cidadania e Documentação" para a Plataforma EV.G/Enap.</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA EM PRODUÇÃO EDITORIAL, DESIGN E DIAGRAMAÇÃO DE PUBLICAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr"/>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1182,17 +1182,17 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46314</v>
+        <v>46308</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46330</v>
+        <v>46316</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>40000</v>
+        <v>28000</v>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>rcn_cidadania@mdh.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1217,11 +1217,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146419</v>
+        <v>146434</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>UNDP-BR/25/024 - Edital nº 9/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização dos instrumentos coletivos de trabalho registrados no Sistema Mediador nas ações ajuizadas nos anos de 2023, 2024 e 2025.</t>
+          <t>Edital 07/2026 - Curso “Direito à Identidade, Cidadania e Documentação" para a Plataforma EV.G/Enap.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1235,31 +1235,31 @@
         </is>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>MTE</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Híbrido, com eventuais reuniões presenciais em Brasília/DF </t>
+          <t>Brasília</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46322</v>
+        <v>46330</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>116812.8</v>
+        <v>40000</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>processoseletivosrt@trabalho.gov.br</t>
+          <t>rcn_cidadania@mdh.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1284,11 +1284,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146420</v>
+        <v>146419</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PNUD BRA/25/024 - Edital nº 10/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização e da atuação jurídica governamental federal nas ações judiciais ajuizadas nos anos de 2024 e 2025 relacionadas a pedidos de registro de entidades sindicais e aos respectivos processos administrativos.</t>
+          <t>UNDP-BR/25/024 - Edital nº 9/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização dos instrumentos coletivos de trabalho registrados no Sistema Mediador nas ações ajuizadas nos anos de 2023, 2024 e 2025.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
+          <t xml:space="preserve">Híbrido, com eventuais reuniões presenciais em Brasília/DF </t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
@@ -1351,16 +1351,16 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146438</v>
+        <v>146420</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Contratação de 1 (um) Consultor para elaborar estudo técnico especializado para projeção de oferta e demanda de combustíveis, conforme produtos descritos no item 6 deste Termo de Referência. A contratação está vinculada ao Projeto BRA/26/002 e ao fortalecimento institucional da Infra S.A., com foco na elaboração de estudos técnicos estratégicos</t>
+          <t>PNUD BRA/25/024 - Edital nº 10/2026 - Contratação de consultoria especializada, pessoa física, para diagnóstico da judicialização e da atuação jurídica governamental federal nas ações judiciais ajuizadas nos anos de 2024 e 2025 relacionadas a pedidos de registro de entidades sindicais e aos respectivos processos administrativos.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
@@ -1373,27 +1373,27 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MTE</t>
         </is>
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>BRASÍLIA DF</t>
+          <t>Híbrido, com eventuais reuniões presenciais em Brasília/DF</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="L9" s="23" t="n">
-        <v>116000</v>
+        <v>116812.8</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>processoseletivo.pnud@infrasa.gov.br</t>
+          <t>processoseletivosrt@trabalho.gov.br</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
@@ -1414,17 +1414,15 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>unesco:8e0c9386-3ad1-41de-cc73-08df25fc88d5</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>146438</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>UNESCO 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
+          <t xml:space="preserve"> Contratação de 1 (um) Consultor para elaborar estudo técnico especializado para projeção de oferta e demanda de combustíveis, conforme produtos descritos no item 6 deste Termo de Referência. A contratação está vinculada ao Projeto BRA/26/002 e ao fortalecimento institucional da Infra S.A., com foco na elaboração de estudos técnicos estratégicos</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1442,31 +1440,41 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I10" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>BRASÍLIA DF</t>
+        </is>
+      </c>
       <c r="J10" s="14" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46320</v>
-      </c>
-      <c r="L10" s="15" t="inlineStr"/>
+        <v>46321</v>
+      </c>
+      <c r="L10" s="15" t="n">
+        <v>116000</v>
+      </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N10" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N10" s="12" t="inlineStr">
+        <is>
+          <t>processoseletivo.pnud@infrasa.gov.br</t>
+        </is>
+      </c>
       <c r="O10" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1478,17 +1486,17 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>unesco:28aedd59-87d7-4b85-60e5-08df20839863</t>
+          <t>unesco:8e0c9386-3ad1-41de-cc73-08df25fc88d5</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1162 - Edital 07/2026 - 01 vaga - Consultor Individual</t>
+          <t>UNESCO 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
@@ -1501,7 +1509,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1511,10 +1519,10 @@
       </c>
       <c r="I11" s="19" t="inlineStr"/>
       <c r="J11" s="22" t="n">
-        <v>46309</v>
+        <v>46314</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46315</v>
+        <v>46320</v>
       </c>
       <c r="L11" s="23" t="inlineStr"/>
       <c r="M11" s="17" t="inlineStr">
@@ -1594,12 +1602,12 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>unesco:5e9b99bd-04d4-46aa-60df-08df20839863</t>
+          <t>unesco:883aa849-19ab-496a-2c7d-08df29fb4e16</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>A2101B5102 | Edital 01/2026 – 01 vaga - Consultor individual</t>
+          <t xml:space="preserve">914BRZ1155 - EDITAL Nº 58/2026 - 1 vaga - Consultor Individual </t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1609,7 +1617,7 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F13" s="21" t="n">
@@ -1617,7 +1625,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1627,10 +1635,10 @@
       </c>
       <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46317</v>
+        <v>46322</v>
       </c>
       <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
@@ -1653,12 +1661,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:4e03075d-fa9c-444b-bf96-08df23ad085e</t>
+          <t>unesco:5e9b99bd-04d4-46aa-60df-08df20839863</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>570BRZ2005 - Edital 01/2026 - Consultor individual</t>
+          <t>A2101B5102 | Edital 01/2026 – 01 vaga - Consultor individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1668,13 +1676,15 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1687,7 +1697,7 @@
         <v>46310</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
@@ -1769,12 +1779,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:27856fe5-63c2-4c4c-7b80-08df26180ec9</t>
+          <t>unesco:f23c483d-4d31-4b0e-0606-08df2ea2a444</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 58/2026 - Arquitetura e Urbanismo - Iphan-PB</t>
+          <t>914BRZ4024 - EDITAL Nº04/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1792,7 +1802,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1802,12 +1812,14 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46318</v>
-      </c>
-      <c r="L16" s="15" t="inlineStr"/>
+        <v>46320</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>58000</v>
+      </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
           <t>Ongoing</t>
@@ -1828,12 +1840,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:bcb9ad69-010a-48cb-2c80-08df29fb4e16</t>
+          <t>unesco:27856fe5-63c2-4c4c-7b80-08df26180ec9</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3061 - EDITAL Nº 16/2026 - 01 VAGA - CONSULTOR INDIVIDUAL</t>
+          <t>914BRZ4027 - Edital 58/2026 - Arquitetura e Urbanismo - Iphan-PB</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1851,7 +1863,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1861,10 +1873,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46325</v>
+        <v>46318</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1887,12 +1899,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:1c199ce7-1aec-45f2-2c7f-08df29fb4e16</t>
+          <t>unesco:bcb9ad69-010a-48cb-2c80-08df29fb4e16</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3061 - EDITAL Nº 14/2026-REPUBLICAÇÃO - 01 VAGA - CONSULTOR INDIVIDUAL</t>
+          <t>914BRZ3061 - EDITAL Nº 16/2026 - 01 VAGA - CONSULTOR INDIVIDUAL</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1902,13 +1914,15 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr"/>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1921,7 +1935,7 @@
         <v>46315</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46320</v>
+        <v>46325</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1944,12 +1958,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
+          <t>unesco:1c199ce7-1aec-45f2-2c7f-08df29fb4e16</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
+          <t>914BRZ3061 - EDITAL Nº 14/2026-REPUBLICAÇÃO - 01 VAGA - CONSULTOR INDIVIDUAL</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1975,10 +1989,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46286</v>
+        <v>46315</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2001,12 +2015,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
+          <t>unesco:e6096467-03ec-4c8e-0c6c-08df0dcf532b</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
+          <t>914BRZ3062 - Edital 01/2026 - 1 vaga - Consultor individual - Arquiteto</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2016,15 +2030,13 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2060,12 +2072,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
+          <t>unesco:0350dc26-be0b-42ba-0c6d-08df0dcf532b</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
+          <t xml:space="preserve">914BRZ3062 - Edital 02/2026 - 1 vaga - Consultor individual – Antropólogo Mobilização </t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2075,13 +2087,15 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2117,12 +2131,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
+          <t>unesco:c61a6d5e-3069-4c1e-0c6e-08df0dcf532b</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
+          <t>914BRZ3062 - Edital 03/2026 - 1 vaga - Consultor individual – Saúde</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2138,7 +2152,7 @@
       <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2174,12 +2188,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
+          <t>unesco:8cb6b1df-8a66-4b19-0c6f-08df0dcf532b</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
+          <t>914BRZ3062 - Edital 04/2026 - 1 vaga - Consultor individual – Antropólogo Referências</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2231,12 +2245,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
+          <t>unesco:26cafda1-3c3b-4854-0c70-08df0dcf532b</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
+          <t>914BRZ3062 - Edital 05/2026 - 1 vaga - Consultor individual – Historiador</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2288,30 +2302,28 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:006fb387-0b8e-43ce-7b81-08df26180ec9</t>
+          <t>unesco:a8acd062-b45d-401e-0c71-08df0dcf532b</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 59/2026 - Fotografia - Iphan-Sede</t>
+          <t>914BRZ3062 - Edital 06/2026 - 1 vaga - Consultor individual - Sênior</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2321,10 +2333,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46314</v>
+        <v>46286</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2342,17 +2354,17 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>unesco:006fb387-0b8e-43ce-7b81-08df26180ec9</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>914BRZ4027 - Edital 59/2026 - Fotografia - Iphan-Sede</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2366,45 +2378,35 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46246</v>
+        <v>46314</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L26" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46318</v>
+      </c>
+      <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr"/>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://roster.brasilia.unesco.org/</t>
         </is>
       </c>
     </row>
@@ -2416,12 +2418,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2439,27 +2441,27 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46280</v>
+        <v>46288</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>50000</v>
+        <v>70000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2473,7 +2475,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -2485,12 +2487,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2504,11 +2506,11 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2518,16 +2520,18 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
         <v>46275</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L28" s="15" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L28" s="15" t="n">
+        <v>50000</v>
+      </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2540,7 +2544,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -2552,17 +2556,17 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2575,31 +2579,31 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46270</v>
+        <v>46272</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>30000</v>
+        <v>54000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2609,7 +2613,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -2621,12 +2625,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR 13238</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2640,32 +2644,30 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46266</v>
+        <v>46275</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46288</v>
-      </c>
-      <c r="L30" s="15" t="n">
-        <v>70000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2678,7 +2680,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
@@ -2690,12 +2692,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2705,7 +2707,7 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F31" s="21" t="n">
@@ -2713,7 +2715,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2723,17 +2725,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Dados Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46281</v>
+        <v>46265</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46286</v>
+        <v>46270</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>110000</v>
+        <v>30000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2747,7 +2749,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -2759,30 +2761,30 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13247</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2792,16 +2794,18 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre - RS</t>
+          <t>Dados Remoto</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46290</v>
+        <v>46281</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46294</v>
-      </c>
-      <c r="L32" s="15" t="inlineStr"/>
+        <v>46286</v>
+      </c>
+      <c r="L32" s="15" t="n">
+        <v>110000</v>
+      </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2814,7 +2818,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13247/</t>
         </is>
       </c>
     </row>
@@ -2895,17 +2899,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13272</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2914,35 +2918,33 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.335</v>
+        <v>0.3</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Rio Grande do Norte</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46298</v>
-      </c>
-      <c r="L34" s="15" t="n">
-        <v>21000</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2952,7 +2954,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13272/</t>
         </is>
       </c>
     </row>
@@ -3031,12 +3033,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR 13274</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3050,11 +3052,11 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3064,7 +3066,7 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
+          <t>Articulação Estadual - Rio Grande do Norte</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
@@ -3074,11 +3076,11 @@
         <v>46298</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>30000</v>
+        <v>21000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3088,7 +3090,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr-13274/</t>
         </is>
       </c>
     </row>
@@ -3100,12 +3102,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13268</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3115,7 +3117,7 @@
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F37" s="21" t="n">
@@ -3123,7 +3125,7 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3133,17 +3135,17 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Articulação territorial - PAS Nordeste Articulação territorial - PAS Nordeste Trabalho Remoto</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>55000</v>
+        <v>30000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3157,7 +3159,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13268/</t>
         </is>
       </c>
     </row>
@@ -3169,12 +3171,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3192,24 +3194,24 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="L38" s="15" t="n">
         <v>60000</v>
@@ -3226,7 +3228,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
         </is>
       </c>
     </row>
@@ -3238,12 +3240,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/002 – TR13290</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3253,7 +3255,7 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F39" s="21" t="n">
@@ -3261,7 +3263,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3275,13 +3277,13 @@
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="K39" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3295,7 +3297,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-002-tr13290/</t>
         </is>
       </c>
     </row>
@@ -3307,12 +3309,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13271</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13275</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3330,24 +3332,24 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="L40" s="15" t="n">
         <v>60000</v>
@@ -3364,7 +3366,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13271/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13275/</t>
         </is>
       </c>
     </row>
@@ -3376,12 +3378,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13269</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3391,25 +3393,25 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.347</v>
+        <v>0.4</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
@@ -3419,7 +3421,7 @@
         <v>46300</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>33000</v>
+        <v>60000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3433,7 +3435,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13269/</t>
         </is>
       </c>
     </row>
@@ -3445,12 +3447,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13300</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3464,7 +3466,7 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.33</v>
+        <v>0.347</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
@@ -3488,7 +3490,7 @@
         <v>46300</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>21000</v>
+        <v>33000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3502,7 +3504,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13300/</t>
         </is>
       </c>
     </row>
@@ -3514,64 +3516,64 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13298</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K43" s="22" t="n">
         <v>46300</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>350000</v>
+        <v>21000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13298/</t>
         </is>
       </c>
     </row>
@@ -3583,17 +3585,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3606,41 +3608,41 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Vitória - ES</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K44" s="14" t="n">
         <v>46296</v>
       </c>
-      <c r="K44" s="14" t="n">
-        <v>46300</v>
-      </c>
       <c r="L44" s="15" t="n">
-        <v>36000</v>
+        <v>935000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3652,17 +3654,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO CAIS DAS ARTES/ES – TR13296</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3675,41 +3677,41 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Vitória - ES</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46244</v>
+        <v>46296</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>935000</v>
+        <v>36000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-cais-das-artes-es-tr13296/</t>
         </is>
       </c>
     </row>
@@ -3928,17 +3930,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3951,41 +3953,41 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46301</v>
+        <v>46244</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46305</v>
+        <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>62500</v>
+        <v>350000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3997,22 +3999,22 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13303</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
@@ -4020,41 +4022,41 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/FPOS</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto, com deslocamentos pontuais para reuniões e eventos</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46322</v>
+        <v>46305</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>2778901.38</v>
+        <v>62500</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13303/</t>
         </is>
       </c>
     </row>
@@ -4066,22 +4068,22 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
+          <t>oei:licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
+          <t>LICITAÇÃO Nº 13292/2026- OEI/FPOS MELHOR TÉCNICA E MENOR PREÇO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="F51" s="21" t="n">
@@ -4089,41 +4091,41 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/FPOS</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
         <v>46302</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46307</v>
+        <v>46322</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>140000</v>
+        <v>2778901.38</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/licitacao-no-13292-2026-oei-fpos-melhor-tecnica-e-menor-preco/</t>
         </is>
       </c>
     </row>
@@ -4135,17 +4137,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13288</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4154,21 +4156,21 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.345</v>
+        <v>0.4</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Consultor especialista em Gestão de Processos Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
@@ -4178,7 +4180,7 @@
         <v>46307</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>27000</v>
+        <v>140000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4192,7 +4194,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13288/</t>
         </is>
       </c>
     </row>
@@ -4204,64 +4206,64 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>PROCEDIMENTO SIMPLIFICADO Nº 13340/2026- OEI/SECULT-ES MENOR PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-05 – Brasil em Rede – TR13321</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F53" s="21" t="n">
-        <v>0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/SECULT</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Vitória/ES.</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46308</v>
+        <v>46302</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46321</v>
+        <v>46307</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>600000</v>
+        <v>27000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/procedimento-simplificado-no-13340-2026-oei-secult-es-menor-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-05-brasil-em-rede-tr13321/</t>
         </is>
       </c>
     </row>
@@ -4342,12 +4344,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327</t>
+          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13327</t>
+          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4361,11 +4363,11 @@
         </is>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.34</v>
+        <v>0.4</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -4375,14 +4377,14 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Salvador/BA</t>
+          <t>Remota e/ou presencial em Brasília - DF</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
+        <v>46294</v>
+      </c>
+      <c r="K55" s="22" t="n">
         <v>46311</v>
-      </c>
-      <c r="K55" s="22" t="n">
-        <v>46315</v>
       </c>
       <c r="L55" s="23" t="n">
         <v>600000</v>
@@ -4399,7 +4401,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13327/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-abdi-tr-13260/</t>
         </is>
       </c>
     </row>
@@ -4411,12 +4413,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-abdi-tr-13260</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-secult-sa-tr-13326</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO ABDI – TR 13260 REPUBLICADO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC SECULT SA – TR 13326</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4430,11 +4432,11 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodolog